<commit_message>
Generate and upload All Test Cases Passed Excel Workbooks artifact on GitHub Actions
</commit_message>
<xml_diff>
--- a/Test Results/Excel/Automation_Test_Report.xlsx
+++ b/Test Results/Excel/Automation_Test_Report.xlsx
@@ -3371,7 +3371,7 @@
         <v>9</v>
       </c>
       <c r="E2">
-        <v>0.12</v>
+        <v>0.26</v>
       </c>
       <c r="F2" t="s">
         <v>10</v>
@@ -3391,7 +3391,7 @@
         <v>9</v>
       </c>
       <c r="E3">
-        <v>0.12</v>
+        <v>0.26</v>
       </c>
       <c r="F3" t="s">
         <v>10</v>
@@ -3411,7 +3411,7 @@
         <v>9</v>
       </c>
       <c r="E4">
-        <v>0.12</v>
+        <v>0.11</v>
       </c>
       <c r="F4" t="s">
         <v>10</v>
@@ -3431,7 +3431,7 @@
         <v>9</v>
       </c>
       <c r="E5">
-        <v>0.21</v>
+        <v>0.15</v>
       </c>
       <c r="F5" t="s">
         <v>10</v>
@@ -3451,7 +3451,7 @@
         <v>9</v>
       </c>
       <c r="E6">
-        <v>0.21</v>
+        <v>0.37</v>
       </c>
       <c r="F6" t="s">
         <v>10</v>
@@ -3471,7 +3471,7 @@
         <v>9</v>
       </c>
       <c r="E7">
-        <v>0.36</v>
+        <v>0.33</v>
       </c>
       <c r="F7" t="s">
         <v>10</v>
@@ -3491,7 +3491,7 @@
         <v>9</v>
       </c>
       <c r="E8">
-        <v>0.35</v>
+        <v>0.2</v>
       </c>
       <c r="F8" t="s">
         <v>10</v>
@@ -3511,7 +3511,7 @@
         <v>9</v>
       </c>
       <c r="E9">
-        <v>0.31</v>
+        <v>0.39</v>
       </c>
       <c r="F9" t="s">
         <v>10</v>
@@ -3531,7 +3531,7 @@
         <v>9</v>
       </c>
       <c r="E10">
-        <v>0.32</v>
+        <v>0.31</v>
       </c>
       <c r="F10" t="s">
         <v>10</v>
@@ -3551,7 +3551,7 @@
         <v>9</v>
       </c>
       <c r="E11">
-        <v>0.14</v>
+        <v>0.34</v>
       </c>
       <c r="F11" t="s">
         <v>10</v>
@@ -3571,7 +3571,7 @@
         <v>9</v>
       </c>
       <c r="E12">
-        <v>0.16</v>
+        <v>0.31</v>
       </c>
       <c r="F12" t="s">
         <v>10</v>
@@ -3591,7 +3591,7 @@
         <v>9</v>
       </c>
       <c r="E13">
-        <v>0.29</v>
+        <v>0.31</v>
       </c>
       <c r="F13" t="s">
         <v>10</v>
@@ -3611,7 +3611,7 @@
         <v>9</v>
       </c>
       <c r="E14">
-        <v>0.26</v>
+        <v>0.33</v>
       </c>
       <c r="F14" t="s">
         <v>35</v>
@@ -3631,7 +3631,7 @@
         <v>9</v>
       </c>
       <c r="E15">
-        <v>0.38</v>
+        <v>0.24</v>
       </c>
       <c r="F15" t="s">
         <v>35</v>
@@ -3651,7 +3651,7 @@
         <v>9</v>
       </c>
       <c r="E16">
-        <v>0.3</v>
+        <v>0.32</v>
       </c>
       <c r="F16" t="s">
         <v>35</v>
@@ -3671,7 +3671,7 @@
         <v>9</v>
       </c>
       <c r="E17">
-        <v>0.34</v>
+        <v>0.38</v>
       </c>
       <c r="F17" t="s">
         <v>35</v>
@@ -3691,7 +3691,7 @@
         <v>9</v>
       </c>
       <c r="E18">
-        <v>0.23</v>
+        <v>0.1</v>
       </c>
       <c r="F18" t="s">
         <v>35</v>
@@ -3711,7 +3711,7 @@
         <v>9</v>
       </c>
       <c r="E19">
-        <v>0.2</v>
+        <v>0.31</v>
       </c>
       <c r="F19" t="s">
         <v>35</v>
@@ -3731,7 +3731,7 @@
         <v>9</v>
       </c>
       <c r="E20">
-        <v>0.12</v>
+        <v>0.15</v>
       </c>
       <c r="F20" t="s">
         <v>35</v>
@@ -3751,7 +3751,7 @@
         <v>9</v>
       </c>
       <c r="E21">
-        <v>0.39</v>
+        <v>0.15</v>
       </c>
       <c r="F21" t="s">
         <v>35</v>
@@ -3771,7 +3771,7 @@
         <v>9</v>
       </c>
       <c r="E22">
-        <v>0.19</v>
+        <v>0.29</v>
       </c>
       <c r="F22" t="s">
         <v>35</v>
@@ -3791,7 +3791,7 @@
         <v>9</v>
       </c>
       <c r="E23">
-        <v>0.26</v>
+        <v>0.28</v>
       </c>
       <c r="F23" t="s">
         <v>35</v>
@@ -3811,7 +3811,7 @@
         <v>9</v>
       </c>
       <c r="E24">
-        <v>0.13</v>
+        <v>0.17</v>
       </c>
       <c r="F24" t="s">
         <v>35</v>
@@ -3831,7 +3831,7 @@
         <v>9</v>
       </c>
       <c r="E25">
-        <v>0.23</v>
+        <v>0.26</v>
       </c>
       <c r="F25" t="s">
         <v>35</v>
@@ -3851,7 +3851,7 @@
         <v>9</v>
       </c>
       <c r="E26">
-        <v>0.25</v>
+        <v>0.39</v>
       </c>
       <c r="F26" t="s">
         <v>60</v>
@@ -3871,7 +3871,7 @@
         <v>9</v>
       </c>
       <c r="E27">
-        <v>0.25</v>
+        <v>0.11</v>
       </c>
       <c r="F27" t="s">
         <v>60</v>
@@ -3891,7 +3891,7 @@
         <v>9</v>
       </c>
       <c r="E28">
-        <v>0.33</v>
+        <v>0.2</v>
       </c>
       <c r="F28" t="s">
         <v>60</v>
@@ -3911,7 +3911,7 @@
         <v>9</v>
       </c>
       <c r="E29">
-        <v>0.18</v>
+        <v>0.26</v>
       </c>
       <c r="F29" t="s">
         <v>60</v>
@@ -3931,7 +3931,7 @@
         <v>9</v>
       </c>
       <c r="E30">
-        <v>0.36</v>
+        <v>0.17</v>
       </c>
       <c r="F30" t="s">
         <v>60</v>
@@ -3971,7 +3971,7 @@
         <v>9</v>
       </c>
       <c r="E32">
-        <v>0.21</v>
+        <v>0.12</v>
       </c>
       <c r="F32" t="s">
         <v>60</v>
@@ -3991,7 +3991,7 @@
         <v>9</v>
       </c>
       <c r="E33">
-        <v>0.11</v>
+        <v>0.27</v>
       </c>
       <c r="F33" t="s">
         <v>60</v>
@@ -4011,7 +4011,7 @@
         <v>9</v>
       </c>
       <c r="E34">
-        <v>0.24</v>
+        <v>0.25</v>
       </c>
       <c r="F34" t="s">
         <v>60</v>
@@ -4031,7 +4031,7 @@
         <v>9</v>
       </c>
       <c r="E35">
-        <v>0.23</v>
+        <v>0.22</v>
       </c>
       <c r="F35" t="s">
         <v>60</v>
@@ -4051,7 +4051,7 @@
         <v>9</v>
       </c>
       <c r="E36">
-        <v>0.28</v>
+        <v>0.39</v>
       </c>
       <c r="F36" t="s">
         <v>60</v>
@@ -4071,7 +4071,7 @@
         <v>9</v>
       </c>
       <c r="E37">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="F37" t="s">
         <v>60</v>
@@ -4091,7 +4091,7 @@
         <v>9</v>
       </c>
       <c r="E38">
-        <v>0.26</v>
+        <v>0.21</v>
       </c>
       <c r="F38" t="s">
         <v>60</v>
@@ -4111,7 +4111,7 @@
         <v>9</v>
       </c>
       <c r="E39">
-        <v>0.28</v>
+        <v>0.19</v>
       </c>
       <c r="F39" t="s">
         <v>60</v>
@@ -4131,7 +4131,7 @@
         <v>9</v>
       </c>
       <c r="E40">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="F40" t="s">
         <v>60</v>
@@ -4151,7 +4151,7 @@
         <v>9</v>
       </c>
       <c r="E41">
-        <v>0.15</v>
+        <v>0.14</v>
       </c>
       <c r="F41" t="s">
         <v>60</v>
@@ -4171,7 +4171,7 @@
         <v>9</v>
       </c>
       <c r="E42">
-        <v>0.17</v>
+        <v>0.21</v>
       </c>
       <c r="F42" t="s">
         <v>10</v>
@@ -4191,7 +4191,7 @@
         <v>9</v>
       </c>
       <c r="E43">
-        <v>0.39</v>
+        <v>0.18</v>
       </c>
       <c r="F43" t="s">
         <v>10</v>
@@ -4211,7 +4211,7 @@
         <v>9</v>
       </c>
       <c r="E44">
-        <v>0.34</v>
+        <v>0.18</v>
       </c>
       <c r="F44" t="s">
         <v>10</v>
@@ -4231,7 +4231,7 @@
         <v>9</v>
       </c>
       <c r="E45">
-        <v>0.11</v>
+        <v>0.26</v>
       </c>
       <c r="F45" t="s">
         <v>10</v>
@@ -4251,7 +4251,7 @@
         <v>9</v>
       </c>
       <c r="E46">
-        <v>0.25</v>
+        <v>0.23</v>
       </c>
       <c r="F46" t="s">
         <v>10</v>
@@ -4271,7 +4271,7 @@
         <v>9</v>
       </c>
       <c r="E47">
-        <v>0.11</v>
+        <v>0.16</v>
       </c>
       <c r="F47" t="s">
         <v>10</v>
@@ -4291,7 +4291,7 @@
         <v>9</v>
       </c>
       <c r="E48">
-        <v>0.29</v>
+        <v>0.31</v>
       </c>
       <c r="F48" t="s">
         <v>10</v>
@@ -4311,7 +4311,7 @@
         <v>9</v>
       </c>
       <c r="E49">
-        <v>0.13</v>
+        <v>0.2</v>
       </c>
       <c r="F49" t="s">
         <v>10</v>
@@ -4331,7 +4331,7 @@
         <v>9</v>
       </c>
       <c r="E50">
-        <v>0.11</v>
+        <v>0.16</v>
       </c>
       <c r="F50" t="s">
         <v>10</v>
@@ -4351,7 +4351,7 @@
         <v>9</v>
       </c>
       <c r="E51">
-        <v>0.15</v>
+        <v>0.33</v>
       </c>
       <c r="F51" t="s">
         <v>10</v>
@@ -4371,7 +4371,7 @@
         <v>9</v>
       </c>
       <c r="E52">
-        <v>0.37</v>
+        <v>0.16</v>
       </c>
       <c r="F52" t="s">
         <v>10</v>
@@ -4391,7 +4391,7 @@
         <v>9</v>
       </c>
       <c r="E53">
-        <v>0.39</v>
+        <v>0.33</v>
       </c>
       <c r="F53" t="s">
         <v>10</v>
@@ -4411,7 +4411,7 @@
         <v>9</v>
       </c>
       <c r="E54">
-        <v>0.23</v>
+        <v>0.19</v>
       </c>
       <c r="F54" t="s">
         <v>35</v>
@@ -4431,7 +4431,7 @@
         <v>9</v>
       </c>
       <c r="E55">
-        <v>0.16</v>
+        <v>0.37</v>
       </c>
       <c r="F55" t="s">
         <v>35</v>
@@ -4451,7 +4451,7 @@
         <v>9</v>
       </c>
       <c r="E56">
-        <v>0.13</v>
+        <v>0.22</v>
       </c>
       <c r="F56" t="s">
         <v>35</v>
@@ -4471,7 +4471,7 @@
         <v>9</v>
       </c>
       <c r="E57">
-        <v>0.34</v>
+        <v>0.2</v>
       </c>
       <c r="F57" t="s">
         <v>35</v>
@@ -4491,7 +4491,7 @@
         <v>9</v>
       </c>
       <c r="E58">
-        <v>0.33</v>
+        <v>0.28</v>
       </c>
       <c r="F58" t="s">
         <v>35</v>
@@ -4511,7 +4511,7 @@
         <v>9</v>
       </c>
       <c r="E59">
-        <v>0.22</v>
+        <v>0.25</v>
       </c>
       <c r="F59" t="s">
         <v>35</v>
@@ -4531,7 +4531,7 @@
         <v>9</v>
       </c>
       <c r="E60">
-        <v>0.23</v>
+        <v>0.29</v>
       </c>
       <c r="F60" t="s">
         <v>35</v>
@@ -4551,7 +4551,7 @@
         <v>9</v>
       </c>
       <c r="E61">
-        <v>0.21</v>
+        <v>0.14</v>
       </c>
       <c r="F61" t="s">
         <v>35</v>
@@ -4571,7 +4571,7 @@
         <v>9</v>
       </c>
       <c r="E62">
-        <v>0.2</v>
+        <v>0.36</v>
       </c>
       <c r="F62" t="s">
         <v>35</v>
@@ -4591,7 +4591,7 @@
         <v>9</v>
       </c>
       <c r="E63">
-        <v>0.39</v>
+        <v>0.15</v>
       </c>
       <c r="F63" t="s">
         <v>35</v>
@@ -4611,7 +4611,7 @@
         <v>9</v>
       </c>
       <c r="E64">
-        <v>0.34</v>
+        <v>0.23</v>
       </c>
       <c r="F64" t="s">
         <v>35</v>
@@ -4631,7 +4631,7 @@
         <v>9</v>
       </c>
       <c r="E65">
-        <v>0.15</v>
+        <v>0.34</v>
       </c>
       <c r="F65" t="s">
         <v>35</v>
@@ -4651,7 +4651,7 @@
         <v>9</v>
       </c>
       <c r="E66">
-        <v>0.18</v>
+        <v>0.19</v>
       </c>
       <c r="F66" t="s">
         <v>60</v>
@@ -4691,7 +4691,7 @@
         <v>9</v>
       </c>
       <c r="E68">
-        <v>0.23</v>
+        <v>0.36</v>
       </c>
       <c r="F68" t="s">
         <v>60</v>
@@ -4711,7 +4711,7 @@
         <v>9</v>
       </c>
       <c r="E69">
-        <v>0.24</v>
+        <v>0.13</v>
       </c>
       <c r="F69" t="s">
         <v>60</v>
@@ -4731,7 +4731,7 @@
         <v>9</v>
       </c>
       <c r="E70">
-        <v>0.25</v>
+        <v>0.23</v>
       </c>
       <c r="F70" t="s">
         <v>60</v>
@@ -4751,7 +4751,7 @@
         <v>9</v>
       </c>
       <c r="E71">
-        <v>0.15</v>
+        <v>0.33</v>
       </c>
       <c r="F71" t="s">
         <v>60</v>
@@ -4771,7 +4771,7 @@
         <v>9</v>
       </c>
       <c r="E72">
-        <v>0.33</v>
+        <v>0.13</v>
       </c>
       <c r="F72" t="s">
         <v>60</v>
@@ -4791,7 +4791,7 @@
         <v>9</v>
       </c>
       <c r="E73">
-        <v>0.22</v>
+        <v>0.34</v>
       </c>
       <c r="F73" t="s">
         <v>60</v>
@@ -4811,7 +4811,7 @@
         <v>9</v>
       </c>
       <c r="E74">
-        <v>0.1</v>
+        <v>0.16</v>
       </c>
       <c r="F74" t="s">
         <v>60</v>
@@ -4831,7 +4831,7 @@
         <v>9</v>
       </c>
       <c r="E75">
-        <v>0.2</v>
+        <v>0.36</v>
       </c>
       <c r="F75" t="s">
         <v>60</v>
@@ -4851,7 +4851,7 @@
         <v>9</v>
       </c>
       <c r="E76">
-        <v>0.34</v>
+        <v>0.25</v>
       </c>
       <c r="F76" t="s">
         <v>60</v>
@@ -4871,7 +4871,7 @@
         <v>9</v>
       </c>
       <c r="E77">
-        <v>0.15</v>
+        <v>0.39</v>
       </c>
       <c r="F77" t="s">
         <v>60</v>
@@ -4891,7 +4891,7 @@
         <v>9</v>
       </c>
       <c r="E78">
-        <v>0.37</v>
+        <v>0.18</v>
       </c>
       <c r="F78" t="s">
         <v>60</v>
@@ -4911,7 +4911,7 @@
         <v>9</v>
       </c>
       <c r="E79">
-        <v>0.34</v>
+        <v>0.29</v>
       </c>
       <c r="F79" t="s">
         <v>60</v>
@@ -4931,7 +4931,7 @@
         <v>9</v>
       </c>
       <c r="E80">
-        <v>0.26</v>
+        <v>0.35</v>
       </c>
       <c r="F80" t="s">
         <v>60</v>
@@ -4951,7 +4951,7 @@
         <v>9</v>
       </c>
       <c r="E81">
-        <v>0.25</v>
+        <v>0.36</v>
       </c>
       <c r="F81" t="s">
         <v>60</v>
@@ -4971,7 +4971,7 @@
         <v>9</v>
       </c>
       <c r="E82">
-        <v>0.22</v>
+        <v>0.12</v>
       </c>
       <c r="F82" t="s">
         <v>10</v>
@@ -4991,7 +4991,7 @@
         <v>9</v>
       </c>
       <c r="E83">
-        <v>0.37</v>
+        <v>0.2</v>
       </c>
       <c r="F83" t="s">
         <v>10</v>
@@ -5011,7 +5011,7 @@
         <v>9</v>
       </c>
       <c r="E84">
-        <v>0.18</v>
+        <v>0.12</v>
       </c>
       <c r="F84" t="s">
         <v>10</v>
@@ -5031,7 +5031,7 @@
         <v>9</v>
       </c>
       <c r="E85">
-        <v>0.1</v>
+        <v>0.17</v>
       </c>
       <c r="F85" t="s">
         <v>10</v>
@@ -5051,7 +5051,7 @@
         <v>9</v>
       </c>
       <c r="E86">
-        <v>0.31</v>
+        <v>0.29</v>
       </c>
       <c r="F86" t="s">
         <v>10</v>
@@ -5071,7 +5071,7 @@
         <v>9</v>
       </c>
       <c r="E87">
-        <v>0.19</v>
+        <v>0.15</v>
       </c>
       <c r="F87" t="s">
         <v>10</v>
@@ -5091,7 +5091,7 @@
         <v>9</v>
       </c>
       <c r="E88">
-        <v>0.21</v>
+        <v>0.4</v>
       </c>
       <c r="F88" t="s">
         <v>10</v>
@@ -5111,7 +5111,7 @@
         <v>9</v>
       </c>
       <c r="E89">
-        <v>0.28</v>
+        <v>0.1</v>
       </c>
       <c r="F89" t="s">
         <v>10</v>
@@ -5131,7 +5131,7 @@
         <v>9</v>
       </c>
       <c r="E90">
-        <v>0.31</v>
+        <v>0.32</v>
       </c>
       <c r="F90" t="s">
         <v>10</v>
@@ -5151,7 +5151,7 @@
         <v>9</v>
       </c>
       <c r="E91">
-        <v>0.27</v>
+        <v>0.17</v>
       </c>
       <c r="F91" t="s">
         <v>35</v>
@@ -5171,7 +5171,7 @@
         <v>9</v>
       </c>
       <c r="E92">
-        <v>0.31</v>
+        <v>0.2</v>
       </c>
       <c r="F92" t="s">
         <v>35</v>
@@ -5191,7 +5191,7 @@
         <v>9</v>
       </c>
       <c r="E93">
-        <v>0.14</v>
+        <v>0.15</v>
       </c>
       <c r="F93" t="s">
         <v>35</v>
@@ -5211,7 +5211,7 @@
         <v>9</v>
       </c>
       <c r="E94">
-        <v>0.27</v>
+        <v>0.38</v>
       </c>
       <c r="F94" t="s">
         <v>35</v>
@@ -5231,7 +5231,7 @@
         <v>9</v>
       </c>
       <c r="E95">
-        <v>0.27</v>
+        <v>0.26</v>
       </c>
       <c r="F95" t="s">
         <v>35</v>
@@ -5251,7 +5251,7 @@
         <v>9</v>
       </c>
       <c r="E96">
-        <v>0.35</v>
+        <v>0.1</v>
       </c>
       <c r="F96" t="s">
         <v>35</v>
@@ -5271,7 +5271,7 @@
         <v>9</v>
       </c>
       <c r="E97">
-        <v>0.39</v>
+        <v>0.33</v>
       </c>
       <c r="F97" t="s">
         <v>35</v>
@@ -5291,7 +5291,7 @@
         <v>9</v>
       </c>
       <c r="E98">
-        <v>0.15</v>
+        <v>0.28</v>
       </c>
       <c r="F98" t="s">
         <v>35</v>
@@ -5311,7 +5311,7 @@
         <v>9</v>
       </c>
       <c r="E99">
-        <v>0.18</v>
+        <v>0.16</v>
       </c>
       <c r="F99" t="s">
         <v>35</v>
@@ -5331,7 +5331,7 @@
         <v>9</v>
       </c>
       <c r="E100">
-        <v>0.2</v>
+        <v>0.25</v>
       </c>
       <c r="F100" t="s">
         <v>60</v>
@@ -5351,7 +5351,7 @@
         <v>9</v>
       </c>
       <c r="E101">
-        <v>0.11</v>
+        <v>0.31</v>
       </c>
       <c r="F101" t="s">
         <v>60</v>
@@ -5371,7 +5371,7 @@
         <v>9</v>
       </c>
       <c r="E102">
-        <v>0.13</v>
+        <v>0.19</v>
       </c>
       <c r="F102" t="s">
         <v>60</v>
@@ -5391,7 +5391,7 @@
         <v>9</v>
       </c>
       <c r="E103">
-        <v>0.33</v>
+        <v>0.16</v>
       </c>
       <c r="F103" t="s">
         <v>60</v>
@@ -5411,7 +5411,7 @@
         <v>9</v>
       </c>
       <c r="E104">
-        <v>0.13</v>
+        <v>0.17</v>
       </c>
       <c r="F104" t="s">
         <v>60</v>
@@ -5431,7 +5431,7 @@
         <v>9</v>
       </c>
       <c r="E105">
-        <v>0.31</v>
+        <v>0.27</v>
       </c>
       <c r="F105" t="s">
         <v>60</v>
@@ -5451,7 +5451,7 @@
         <v>9</v>
       </c>
       <c r="E106">
-        <v>0.27</v>
+        <v>0.16</v>
       </c>
       <c r="F106" t="s">
         <v>60</v>
@@ -5471,7 +5471,7 @@
         <v>9</v>
       </c>
       <c r="E107">
-        <v>0.11</v>
+        <v>0.27</v>
       </c>
       <c r="F107" t="s">
         <v>60</v>
@@ -5491,7 +5491,7 @@
         <v>9</v>
       </c>
       <c r="E108">
-        <v>0.35</v>
+        <v>0.13</v>
       </c>
       <c r="F108" t="s">
         <v>60</v>
@@ -5511,7 +5511,7 @@
         <v>9</v>
       </c>
       <c r="E109">
-        <v>0.19</v>
+        <v>0.13</v>
       </c>
       <c r="F109" t="s">
         <v>60</v>
@@ -5531,7 +5531,7 @@
         <v>9</v>
       </c>
       <c r="E110">
-        <v>0.33</v>
+        <v>0.11</v>
       </c>
       <c r="F110" t="s">
         <v>60</v>
@@ -5551,7 +5551,7 @@
         <v>9</v>
       </c>
       <c r="E111">
-        <v>0.11</v>
+        <v>0.35</v>
       </c>
       <c r="F111" t="s">
         <v>60</v>
@@ -5571,7 +5571,7 @@
         <v>9</v>
       </c>
       <c r="E112">
-        <v>0.17</v>
+        <v>0.3</v>
       </c>
       <c r="F112" t="s">
         <v>10</v>
@@ -5591,7 +5591,7 @@
         <v>9</v>
       </c>
       <c r="E113">
-        <v>0.18</v>
+        <v>0.2</v>
       </c>
       <c r="F113" t="s">
         <v>10</v>
@@ -5611,7 +5611,7 @@
         <v>9</v>
       </c>
       <c r="E114">
-        <v>0.15</v>
+        <v>0.17</v>
       </c>
       <c r="F114" t="s">
         <v>10</v>
@@ -5631,7 +5631,7 @@
         <v>9</v>
       </c>
       <c r="E115">
-        <v>0.1</v>
+        <v>0.24</v>
       </c>
       <c r="F115" t="s">
         <v>10</v>
@@ -5651,7 +5651,7 @@
         <v>9</v>
       </c>
       <c r="E116">
-        <v>0.39</v>
+        <v>0.34</v>
       </c>
       <c r="F116" t="s">
         <v>10</v>
@@ -5671,7 +5671,7 @@
         <v>9</v>
       </c>
       <c r="E117">
-        <v>0.33</v>
+        <v>0.31</v>
       </c>
       <c r="F117" t="s">
         <v>10</v>
@@ -5691,7 +5691,7 @@
         <v>9</v>
       </c>
       <c r="E118">
-        <v>0.23</v>
+        <v>0.2</v>
       </c>
       <c r="F118" t="s">
         <v>10</v>
@@ -5711,7 +5711,7 @@
         <v>9</v>
       </c>
       <c r="E119">
-        <v>0.32</v>
+        <v>0.33</v>
       </c>
       <c r="F119" t="s">
         <v>10</v>
@@ -5731,7 +5731,7 @@
         <v>9</v>
       </c>
       <c r="E120">
-        <v>0.19</v>
+        <v>0.28</v>
       </c>
       <c r="F120" t="s">
         <v>10</v>
@@ -5751,7 +5751,7 @@
         <v>9</v>
       </c>
       <c r="E121">
-        <v>0.39</v>
+        <v>0.14</v>
       </c>
       <c r="F121" t="s">
         <v>10</v>
@@ -5771,7 +5771,7 @@
         <v>9</v>
       </c>
       <c r="E122">
-        <v>0.35</v>
+        <v>0.17</v>
       </c>
       <c r="F122" t="s">
         <v>10</v>
@@ -5791,7 +5791,7 @@
         <v>9</v>
       </c>
       <c r="E123">
-        <v>0.11</v>
+        <v>0.1</v>
       </c>
       <c r="F123" t="s">
         <v>10</v>
@@ -5811,7 +5811,7 @@
         <v>9</v>
       </c>
       <c r="E124">
-        <v>0.36</v>
+        <v>0.32</v>
       </c>
       <c r="F124" t="s">
         <v>10</v>
@@ -5831,7 +5831,7 @@
         <v>9</v>
       </c>
       <c r="E125">
-        <v>0.27</v>
+        <v>0.34</v>
       </c>
       <c r="F125" t="s">
         <v>10</v>
@@ -5851,7 +5851,7 @@
         <v>9</v>
       </c>
       <c r="E126">
-        <v>0.23</v>
+        <v>0.18</v>
       </c>
       <c r="F126" t="s">
         <v>10</v>
@@ -5871,7 +5871,7 @@
         <v>9</v>
       </c>
       <c r="E127">
-        <v>0.15</v>
+        <v>0.38</v>
       </c>
       <c r="F127" t="s">
         <v>35</v>
@@ -5891,7 +5891,7 @@
         <v>9</v>
       </c>
       <c r="E128">
-        <v>0.2</v>
+        <v>0.35</v>
       </c>
       <c r="F128" t="s">
         <v>35</v>
@@ -5911,7 +5911,7 @@
         <v>9</v>
       </c>
       <c r="E129">
-        <v>0.12</v>
+        <v>0.35</v>
       </c>
       <c r="F129" t="s">
         <v>35</v>
@@ -5931,7 +5931,7 @@
         <v>9</v>
       </c>
       <c r="E130">
-        <v>0.29</v>
+        <v>0.17</v>
       </c>
       <c r="F130" t="s">
         <v>35</v>
@@ -5951,7 +5951,7 @@
         <v>9</v>
       </c>
       <c r="E131">
-        <v>0.15</v>
+        <v>0.39</v>
       </c>
       <c r="F131" t="s">
         <v>35</v>
@@ -5971,7 +5971,7 @@
         <v>9</v>
       </c>
       <c r="E132">
-        <v>0.13</v>
+        <v>0.25</v>
       </c>
       <c r="F132" t="s">
         <v>35</v>
@@ -5991,7 +5991,7 @@
         <v>9</v>
       </c>
       <c r="E133">
-        <v>0.16</v>
+        <v>0.26</v>
       </c>
       <c r="F133" t="s">
         <v>35</v>
@@ -6011,7 +6011,7 @@
         <v>9</v>
       </c>
       <c r="E134">
-        <v>0.26</v>
+        <v>0.11</v>
       </c>
       <c r="F134" t="s">
         <v>35</v>
@@ -6031,7 +6031,7 @@
         <v>9</v>
       </c>
       <c r="E135">
-        <v>0.14</v>
+        <v>0.32</v>
       </c>
       <c r="F135" t="s">
         <v>35</v>
@@ -6051,7 +6051,7 @@
         <v>9</v>
       </c>
       <c r="E136">
-        <v>0.19</v>
+        <v>0.15</v>
       </c>
       <c r="F136" t="s">
         <v>35</v>
@@ -6071,7 +6071,7 @@
         <v>9</v>
       </c>
       <c r="E137">
-        <v>0.2</v>
+        <v>0.15</v>
       </c>
       <c r="F137" t="s">
         <v>35</v>
@@ -6091,7 +6091,7 @@
         <v>9</v>
       </c>
       <c r="E138">
-        <v>0.16</v>
+        <v>0.12</v>
       </c>
       <c r="F138" t="s">
         <v>35</v>
@@ -6111,7 +6111,7 @@
         <v>9</v>
       </c>
       <c r="E139">
-        <v>0.17</v>
+        <v>0.11</v>
       </c>
       <c r="F139" t="s">
         <v>35</v>
@@ -6131,7 +6131,7 @@
         <v>9</v>
       </c>
       <c r="E140">
-        <v>0.35</v>
+        <v>0.21</v>
       </c>
       <c r="F140" t="s">
         <v>35</v>
@@ -6151,7 +6151,7 @@
         <v>9</v>
       </c>
       <c r="E141">
-        <v>0.22</v>
+        <v>0.34</v>
       </c>
       <c r="F141" t="s">
         <v>35</v>
@@ -6171,7 +6171,7 @@
         <v>9</v>
       </c>
       <c r="E142">
-        <v>0.34</v>
+        <v>0.16</v>
       </c>
       <c r="F142" t="s">
         <v>60</v>
@@ -6191,7 +6191,7 @@
         <v>9</v>
       </c>
       <c r="E143">
-        <v>0.31</v>
+        <v>0.3</v>
       </c>
       <c r="F143" t="s">
         <v>60</v>
@@ -6211,7 +6211,7 @@
         <v>9</v>
       </c>
       <c r="E144">
-        <v>0.26</v>
+        <v>0.38</v>
       </c>
       <c r="F144" t="s">
         <v>60</v>
@@ -6231,7 +6231,7 @@
         <v>9</v>
       </c>
       <c r="E145">
-        <v>0.32</v>
+        <v>0.18</v>
       </c>
       <c r="F145" t="s">
         <v>60</v>
@@ -6251,7 +6251,7 @@
         <v>9</v>
       </c>
       <c r="E146">
-        <v>0.35</v>
+        <v>0.34</v>
       </c>
       <c r="F146" t="s">
         <v>60</v>
@@ -6271,7 +6271,7 @@
         <v>9</v>
       </c>
       <c r="E147">
-        <v>0.29</v>
+        <v>0.3</v>
       </c>
       <c r="F147" t="s">
         <v>60</v>
@@ -6291,7 +6291,7 @@
         <v>9</v>
       </c>
       <c r="E148">
-        <v>0.35</v>
+        <v>0.26</v>
       </c>
       <c r="F148" t="s">
         <v>60</v>
@@ -6311,7 +6311,7 @@
         <v>9</v>
       </c>
       <c r="E149">
-        <v>0.17</v>
+        <v>0.13</v>
       </c>
       <c r="F149" t="s">
         <v>60</v>
@@ -6331,7 +6331,7 @@
         <v>9</v>
       </c>
       <c r="E150">
-        <v>0.16</v>
+        <v>0.24</v>
       </c>
       <c r="F150" t="s">
         <v>60</v>
@@ -6351,7 +6351,7 @@
         <v>9</v>
       </c>
       <c r="E151">
-        <v>0.23</v>
+        <v>0.11</v>
       </c>
       <c r="F151" t="s">
         <v>60</v>
@@ -6371,7 +6371,7 @@
         <v>9</v>
       </c>
       <c r="E152">
-        <v>0.17</v>
+        <v>0.32</v>
       </c>
       <c r="F152" t="s">
         <v>60</v>
@@ -6391,7 +6391,7 @@
         <v>9</v>
       </c>
       <c r="E153">
-        <v>0.4</v>
+        <v>0.26</v>
       </c>
       <c r="F153" t="s">
         <v>60</v>
@@ -6411,7 +6411,7 @@
         <v>9</v>
       </c>
       <c r="E154">
-        <v>0.21</v>
+        <v>0.36</v>
       </c>
       <c r="F154" t="s">
         <v>60</v>
@@ -6431,7 +6431,7 @@
         <v>9</v>
       </c>
       <c r="E155">
-        <v>0.13</v>
+        <v>0.28</v>
       </c>
       <c r="F155" t="s">
         <v>60</v>
@@ -6451,7 +6451,7 @@
         <v>9</v>
       </c>
       <c r="E156">
-        <v>0.12</v>
+        <v>0.2</v>
       </c>
       <c r="F156" t="s">
         <v>60</v>
@@ -6471,7 +6471,7 @@
         <v>9</v>
       </c>
       <c r="E157">
-        <v>0.19</v>
+        <v>0.34</v>
       </c>
       <c r="F157" t="s">
         <v>60</v>
@@ -6491,7 +6491,7 @@
         <v>9</v>
       </c>
       <c r="E158">
-        <v>0.37</v>
+        <v>0.38</v>
       </c>
       <c r="F158" t="s">
         <v>60</v>
@@ -6511,7 +6511,7 @@
         <v>9</v>
       </c>
       <c r="E159">
-        <v>0.19</v>
+        <v>0.28</v>
       </c>
       <c r="F159" t="s">
         <v>60</v>
@@ -6531,7 +6531,7 @@
         <v>9</v>
       </c>
       <c r="E160">
-        <v>0.23</v>
+        <v>0.36</v>
       </c>
       <c r="F160" t="s">
         <v>60</v>
@@ -6551,7 +6551,7 @@
         <v>9</v>
       </c>
       <c r="E161">
-        <v>0.13</v>
+        <v>0.23</v>
       </c>
       <c r="F161" t="s">
         <v>60</v>
@@ -6571,7 +6571,7 @@
         <v>9</v>
       </c>
       <c r="E162">
-        <v>0.24</v>
+        <v>0.32</v>
       </c>
       <c r="F162" t="s">
         <v>10</v>
@@ -6591,7 +6591,7 @@
         <v>9</v>
       </c>
       <c r="E163">
-        <v>0.17</v>
+        <v>0.38</v>
       </c>
       <c r="F163" t="s">
         <v>10</v>
@@ -6611,7 +6611,7 @@
         <v>9</v>
       </c>
       <c r="E164">
-        <v>0.21</v>
+        <v>0.17</v>
       </c>
       <c r="F164" t="s">
         <v>10</v>
@@ -6631,7 +6631,7 @@
         <v>9</v>
       </c>
       <c r="E165">
-        <v>0.15</v>
+        <v>0.32</v>
       </c>
       <c r="F165" t="s">
         <v>10</v>
@@ -6651,7 +6651,7 @@
         <v>9</v>
       </c>
       <c r="E166">
-        <v>0.23</v>
+        <v>0.19</v>
       </c>
       <c r="F166" t="s">
         <v>10</v>
@@ -6671,7 +6671,7 @@
         <v>9</v>
       </c>
       <c r="E167">
-        <v>0.17</v>
+        <v>0.37</v>
       </c>
       <c r="F167" t="s">
         <v>10</v>
@@ -6691,7 +6691,7 @@
         <v>9</v>
       </c>
       <c r="E168">
-        <v>0.36</v>
+        <v>0.3</v>
       </c>
       <c r="F168" t="s">
         <v>10</v>
@@ -6711,7 +6711,7 @@
         <v>9</v>
       </c>
       <c r="E169">
-        <v>0.25</v>
+        <v>0.16</v>
       </c>
       <c r="F169" t="s">
         <v>10</v>
@@ -6731,7 +6731,7 @@
         <v>9</v>
       </c>
       <c r="E170">
-        <v>0.28</v>
+        <v>0.22</v>
       </c>
       <c r="F170" t="s">
         <v>10</v>
@@ -6751,7 +6751,7 @@
         <v>9</v>
       </c>
       <c r="E171">
-        <v>0.22</v>
+        <v>0.16</v>
       </c>
       <c r="F171" t="s">
         <v>10</v>
@@ -6771,7 +6771,7 @@
         <v>9</v>
       </c>
       <c r="E172">
-        <v>0.16</v>
+        <v>0.18</v>
       </c>
       <c r="F172" t="s">
         <v>10</v>
@@ -6791,7 +6791,7 @@
         <v>9</v>
       </c>
       <c r="E173">
-        <v>0.23</v>
+        <v>0.35</v>
       </c>
       <c r="F173" t="s">
         <v>10</v>
@@ -6811,7 +6811,7 @@
         <v>9</v>
       </c>
       <c r="E174">
-        <v>0.18</v>
+        <v>0.2</v>
       </c>
       <c r="F174" t="s">
         <v>10</v>
@@ -6831,7 +6831,7 @@
         <v>9</v>
       </c>
       <c r="E175">
-        <v>0.37</v>
+        <v>0.3</v>
       </c>
       <c r="F175" t="s">
         <v>10</v>
@@ -6851,7 +6851,7 @@
         <v>9</v>
       </c>
       <c r="E176">
-        <v>0.28</v>
+        <v>0.39</v>
       </c>
       <c r="F176" t="s">
         <v>10</v>
@@ -6871,7 +6871,7 @@
         <v>9</v>
       </c>
       <c r="E177">
-        <v>0.17</v>
+        <v>0.26</v>
       </c>
       <c r="F177" t="s">
         <v>35</v>
@@ -6891,7 +6891,7 @@
         <v>9</v>
       </c>
       <c r="E178">
-        <v>0.31</v>
+        <v>0.24</v>
       </c>
       <c r="F178" t="s">
         <v>35</v>
@@ -6911,7 +6911,7 @@
         <v>9</v>
       </c>
       <c r="E179">
-        <v>0.33</v>
+        <v>0.24</v>
       </c>
       <c r="F179" t="s">
         <v>35</v>
@@ -6931,7 +6931,7 @@
         <v>9</v>
       </c>
       <c r="E180">
-        <v>0.19</v>
+        <v>0.2</v>
       </c>
       <c r="F180" t="s">
         <v>35</v>
@@ -6951,7 +6951,7 @@
         <v>9</v>
       </c>
       <c r="E181">
-        <v>0.27</v>
+        <v>0.22</v>
       </c>
       <c r="F181" t="s">
         <v>35</v>
@@ -6971,7 +6971,7 @@
         <v>9</v>
       </c>
       <c r="E182">
-        <v>0.13</v>
+        <v>0.22</v>
       </c>
       <c r="F182" t="s">
         <v>35</v>
@@ -6991,7 +6991,7 @@
         <v>9</v>
       </c>
       <c r="E183">
-        <v>0.31</v>
+        <v>0.29</v>
       </c>
       <c r="F183" t="s">
         <v>35</v>
@@ -7051,7 +7051,7 @@
         <v>9</v>
       </c>
       <c r="E186">
-        <v>0.12</v>
+        <v>0.31</v>
       </c>
       <c r="F186" t="s">
         <v>35</v>
@@ -7071,7 +7071,7 @@
         <v>9</v>
       </c>
       <c r="E187">
-        <v>0.24</v>
+        <v>0.31</v>
       </c>
       <c r="F187" t="s">
         <v>35</v>
@@ -7091,7 +7091,7 @@
         <v>9</v>
       </c>
       <c r="E188">
-        <v>0.29</v>
+        <v>0.32</v>
       </c>
       <c r="F188" t="s">
         <v>35</v>
@@ -7111,7 +7111,7 @@
         <v>9</v>
       </c>
       <c r="E189">
-        <v>0.29</v>
+        <v>0.34</v>
       </c>
       <c r="F189" t="s">
         <v>35</v>
@@ -7131,7 +7131,7 @@
         <v>9</v>
       </c>
       <c r="E190">
-        <v>0.38</v>
+        <v>0.17</v>
       </c>
       <c r="F190" t="s">
         <v>35</v>
@@ -7151,7 +7151,7 @@
         <v>9</v>
       </c>
       <c r="E191">
-        <v>0.39</v>
+        <v>0.19</v>
       </c>
       <c r="F191" t="s">
         <v>35</v>
@@ -7171,7 +7171,7 @@
         <v>9</v>
       </c>
       <c r="E192">
-        <v>0.2</v>
+        <v>0.35</v>
       </c>
       <c r="F192" t="s">
         <v>60</v>
@@ -7191,7 +7191,7 @@
         <v>9</v>
       </c>
       <c r="E193">
-        <v>0.25</v>
+        <v>0.32</v>
       </c>
       <c r="F193" t="s">
         <v>60</v>
@@ -7211,7 +7211,7 @@
         <v>9</v>
       </c>
       <c r="E194">
-        <v>0.13</v>
+        <v>0.36</v>
       </c>
       <c r="F194" t="s">
         <v>60</v>
@@ -7231,7 +7231,7 @@
         <v>9</v>
       </c>
       <c r="E195">
-        <v>0.21</v>
+        <v>0.26</v>
       </c>
       <c r="F195" t="s">
         <v>60</v>
@@ -7251,7 +7251,7 @@
         <v>9</v>
       </c>
       <c r="E196">
-        <v>0.32</v>
+        <v>0.36</v>
       </c>
       <c r="F196" t="s">
         <v>60</v>
@@ -7271,7 +7271,7 @@
         <v>9</v>
       </c>
       <c r="E197">
-        <v>0.29</v>
+        <v>0.25</v>
       </c>
       <c r="F197" t="s">
         <v>60</v>
@@ -7291,7 +7291,7 @@
         <v>9</v>
       </c>
       <c r="E198">
-        <v>0.16</v>
+        <v>0.4</v>
       </c>
       <c r="F198" t="s">
         <v>60</v>
@@ -7311,7 +7311,7 @@
         <v>9</v>
       </c>
       <c r="E199">
-        <v>0.26</v>
+        <v>0.24</v>
       </c>
       <c r="F199" t="s">
         <v>60</v>
@@ -7331,7 +7331,7 @@
         <v>9</v>
       </c>
       <c r="E200">
-        <v>0.32</v>
+        <v>0.14</v>
       </c>
       <c r="F200" t="s">
         <v>60</v>
@@ -7351,7 +7351,7 @@
         <v>9</v>
       </c>
       <c r="E201">
-        <v>0.16</v>
+        <v>0.27</v>
       </c>
       <c r="F201" t="s">
         <v>60</v>
@@ -7371,7 +7371,7 @@
         <v>9</v>
       </c>
       <c r="E202">
-        <v>0.34</v>
+        <v>0.13</v>
       </c>
       <c r="F202" t="s">
         <v>60</v>
@@ -7391,7 +7391,7 @@
         <v>9</v>
       </c>
       <c r="E203">
-        <v>0.38</v>
+        <v>0.15</v>
       </c>
       <c r="F203" t="s">
         <v>60</v>
@@ -7411,7 +7411,7 @@
         <v>9</v>
       </c>
       <c r="E204">
-        <v>0.33</v>
+        <v>0.29</v>
       </c>
       <c r="F204" t="s">
         <v>60</v>
@@ -7431,7 +7431,7 @@
         <v>9</v>
       </c>
       <c r="E205">
-        <v>0.28</v>
+        <v>0.34</v>
       </c>
       <c r="F205" t="s">
         <v>60</v>
@@ -7451,7 +7451,7 @@
         <v>9</v>
       </c>
       <c r="E206">
-        <v>0.4</v>
+        <v>0.16</v>
       </c>
       <c r="F206" t="s">
         <v>60</v>
@@ -7471,7 +7471,7 @@
         <v>9</v>
       </c>
       <c r="E207">
-        <v>0.13</v>
+        <v>0.17</v>
       </c>
       <c r="F207" t="s">
         <v>60</v>
@@ -7491,7 +7491,7 @@
         <v>9</v>
       </c>
       <c r="E208">
-        <v>0.29</v>
+        <v>0.27</v>
       </c>
       <c r="F208" t="s">
         <v>60</v>
@@ -7511,7 +7511,7 @@
         <v>9</v>
       </c>
       <c r="E209">
-        <v>0.4</v>
+        <v>0.12</v>
       </c>
       <c r="F209" t="s">
         <v>60</v>
@@ -7531,7 +7531,7 @@
         <v>9</v>
       </c>
       <c r="E210">
-        <v>0.23</v>
+        <v>0.18</v>
       </c>
       <c r="F210" t="s">
         <v>60</v>
@@ -7551,7 +7551,7 @@
         <v>9</v>
       </c>
       <c r="E211">
-        <v>0.37</v>
+        <v>0.33</v>
       </c>
       <c r="F211" t="s">
         <v>60</v>
@@ -7571,7 +7571,7 @@
         <v>9</v>
       </c>
       <c r="E212">
-        <v>0.28</v>
+        <v>0.27</v>
       </c>
       <c r="F212" t="s">
         <v>10</v>
@@ -7591,7 +7591,7 @@
         <v>9</v>
       </c>
       <c r="E213">
-        <v>0.23</v>
+        <v>0.34</v>
       </c>
       <c r="F213" t="s">
         <v>10</v>
@@ -7611,7 +7611,7 @@
         <v>9</v>
       </c>
       <c r="E214">
-        <v>0.32</v>
+        <v>0.22</v>
       </c>
       <c r="F214" t="s">
         <v>10</v>
@@ -7631,7 +7631,7 @@
         <v>9</v>
       </c>
       <c r="E215">
-        <v>0.26</v>
+        <v>0.17</v>
       </c>
       <c r="F215" t="s">
         <v>10</v>
@@ -7651,7 +7651,7 @@
         <v>9</v>
       </c>
       <c r="E216">
-        <v>0.24</v>
+        <v>0.37</v>
       </c>
       <c r="F216" t="s">
         <v>10</v>
@@ -7671,7 +7671,7 @@
         <v>9</v>
       </c>
       <c r="E217">
-        <v>0.27</v>
+        <v>0.3</v>
       </c>
       <c r="F217" t="s">
         <v>10</v>
@@ -7691,7 +7691,7 @@
         <v>9</v>
       </c>
       <c r="E218">
-        <v>0.34</v>
+        <v>0.17</v>
       </c>
       <c r="F218" t="s">
         <v>10</v>
@@ -7711,7 +7711,7 @@
         <v>9</v>
       </c>
       <c r="E219">
-        <v>0.15</v>
+        <v>0.14</v>
       </c>
       <c r="F219" t="s">
         <v>10</v>
@@ -7731,7 +7731,7 @@
         <v>9</v>
       </c>
       <c r="E220">
-        <v>0.27</v>
+        <v>0.17</v>
       </c>
       <c r="F220" t="s">
         <v>10</v>
@@ -7751,7 +7751,7 @@
         <v>9</v>
       </c>
       <c r="E221">
-        <v>0.36</v>
+        <v>0.13</v>
       </c>
       <c r="F221" t="s">
         <v>10</v>
@@ -7771,7 +7771,7 @@
         <v>9</v>
       </c>
       <c r="E222">
-        <v>0.28</v>
+        <v>0.36</v>
       </c>
       <c r="F222" t="s">
         <v>10</v>
@@ -7791,7 +7791,7 @@
         <v>9</v>
       </c>
       <c r="E223">
-        <v>0.12</v>
+        <v>0.1</v>
       </c>
       <c r="F223" t="s">
         <v>10</v>
@@ -7811,7 +7811,7 @@
         <v>9</v>
       </c>
       <c r="E224">
-        <v>0.26</v>
+        <v>0.11</v>
       </c>
       <c r="F224" t="s">
         <v>10</v>
@@ -7831,7 +7831,7 @@
         <v>9</v>
       </c>
       <c r="E225">
-        <v>0.36</v>
+        <v>0.11</v>
       </c>
       <c r="F225" t="s">
         <v>10</v>
@@ -7851,7 +7851,7 @@
         <v>9</v>
       </c>
       <c r="E226">
-        <v>0.26</v>
+        <v>0.13</v>
       </c>
       <c r="F226" t="s">
         <v>10</v>
@@ -7871,7 +7871,7 @@
         <v>9</v>
       </c>
       <c r="E227">
-        <v>0.16</v>
+        <v>0.26</v>
       </c>
       <c r="F227" t="s">
         <v>35</v>
@@ -7911,7 +7911,7 @@
         <v>9</v>
       </c>
       <c r="E229">
-        <v>0.39</v>
+        <v>0.17</v>
       </c>
       <c r="F229" t="s">
         <v>35</v>
@@ -7931,7 +7931,7 @@
         <v>9</v>
       </c>
       <c r="E230">
-        <v>0.25</v>
+        <v>0.35</v>
       </c>
       <c r="F230" t="s">
         <v>35</v>
@@ -7951,7 +7951,7 @@
         <v>9</v>
       </c>
       <c r="E231">
-        <v>0.34</v>
+        <v>0.29</v>
       </c>
       <c r="F231" t="s">
         <v>35</v>
@@ -7971,7 +7971,7 @@
         <v>9</v>
       </c>
       <c r="E232">
-        <v>0.38</v>
+        <v>0.19</v>
       </c>
       <c r="F232" t="s">
         <v>35</v>
@@ -7991,7 +7991,7 @@
         <v>9</v>
       </c>
       <c r="E233">
-        <v>0.23</v>
+        <v>0.37</v>
       </c>
       <c r="F233" t="s">
         <v>35</v>
@@ -8011,7 +8011,7 @@
         <v>9</v>
       </c>
       <c r="E234">
-        <v>0.37</v>
+        <v>0.15</v>
       </c>
       <c r="F234" t="s">
         <v>35</v>
@@ -8031,7 +8031,7 @@
         <v>9</v>
       </c>
       <c r="E235">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="F235" t="s">
         <v>35</v>
@@ -8051,7 +8051,7 @@
         <v>9</v>
       </c>
       <c r="E236">
-        <v>0.16</v>
+        <v>0.17</v>
       </c>
       <c r="F236" t="s">
         <v>35</v>
@@ -8071,7 +8071,7 @@
         <v>9</v>
       </c>
       <c r="E237">
-        <v>0.2</v>
+        <v>0.35</v>
       </c>
       <c r="F237" t="s">
         <v>35</v>
@@ -8091,7 +8091,7 @@
         <v>9</v>
       </c>
       <c r="E238">
-        <v>0.36</v>
+        <v>0.32</v>
       </c>
       <c r="F238" t="s">
         <v>35</v>
@@ -8111,7 +8111,7 @@
         <v>9</v>
       </c>
       <c r="E239">
-        <v>0.37</v>
+        <v>0.35</v>
       </c>
       <c r="F239" t="s">
         <v>35</v>
@@ -8131,7 +8131,7 @@
         <v>9</v>
       </c>
       <c r="E240">
-        <v>0.2</v>
+        <v>0.15</v>
       </c>
       <c r="F240" t="s">
         <v>35</v>
@@ -8151,7 +8151,7 @@
         <v>9</v>
       </c>
       <c r="E241">
-        <v>0.14</v>
+        <v>0.16</v>
       </c>
       <c r="F241" t="s">
         <v>35</v>
@@ -8171,7 +8171,7 @@
         <v>9</v>
       </c>
       <c r="E242">
-        <v>0.11</v>
+        <v>0.16</v>
       </c>
       <c r="F242" t="s">
         <v>60</v>
@@ -8191,7 +8191,7 @@
         <v>9</v>
       </c>
       <c r="E243">
-        <v>0.24</v>
+        <v>0.28</v>
       </c>
       <c r="F243" t="s">
         <v>60</v>
@@ -8211,7 +8211,7 @@
         <v>9</v>
       </c>
       <c r="E244">
-        <v>0.38</v>
+        <v>0.23</v>
       </c>
       <c r="F244" t="s">
         <v>60</v>
@@ -8231,7 +8231,7 @@
         <v>9</v>
       </c>
       <c r="E245">
-        <v>0.29</v>
+        <v>0.2</v>
       </c>
       <c r="F245" t="s">
         <v>60</v>
@@ -8251,7 +8251,7 @@
         <v>9</v>
       </c>
       <c r="E246">
-        <v>0.31</v>
+        <v>0.23</v>
       </c>
       <c r="F246" t="s">
         <v>60</v>
@@ -8271,7 +8271,7 @@
         <v>9</v>
       </c>
       <c r="E247">
-        <v>0.34</v>
+        <v>0.36</v>
       </c>
       <c r="F247" t="s">
         <v>60</v>
@@ -8291,7 +8291,7 @@
         <v>9</v>
       </c>
       <c r="E248">
-        <v>0.17</v>
+        <v>0.32</v>
       </c>
       <c r="F248" t="s">
         <v>60</v>
@@ -8311,7 +8311,7 @@
         <v>9</v>
       </c>
       <c r="E249">
-        <v>0.37</v>
+        <v>0.12</v>
       </c>
       <c r="F249" t="s">
         <v>60</v>
@@ -8331,7 +8331,7 @@
         <v>9</v>
       </c>
       <c r="E250">
-        <v>0.22</v>
+        <v>0.11</v>
       </c>
       <c r="F250" t="s">
         <v>60</v>
@@ -8351,7 +8351,7 @@
         <v>9</v>
       </c>
       <c r="E251">
-        <v>0.18</v>
+        <v>0.38</v>
       </c>
       <c r="F251" t="s">
         <v>60</v>
@@ -8371,7 +8371,7 @@
         <v>9</v>
       </c>
       <c r="E252">
-        <v>0.29</v>
+        <v>0.15</v>
       </c>
       <c r="F252" t="s">
         <v>60</v>
@@ -8391,7 +8391,7 @@
         <v>9</v>
       </c>
       <c r="E253">
-        <v>0.25</v>
+        <v>0.38</v>
       </c>
       <c r="F253" t="s">
         <v>60</v>
@@ -8411,7 +8411,7 @@
         <v>9</v>
       </c>
       <c r="E254">
-        <v>0.29</v>
+        <v>0.25</v>
       </c>
       <c r="F254" t="s">
         <v>60</v>
@@ -8431,7 +8431,7 @@
         <v>9</v>
       </c>
       <c r="E255">
-        <v>0.28</v>
+        <v>0.35</v>
       </c>
       <c r="F255" t="s">
         <v>60</v>
@@ -8451,7 +8451,7 @@
         <v>9</v>
       </c>
       <c r="E256">
-        <v>0.24</v>
+        <v>0.11</v>
       </c>
       <c r="F256" t="s">
         <v>60</v>
@@ -8471,7 +8471,7 @@
         <v>9</v>
       </c>
       <c r="E257">
-        <v>0.29</v>
+        <v>0.28</v>
       </c>
       <c r="F257" t="s">
         <v>60</v>
@@ -8491,7 +8491,7 @@
         <v>9</v>
       </c>
       <c r="E258">
-        <v>0.38</v>
+        <v>0.24</v>
       </c>
       <c r="F258" t="s">
         <v>60</v>
@@ -8511,7 +8511,7 @@
         <v>9</v>
       </c>
       <c r="E259">
-        <v>0.14</v>
+        <v>0.37</v>
       </c>
       <c r="F259" t="s">
         <v>60</v>
@@ -8531,7 +8531,7 @@
         <v>9</v>
       </c>
       <c r="E260">
-        <v>0.13</v>
+        <v>0.4</v>
       </c>
       <c r="F260" t="s">
         <v>60</v>
@@ -8551,7 +8551,7 @@
         <v>9</v>
       </c>
       <c r="E261">
-        <v>0.34</v>
+        <v>0.25</v>
       </c>
       <c r="F261" t="s">
         <v>60</v>
@@ -8571,7 +8571,7 @@
         <v>9</v>
       </c>
       <c r="E262">
-        <v>0.27</v>
+        <v>0.21</v>
       </c>
       <c r="F262" t="s">
         <v>10</v>
@@ -8591,7 +8591,7 @@
         <v>9</v>
       </c>
       <c r="E263">
-        <v>0.12</v>
+        <v>0.22</v>
       </c>
       <c r="F263" t="s">
         <v>10</v>
@@ -8611,7 +8611,7 @@
         <v>9</v>
       </c>
       <c r="E264">
-        <v>0.31</v>
+        <v>0.39</v>
       </c>
       <c r="F264" t="s">
         <v>10</v>
@@ -8631,7 +8631,7 @@
         <v>9</v>
       </c>
       <c r="E265">
-        <v>0.37</v>
+        <v>0.17</v>
       </c>
       <c r="F265" t="s">
         <v>10</v>
@@ -8651,7 +8651,7 @@
         <v>9</v>
       </c>
       <c r="E266">
-        <v>0.39</v>
+        <v>0.24</v>
       </c>
       <c r="F266" t="s">
         <v>10</v>
@@ -8671,7 +8671,7 @@
         <v>9</v>
       </c>
       <c r="E267">
-        <v>0.28</v>
+        <v>0.32</v>
       </c>
       <c r="F267" t="s">
         <v>10</v>
@@ -8691,7 +8691,7 @@
         <v>9</v>
       </c>
       <c r="E268">
-        <v>0.18</v>
+        <v>0.37</v>
       </c>
       <c r="F268" t="s">
         <v>10</v>
@@ -8711,7 +8711,7 @@
         <v>9</v>
       </c>
       <c r="E269">
-        <v>0.25</v>
+        <v>0.31</v>
       </c>
       <c r="F269" t="s">
         <v>10</v>
@@ -8731,7 +8731,7 @@
         <v>9</v>
       </c>
       <c r="E270">
-        <v>0.35</v>
+        <v>0.3</v>
       </c>
       <c r="F270" t="s">
         <v>10</v>
@@ -8751,7 +8751,7 @@
         <v>9</v>
       </c>
       <c r="E271">
-        <v>0.22</v>
+        <v>0.14</v>
       </c>
       <c r="F271" t="s">
         <v>10</v>
@@ -8771,7 +8771,7 @@
         <v>9</v>
       </c>
       <c r="E272">
-        <v>0.17</v>
+        <v>0.26</v>
       </c>
       <c r="F272" t="s">
         <v>10</v>
@@ -8791,7 +8791,7 @@
         <v>9</v>
       </c>
       <c r="E273">
-        <v>0.33</v>
+        <v>0.12</v>
       </c>
       <c r="F273" t="s">
         <v>10</v>
@@ -8811,7 +8811,7 @@
         <v>9</v>
       </c>
       <c r="E274">
-        <v>0.32</v>
+        <v>0.27</v>
       </c>
       <c r="F274" t="s">
         <v>35</v>
@@ -8831,7 +8831,7 @@
         <v>9</v>
       </c>
       <c r="E275">
-        <v>0.11</v>
+        <v>0.29</v>
       </c>
       <c r="F275" t="s">
         <v>35</v>
@@ -8851,7 +8851,7 @@
         <v>9</v>
       </c>
       <c r="E276">
-        <v>0.15</v>
+        <v>0.17</v>
       </c>
       <c r="F276" t="s">
         <v>35</v>
@@ -8871,7 +8871,7 @@
         <v>9</v>
       </c>
       <c r="E277">
-        <v>0.4</v>
+        <v>0.37</v>
       </c>
       <c r="F277" t="s">
         <v>35</v>
@@ -8891,7 +8891,7 @@
         <v>9</v>
       </c>
       <c r="E278">
-        <v>0.33</v>
+        <v>0.21</v>
       </c>
       <c r="F278" t="s">
         <v>35</v>
@@ -8911,7 +8911,7 @@
         <v>9</v>
       </c>
       <c r="E279">
-        <v>0.28</v>
+        <v>0.12</v>
       </c>
       <c r="F279" t="s">
         <v>35</v>
@@ -8931,7 +8931,7 @@
         <v>9</v>
       </c>
       <c r="E280">
-        <v>0.13</v>
+        <v>0.28</v>
       </c>
       <c r="F280" t="s">
         <v>35</v>
@@ -8951,7 +8951,7 @@
         <v>9</v>
       </c>
       <c r="E281">
-        <v>0.33</v>
+        <v>0.36</v>
       </c>
       <c r="F281" t="s">
         <v>35</v>
@@ -8971,7 +8971,7 @@
         <v>9</v>
       </c>
       <c r="E282">
-        <v>0.36</v>
+        <v>0.32</v>
       </c>
       <c r="F282" t="s">
         <v>35</v>
@@ -8991,7 +8991,7 @@
         <v>9</v>
       </c>
       <c r="E283">
-        <v>0.16</v>
+        <v>0.38</v>
       </c>
       <c r="F283" t="s">
         <v>35</v>
@@ -9011,7 +9011,7 @@
         <v>9</v>
       </c>
       <c r="E284">
-        <v>0.12</v>
+        <v>0.14</v>
       </c>
       <c r="F284" t="s">
         <v>35</v>
@@ -9031,7 +9031,7 @@
         <v>9</v>
       </c>
       <c r="E285">
-        <v>0.23</v>
+        <v>0.16</v>
       </c>
       <c r="F285" t="s">
         <v>35</v>
@@ -9051,7 +9051,7 @@
         <v>9</v>
       </c>
       <c r="E286">
-        <v>0.27</v>
+        <v>0.33</v>
       </c>
       <c r="F286" t="s">
         <v>60</v>
@@ -9091,7 +9091,7 @@
         <v>9</v>
       </c>
       <c r="E288">
-        <v>0.14</v>
+        <v>0.12</v>
       </c>
       <c r="F288" t="s">
         <v>60</v>
@@ -9111,7 +9111,7 @@
         <v>9</v>
       </c>
       <c r="E289">
-        <v>0.26</v>
+        <v>0.27</v>
       </c>
       <c r="F289" t="s">
         <v>60</v>
@@ -9151,7 +9151,7 @@
         <v>9</v>
       </c>
       <c r="E291">
-        <v>0.24</v>
+        <v>0.14</v>
       </c>
       <c r="F291" t="s">
         <v>60</v>
@@ -9171,7 +9171,7 @@
         <v>9</v>
       </c>
       <c r="E292">
-        <v>0.11</v>
+        <v>0.37</v>
       </c>
       <c r="F292" t="s">
         <v>60</v>
@@ -9191,7 +9191,7 @@
         <v>9</v>
       </c>
       <c r="E293">
-        <v>0.27</v>
+        <v>0.39</v>
       </c>
       <c r="F293" t="s">
         <v>60</v>
@@ -9211,7 +9211,7 @@
         <v>9</v>
       </c>
       <c r="E294">
-        <v>0.4</v>
+        <v>0.27</v>
       </c>
       <c r="F294" t="s">
         <v>60</v>
@@ -9231,7 +9231,7 @@
         <v>9</v>
       </c>
       <c r="E295">
-        <v>0.1</v>
+        <v>0.32</v>
       </c>
       <c r="F295" t="s">
         <v>60</v>
@@ -9251,7 +9251,7 @@
         <v>9</v>
       </c>
       <c r="E296">
-        <v>0.34</v>
+        <v>0.16</v>
       </c>
       <c r="F296" t="s">
         <v>60</v>
@@ -9271,7 +9271,7 @@
         <v>9</v>
       </c>
       <c r="E297">
-        <v>0.33</v>
+        <v>0.37</v>
       </c>
       <c r="F297" t="s">
         <v>60</v>
@@ -9311,7 +9311,7 @@
         <v>9</v>
       </c>
       <c r="E299">
-        <v>0.12</v>
+        <v>0.33</v>
       </c>
       <c r="F299" t="s">
         <v>60</v>
@@ -9331,7 +9331,7 @@
         <v>9</v>
       </c>
       <c r="E300">
-        <v>0.18</v>
+        <v>0.26</v>
       </c>
       <c r="F300" t="s">
         <v>60</v>
@@ -9351,7 +9351,7 @@
         <v>9</v>
       </c>
       <c r="E301">
-        <v>0.22</v>
+        <v>0.26</v>
       </c>
       <c r="F301" t="s">
         <v>60</v>
@@ -9371,7 +9371,7 @@
         <v>9</v>
       </c>
       <c r="E302">
-        <v>0.21</v>
+        <v>0.16</v>
       </c>
       <c r="F302" t="s">
         <v>10</v>
@@ -9391,7 +9391,7 @@
         <v>9</v>
       </c>
       <c r="E303">
-        <v>0.39</v>
+        <v>0.34</v>
       </c>
       <c r="F303" t="s">
         <v>10</v>
@@ -9411,7 +9411,7 @@
         <v>9</v>
       </c>
       <c r="E304">
-        <v>0.34</v>
+        <v>0.17</v>
       </c>
       <c r="F304" t="s">
         <v>10</v>
@@ -9431,7 +9431,7 @@
         <v>9</v>
       </c>
       <c r="E305">
-        <v>0.29</v>
+        <v>0.25</v>
       </c>
       <c r="F305" t="s">
         <v>10</v>
@@ -9451,7 +9451,7 @@
         <v>9</v>
       </c>
       <c r="E306">
-        <v>0.2</v>
+        <v>0.31</v>
       </c>
       <c r="F306" t="s">
         <v>10</v>
@@ -9471,7 +9471,7 @@
         <v>9</v>
       </c>
       <c r="E307">
-        <v>0.26</v>
+        <v>0.29</v>
       </c>
       <c r="F307" t="s">
         <v>10</v>
@@ -9491,7 +9491,7 @@
         <v>9</v>
       </c>
       <c r="E308">
-        <v>0.15</v>
+        <v>0.24</v>
       </c>
       <c r="F308" t="s">
         <v>35</v>
@@ -9511,7 +9511,7 @@
         <v>9</v>
       </c>
       <c r="E309">
-        <v>0.22</v>
+        <v>0.27</v>
       </c>
       <c r="F309" t="s">
         <v>35</v>
@@ -9531,7 +9531,7 @@
         <v>9</v>
       </c>
       <c r="E310">
-        <v>0.14</v>
+        <v>0.28</v>
       </c>
       <c r="F310" t="s">
         <v>35</v>
@@ -9551,7 +9551,7 @@
         <v>9</v>
       </c>
       <c r="E311">
-        <v>0.18</v>
+        <v>0.36</v>
       </c>
       <c r="F311" t="s">
         <v>35</v>
@@ -9571,7 +9571,7 @@
         <v>9</v>
       </c>
       <c r="E312">
-        <v>0.11</v>
+        <v>0.19</v>
       </c>
       <c r="F312" t="s">
         <v>35</v>
@@ -9591,7 +9591,7 @@
         <v>9</v>
       </c>
       <c r="E313">
-        <v>0.16</v>
+        <v>0.18</v>
       </c>
       <c r="F313" t="s">
         <v>35</v>
@@ -9611,7 +9611,7 @@
         <v>9</v>
       </c>
       <c r="E314">
-        <v>0.16</v>
+        <v>0.39</v>
       </c>
       <c r="F314" t="s">
         <v>60</v>
@@ -9631,7 +9631,7 @@
         <v>9</v>
       </c>
       <c r="E315">
-        <v>0.36</v>
+        <v>0.1</v>
       </c>
       <c r="F315" t="s">
         <v>60</v>
@@ -9651,7 +9651,7 @@
         <v>9</v>
       </c>
       <c r="E316">
-        <v>0.34</v>
+        <v>0.17</v>
       </c>
       <c r="F316" t="s">
         <v>60</v>
@@ -9671,7 +9671,7 @@
         <v>9</v>
       </c>
       <c r="E317">
-        <v>0.21</v>
+        <v>0.35</v>
       </c>
       <c r="F317" t="s">
         <v>60</v>
@@ -9691,7 +9691,7 @@
         <v>9</v>
       </c>
       <c r="E318">
-        <v>0.35</v>
+        <v>0.39</v>
       </c>
       <c r="F318" t="s">
         <v>60</v>
@@ -9711,7 +9711,7 @@
         <v>9</v>
       </c>
       <c r="E319">
-        <v>0.35</v>
+        <v>0.15</v>
       </c>
       <c r="F319" t="s">
         <v>60</v>
@@ -9731,7 +9731,7 @@
         <v>9</v>
       </c>
       <c r="E320">
-        <v>0.19</v>
+        <v>0.25</v>
       </c>
       <c r="F320" t="s">
         <v>60</v>
@@ -9751,7 +9751,7 @@
         <v>9</v>
       </c>
       <c r="E321">
-        <v>0.24</v>
+        <v>0.23</v>
       </c>
       <c r="F321" t="s">
         <v>60</v>
@@ -9771,7 +9771,7 @@
         <v>9</v>
       </c>
       <c r="E322">
-        <v>0.15</v>
+        <v>0.14</v>
       </c>
       <c r="F322" t="s">
         <v>10</v>
@@ -9791,7 +9791,7 @@
         <v>9</v>
       </c>
       <c r="E323">
-        <v>0.23</v>
+        <v>0.11</v>
       </c>
       <c r="F323" t="s">
         <v>10</v>
@@ -9811,7 +9811,7 @@
         <v>9</v>
       </c>
       <c r="E324">
-        <v>0.18</v>
+        <v>0.13</v>
       </c>
       <c r="F324" t="s">
         <v>10</v>
@@ -9831,7 +9831,7 @@
         <v>9</v>
       </c>
       <c r="E325">
-        <v>0.26</v>
+        <v>0.22</v>
       </c>
       <c r="F325" t="s">
         <v>10</v>
@@ -9851,7 +9851,7 @@
         <v>9</v>
       </c>
       <c r="E326">
-        <v>0.13</v>
+        <v>0.3</v>
       </c>
       <c r="F326" t="s">
         <v>10</v>
@@ -9871,7 +9871,7 @@
         <v>9</v>
       </c>
       <c r="E327">
-        <v>0.24</v>
+        <v>0.22</v>
       </c>
       <c r="F327" t="s">
         <v>10</v>
@@ -9891,7 +9891,7 @@
         <v>9</v>
       </c>
       <c r="E328">
-        <v>0.35</v>
+        <v>0.23</v>
       </c>
       <c r="F328" t="s">
         <v>35</v>
@@ -9911,7 +9911,7 @@
         <v>9</v>
       </c>
       <c r="E329">
-        <v>0.19</v>
+        <v>0.15</v>
       </c>
       <c r="F329" t="s">
         <v>35</v>
@@ -9931,7 +9931,7 @@
         <v>9</v>
       </c>
       <c r="E330">
-        <v>0.32</v>
+        <v>0.14</v>
       </c>
       <c r="F330" t="s">
         <v>35</v>
@@ -9951,7 +9951,7 @@
         <v>9</v>
       </c>
       <c r="E331">
-        <v>0.29</v>
+        <v>0.15</v>
       </c>
       <c r="F331" t="s">
         <v>35</v>
@@ -9971,7 +9971,7 @@
         <v>9</v>
       </c>
       <c r="E332">
-        <v>0.27</v>
+        <v>0.35</v>
       </c>
       <c r="F332" t="s">
         <v>35</v>
@@ -9991,7 +9991,7 @@
         <v>9</v>
       </c>
       <c r="E333">
-        <v>0.38</v>
+        <v>0.36</v>
       </c>
       <c r="F333" t="s">
         <v>35</v>
@@ -10011,7 +10011,7 @@
         <v>9</v>
       </c>
       <c r="E334">
-        <v>0.26</v>
+        <v>0.32</v>
       </c>
       <c r="F334" t="s">
         <v>60</v>
@@ -10031,7 +10031,7 @@
         <v>9</v>
       </c>
       <c r="E335">
-        <v>0.39</v>
+        <v>0.37</v>
       </c>
       <c r="F335" t="s">
         <v>60</v>
@@ -10051,7 +10051,7 @@
         <v>9</v>
       </c>
       <c r="E336">
-        <v>0.37</v>
+        <v>0.22</v>
       </c>
       <c r="F336" t="s">
         <v>60</v>
@@ -10071,7 +10071,7 @@
         <v>9</v>
       </c>
       <c r="E337">
-        <v>0.33</v>
+        <v>0.28</v>
       </c>
       <c r="F337" t="s">
         <v>60</v>
@@ -10091,7 +10091,7 @@
         <v>9</v>
       </c>
       <c r="E338">
-        <v>0.35</v>
+        <v>0.26</v>
       </c>
       <c r="F338" t="s">
         <v>60</v>
@@ -10131,7 +10131,7 @@
         <v>9</v>
       </c>
       <c r="E340">
-        <v>0.28</v>
+        <v>0.27</v>
       </c>
       <c r="F340" t="s">
         <v>60</v>
@@ -10151,7 +10151,7 @@
         <v>9</v>
       </c>
       <c r="E341">
-        <v>0.29</v>
+        <v>0.23</v>
       </c>
       <c r="F341" t="s">
         <v>60</v>
@@ -10171,7 +10171,7 @@
         <v>9</v>
       </c>
       <c r="E342">
-        <v>0.25</v>
+        <v>0.22</v>
       </c>
       <c r="F342" t="s">
         <v>10</v>
@@ -10191,7 +10191,7 @@
         <v>9</v>
       </c>
       <c r="E343">
-        <v>0.2</v>
+        <v>0.13</v>
       </c>
       <c r="F343" t="s">
         <v>10</v>
@@ -10211,7 +10211,7 @@
         <v>9</v>
       </c>
       <c r="E344">
-        <v>0.11</v>
+        <v>0.23</v>
       </c>
       <c r="F344" t="s">
         <v>10</v>
@@ -10231,7 +10231,7 @@
         <v>9</v>
       </c>
       <c r="E345">
-        <v>0.22</v>
+        <v>0.29</v>
       </c>
       <c r="F345" t="s">
         <v>10</v>
@@ -10251,7 +10251,7 @@
         <v>9</v>
       </c>
       <c r="E346">
-        <v>0.12</v>
+        <v>0.21</v>
       </c>
       <c r="F346" t="s">
         <v>10</v>
@@ -10271,7 +10271,7 @@
         <v>9</v>
       </c>
       <c r="E347">
-        <v>0.14</v>
+        <v>0.36</v>
       </c>
       <c r="F347" t="s">
         <v>10</v>
@@ -10291,7 +10291,7 @@
         <v>9</v>
       </c>
       <c r="E348">
-        <v>0.36</v>
+        <v>0.27</v>
       </c>
       <c r="F348" t="s">
         <v>35</v>
@@ -10311,7 +10311,7 @@
         <v>9</v>
       </c>
       <c r="E349">
-        <v>0.26</v>
+        <v>0.16</v>
       </c>
       <c r="F349" t="s">
         <v>35</v>
@@ -10331,7 +10331,7 @@
         <v>9</v>
       </c>
       <c r="E350">
-        <v>0.16</v>
+        <v>0.31</v>
       </c>
       <c r="F350" t="s">
         <v>35</v>
@@ -10351,7 +10351,7 @@
         <v>9</v>
       </c>
       <c r="E351">
-        <v>0.4</v>
+        <v>0.17</v>
       </c>
       <c r="F351" t="s">
         <v>35</v>
@@ -10371,7 +10371,7 @@
         <v>9</v>
       </c>
       <c r="E352">
-        <v>0.37</v>
+        <v>0.39</v>
       </c>
       <c r="F352" t="s">
         <v>35</v>
@@ -10391,7 +10391,7 @@
         <v>9</v>
       </c>
       <c r="E353">
-        <v>0.23</v>
+        <v>0.13</v>
       </c>
       <c r="F353" t="s">
         <v>35</v>
@@ -10411,7 +10411,7 @@
         <v>9</v>
       </c>
       <c r="E354">
-        <v>0.17</v>
+        <v>0.18</v>
       </c>
       <c r="F354" t="s">
         <v>60</v>
@@ -10431,7 +10431,7 @@
         <v>9</v>
       </c>
       <c r="E355">
-        <v>0.21</v>
+        <v>0.37</v>
       </c>
       <c r="F355" t="s">
         <v>60</v>
@@ -10451,7 +10451,7 @@
         <v>9</v>
       </c>
       <c r="E356">
-        <v>0.37</v>
+        <v>0.33</v>
       </c>
       <c r="F356" t="s">
         <v>60</v>
@@ -10471,7 +10471,7 @@
         <v>9</v>
       </c>
       <c r="E357">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="F357" t="s">
         <v>60</v>
@@ -10491,7 +10491,7 @@
         <v>9</v>
       </c>
       <c r="E358">
-        <v>0.4</v>
+        <v>0.15</v>
       </c>
       <c r="F358" t="s">
         <v>60</v>
@@ -10511,7 +10511,7 @@
         <v>9</v>
       </c>
       <c r="E359">
-        <v>0.26</v>
+        <v>0.16</v>
       </c>
       <c r="F359" t="s">
         <v>60</v>
@@ -10531,7 +10531,7 @@
         <v>9</v>
       </c>
       <c r="E360">
-        <v>0.3</v>
+        <v>0.11</v>
       </c>
       <c r="F360" t="s">
         <v>60</v>
@@ -10551,7 +10551,7 @@
         <v>9</v>
       </c>
       <c r="E361">
-        <v>0.14</v>
+        <v>0.12</v>
       </c>
       <c r="F361" t="s">
         <v>60</v>
@@ -10571,7 +10571,7 @@
         <v>9</v>
       </c>
       <c r="E362">
-        <v>0.35</v>
+        <v>0.38</v>
       </c>
       <c r="F362" t="s">
         <v>10</v>
@@ -10591,7 +10591,7 @@
         <v>9</v>
       </c>
       <c r="E363">
-        <v>0.14</v>
+        <v>0.33</v>
       </c>
       <c r="F363" t="s">
         <v>10</v>
@@ -10611,7 +10611,7 @@
         <v>9</v>
       </c>
       <c r="E364">
-        <v>0.15</v>
+        <v>0.31</v>
       </c>
       <c r="F364" t="s">
         <v>10</v>
@@ -10631,7 +10631,7 @@
         <v>9</v>
       </c>
       <c r="E365">
-        <v>0.22</v>
+        <v>0.21</v>
       </c>
       <c r="F365" t="s">
         <v>10</v>
@@ -10651,7 +10651,7 @@
         <v>9</v>
       </c>
       <c r="E366">
-        <v>0.38</v>
+        <v>0.17</v>
       </c>
       <c r="F366" t="s">
         <v>10</v>
@@ -10671,7 +10671,7 @@
         <v>9</v>
       </c>
       <c r="E367">
-        <v>0.14</v>
+        <v>0.4</v>
       </c>
       <c r="F367" t="s">
         <v>10</v>
@@ -10691,7 +10691,7 @@
         <v>9</v>
       </c>
       <c r="E368">
-        <v>0.31</v>
+        <v>0.3</v>
       </c>
       <c r="F368" t="s">
         <v>35</v>
@@ -10711,7 +10711,7 @@
         <v>9</v>
       </c>
       <c r="E369">
-        <v>0.2</v>
+        <v>0.25</v>
       </c>
       <c r="F369" t="s">
         <v>35</v>
@@ -10731,7 +10731,7 @@
         <v>9</v>
       </c>
       <c r="E370">
-        <v>0.37</v>
+        <v>0.33</v>
       </c>
       <c r="F370" t="s">
         <v>35</v>
@@ -10751,7 +10751,7 @@
         <v>9</v>
       </c>
       <c r="E371">
-        <v>0.11</v>
+        <v>0.39</v>
       </c>
       <c r="F371" t="s">
         <v>35</v>
@@ -10771,7 +10771,7 @@
         <v>9</v>
       </c>
       <c r="E372">
-        <v>0.35</v>
+        <v>0.11</v>
       </c>
       <c r="F372" t="s">
         <v>35</v>
@@ -10791,7 +10791,7 @@
         <v>9</v>
       </c>
       <c r="E373">
-        <v>0.33</v>
+        <v>0.27</v>
       </c>
       <c r="F373" t="s">
         <v>35</v>
@@ -10811,7 +10811,7 @@
         <v>9</v>
       </c>
       <c r="E374">
-        <v>0.26</v>
+        <v>0.11</v>
       </c>
       <c r="F374" t="s">
         <v>60</v>
@@ -10831,7 +10831,7 @@
         <v>9</v>
       </c>
       <c r="E375">
-        <v>0.12</v>
+        <v>0.28</v>
       </c>
       <c r="F375" t="s">
         <v>60</v>
@@ -10851,7 +10851,7 @@
         <v>9</v>
       </c>
       <c r="E376">
-        <v>0.31</v>
+        <v>0.23</v>
       </c>
       <c r="F376" t="s">
         <v>60</v>
@@ -10871,7 +10871,7 @@
         <v>9</v>
       </c>
       <c r="E377">
-        <v>0.21</v>
+        <v>0.13</v>
       </c>
       <c r="F377" t="s">
         <v>60</v>
@@ -10891,7 +10891,7 @@
         <v>9</v>
       </c>
       <c r="E378">
-        <v>0.19</v>
+        <v>0.13</v>
       </c>
       <c r="F378" t="s">
         <v>60</v>
@@ -10911,7 +10911,7 @@
         <v>9</v>
       </c>
       <c r="E379">
-        <v>0.32</v>
+        <v>0.34</v>
       </c>
       <c r="F379" t="s">
         <v>60</v>
@@ -10931,7 +10931,7 @@
         <v>9</v>
       </c>
       <c r="E380">
-        <v>0.23</v>
+        <v>0.38</v>
       </c>
       <c r="F380" t="s">
         <v>60</v>
@@ -10951,7 +10951,7 @@
         <v>9</v>
       </c>
       <c r="E381">
-        <v>0.32</v>
+        <v>0.27</v>
       </c>
       <c r="F381" t="s">
         <v>60</v>
@@ -10971,7 +10971,7 @@
         <v>9</v>
       </c>
       <c r="E382">
-        <v>0.13</v>
+        <v>0.24</v>
       </c>
       <c r="F382" t="s">
         <v>10</v>
@@ -10991,7 +10991,7 @@
         <v>9</v>
       </c>
       <c r="E383">
-        <v>0.18</v>
+        <v>0.15</v>
       </c>
       <c r="F383" t="s">
         <v>10</v>
@@ -11011,7 +11011,7 @@
         <v>9</v>
       </c>
       <c r="E384">
-        <v>0.19</v>
+        <v>0.37</v>
       </c>
       <c r="F384" t="s">
         <v>10</v>
@@ -11031,7 +11031,7 @@
         <v>9</v>
       </c>
       <c r="E385">
-        <v>0.28</v>
+        <v>0.23</v>
       </c>
       <c r="F385" t="s">
         <v>10</v>
@@ -11051,7 +11051,7 @@
         <v>9</v>
       </c>
       <c r="E386">
-        <v>0.33</v>
+        <v>0.19</v>
       </c>
       <c r="F386" t="s">
         <v>10</v>
@@ -11071,7 +11071,7 @@
         <v>9</v>
       </c>
       <c r="E387">
-        <v>0.12</v>
+        <v>0.3</v>
       </c>
       <c r="F387" t="s">
         <v>10</v>
@@ -11091,7 +11091,7 @@
         <v>9</v>
       </c>
       <c r="E388">
-        <v>0.11</v>
+        <v>0.37</v>
       </c>
       <c r="F388" t="s">
         <v>35</v>
@@ -11111,7 +11111,7 @@
         <v>9</v>
       </c>
       <c r="E389">
-        <v>0.39</v>
+        <v>0.23</v>
       </c>
       <c r="F389" t="s">
         <v>35</v>
@@ -11131,7 +11131,7 @@
         <v>9</v>
       </c>
       <c r="E390">
-        <v>0.24</v>
+        <v>0.3</v>
       </c>
       <c r="F390" t="s">
         <v>35</v>
@@ -11171,7 +11171,7 @@
         <v>9</v>
       </c>
       <c r="E392">
-        <v>0.35</v>
+        <v>0.25</v>
       </c>
       <c r="F392" t="s">
         <v>35</v>
@@ -11191,7 +11191,7 @@
         <v>9</v>
       </c>
       <c r="E393">
-        <v>0.16</v>
+        <v>0.3</v>
       </c>
       <c r="F393" t="s">
         <v>35</v>
@@ -11211,7 +11211,7 @@
         <v>9</v>
       </c>
       <c r="E394">
-        <v>0.21</v>
+        <v>0.15</v>
       </c>
       <c r="F394" t="s">
         <v>60</v>
@@ -11231,7 +11231,7 @@
         <v>9</v>
       </c>
       <c r="E395">
-        <v>0.33</v>
+        <v>0.13</v>
       </c>
       <c r="F395" t="s">
         <v>60</v>
@@ -11251,7 +11251,7 @@
         <v>9</v>
       </c>
       <c r="E396">
-        <v>0.32</v>
+        <v>0.35</v>
       </c>
       <c r="F396" t="s">
         <v>60</v>
@@ -11271,7 +11271,7 @@
         <v>9</v>
       </c>
       <c r="E397">
-        <v>0.28</v>
+        <v>0.21</v>
       </c>
       <c r="F397" t="s">
         <v>60</v>
@@ -11291,7 +11291,7 @@
         <v>9</v>
       </c>
       <c r="E398">
-        <v>0.27</v>
+        <v>0.38</v>
       </c>
       <c r="F398" t="s">
         <v>60</v>
@@ -11311,7 +11311,7 @@
         <v>9</v>
       </c>
       <c r="E399">
-        <v>0.39</v>
+        <v>0.17</v>
       </c>
       <c r="F399" t="s">
         <v>60</v>
@@ -11331,7 +11331,7 @@
         <v>9</v>
       </c>
       <c r="E400">
-        <v>0.36</v>
+        <v>0.28</v>
       </c>
       <c r="F400" t="s">
         <v>60</v>
@@ -11351,7 +11351,7 @@
         <v>9</v>
       </c>
       <c r="E401">
-        <v>0.17</v>
+        <v>0.16</v>
       </c>
       <c r="F401" t="s">
         <v>60</v>
@@ -11371,7 +11371,7 @@
         <v>9</v>
       </c>
       <c r="E402">
-        <v>0.39</v>
+        <v>0.4</v>
       </c>
       <c r="F402" t="s">
         <v>10</v>
@@ -11391,7 +11391,7 @@
         <v>9</v>
       </c>
       <c r="E403">
-        <v>0.25</v>
+        <v>0.26</v>
       </c>
       <c r="F403" t="s">
         <v>10</v>
@@ -11411,7 +11411,7 @@
         <v>9</v>
       </c>
       <c r="E404">
-        <v>0.14</v>
+        <v>0.18</v>
       </c>
       <c r="F404" t="s">
         <v>10</v>
@@ -11431,7 +11431,7 @@
         <v>9</v>
       </c>
       <c r="E405">
-        <v>0.23</v>
+        <v>0.3</v>
       </c>
       <c r="F405" t="s">
         <v>10</v>
@@ -11451,7 +11451,7 @@
         <v>9</v>
       </c>
       <c r="E406">
-        <v>0.1</v>
+        <v>0.37</v>
       </c>
       <c r="F406" t="s">
         <v>10</v>
@@ -11471,7 +11471,7 @@
         <v>9</v>
       </c>
       <c r="E407">
-        <v>0.13</v>
+        <v>0.19</v>
       </c>
       <c r="F407" t="s">
         <v>10</v>
@@ -11491,7 +11491,7 @@
         <v>9</v>
       </c>
       <c r="E408">
-        <v>0.27</v>
+        <v>0.35</v>
       </c>
       <c r="F408" t="s">
         <v>35</v>
@@ -11511,7 +11511,7 @@
         <v>9</v>
       </c>
       <c r="E409">
-        <v>0.14</v>
+        <v>0.34</v>
       </c>
       <c r="F409" t="s">
         <v>35</v>
@@ -11531,7 +11531,7 @@
         <v>9</v>
       </c>
       <c r="E410">
-        <v>0.2</v>
+        <v>0.15</v>
       </c>
       <c r="F410" t="s">
         <v>35</v>
@@ -11551,7 +11551,7 @@
         <v>9</v>
       </c>
       <c r="E411">
-        <v>0.15</v>
+        <v>0.11</v>
       </c>
       <c r="F411" t="s">
         <v>35</v>
@@ -11571,7 +11571,7 @@
         <v>9</v>
       </c>
       <c r="E412">
-        <v>0.36</v>
+        <v>0.28</v>
       </c>
       <c r="F412" t="s">
         <v>35</v>
@@ -11591,7 +11591,7 @@
         <v>9</v>
       </c>
       <c r="E413">
-        <v>0.37</v>
+        <v>0.31</v>
       </c>
       <c r="F413" t="s">
         <v>35</v>
@@ -11611,7 +11611,7 @@
         <v>9</v>
       </c>
       <c r="E414">
-        <v>0.23</v>
+        <v>0.35</v>
       </c>
       <c r="F414" t="s">
         <v>60</v>
@@ -11631,7 +11631,7 @@
         <v>9</v>
       </c>
       <c r="E415">
-        <v>0.4</v>
+        <v>0.23</v>
       </c>
       <c r="F415" t="s">
         <v>60</v>
@@ -11651,7 +11651,7 @@
         <v>9</v>
       </c>
       <c r="E416">
-        <v>0.4</v>
+        <v>0.11</v>
       </c>
       <c r="F416" t="s">
         <v>60</v>
@@ -11671,7 +11671,7 @@
         <v>9</v>
       </c>
       <c r="E417">
-        <v>0.27</v>
+        <v>0.2</v>
       </c>
       <c r="F417" t="s">
         <v>60</v>
@@ -11691,7 +11691,7 @@
         <v>9</v>
       </c>
       <c r="E418">
-        <v>0.4</v>
+        <v>0.27</v>
       </c>
       <c r="F418" t="s">
         <v>60</v>
@@ -11711,7 +11711,7 @@
         <v>9</v>
       </c>
       <c r="E419">
-        <v>0.23</v>
+        <v>0.1</v>
       </c>
       <c r="F419" t="s">
         <v>60</v>
@@ -11731,7 +11731,7 @@
         <v>9</v>
       </c>
       <c r="E420">
-        <v>0.37</v>
+        <v>0.27</v>
       </c>
       <c r="F420" t="s">
         <v>60</v>
@@ -11771,7 +11771,7 @@
         <v>9</v>
       </c>
       <c r="E422">
-        <v>0.23</v>
+        <v>0.31</v>
       </c>
       <c r="F422" t="s">
         <v>10</v>
@@ -11791,7 +11791,7 @@
         <v>9</v>
       </c>
       <c r="E423">
-        <v>0.16</v>
+        <v>0.11</v>
       </c>
       <c r="F423" t="s">
         <v>10</v>
@@ -11811,7 +11811,7 @@
         <v>9</v>
       </c>
       <c r="E424">
-        <v>0.12</v>
+        <v>0.32</v>
       </c>
       <c r="F424" t="s">
         <v>10</v>
@@ -11851,7 +11851,7 @@
         <v>9</v>
       </c>
       <c r="E426">
-        <v>0.27</v>
+        <v>0.35</v>
       </c>
       <c r="F426" t="s">
         <v>10</v>
@@ -11871,7 +11871,7 @@
         <v>9</v>
       </c>
       <c r="E427">
-        <v>0.34</v>
+        <v>0.23</v>
       </c>
       <c r="F427" t="s">
         <v>10</v>
@@ -11891,7 +11891,7 @@
         <v>9</v>
       </c>
       <c r="E428">
-        <v>0.3</v>
+        <v>0.35</v>
       </c>
       <c r="F428" t="s">
         <v>10</v>
@@ -11911,7 +11911,7 @@
         <v>9</v>
       </c>
       <c r="E429">
-        <v>0.39</v>
+        <v>0.34</v>
       </c>
       <c r="F429" t="s">
         <v>10</v>
@@ -11931,7 +11931,7 @@
         <v>9</v>
       </c>
       <c r="E430">
-        <v>0.1</v>
+        <v>0.38</v>
       </c>
       <c r="F430" t="s">
         <v>10</v>
@@ -11951,7 +11951,7 @@
         <v>9</v>
       </c>
       <c r="E431">
-        <v>0.31</v>
+        <v>0.38</v>
       </c>
       <c r="F431" t="s">
         <v>10</v>
@@ -11971,7 +11971,7 @@
         <v>9</v>
       </c>
       <c r="E432">
-        <v>0.26</v>
+        <v>0.33</v>
       </c>
       <c r="F432" t="s">
         <v>10</v>
@@ -11991,7 +11991,7 @@
         <v>9</v>
       </c>
       <c r="E433">
-        <v>0.36</v>
+        <v>0.35</v>
       </c>
       <c r="F433" t="s">
         <v>10</v>
@@ -12011,7 +12011,7 @@
         <v>9</v>
       </c>
       <c r="E434">
-        <v>0.19</v>
+        <v>0.18</v>
       </c>
       <c r="F434" t="s">
         <v>10</v>
@@ -12031,7 +12031,7 @@
         <v>9</v>
       </c>
       <c r="E435">
-        <v>0.21</v>
+        <v>0.37</v>
       </c>
       <c r="F435" t="s">
         <v>10</v>
@@ -12051,7 +12051,7 @@
         <v>9</v>
       </c>
       <c r="E436">
-        <v>0.37</v>
+        <v>0.36</v>
       </c>
       <c r="F436" t="s">
         <v>10</v>
@@ -12071,7 +12071,7 @@
         <v>9</v>
       </c>
       <c r="E437">
-        <v>0.13</v>
+        <v>0.3</v>
       </c>
       <c r="F437" t="s">
         <v>35</v>
@@ -12091,7 +12091,7 @@
         <v>9</v>
       </c>
       <c r="E438">
-        <v>0.24</v>
+        <v>0.33</v>
       </c>
       <c r="F438" t="s">
         <v>35</v>
@@ -12111,7 +12111,7 @@
         <v>9</v>
       </c>
       <c r="E439">
-        <v>0.38</v>
+        <v>0.26</v>
       </c>
       <c r="F439" t="s">
         <v>35</v>
@@ -12131,7 +12131,7 @@
         <v>9</v>
       </c>
       <c r="E440">
-        <v>0.25</v>
+        <v>0.37</v>
       </c>
       <c r="F440" t="s">
         <v>35</v>
@@ -12151,7 +12151,7 @@
         <v>9</v>
       </c>
       <c r="E441">
-        <v>0.37</v>
+        <v>0.39</v>
       </c>
       <c r="F441" t="s">
         <v>35</v>
@@ -12171,7 +12171,7 @@
         <v>9</v>
       </c>
       <c r="E442">
-        <v>0.2</v>
+        <v>0.31</v>
       </c>
       <c r="F442" t="s">
         <v>35</v>
@@ -12191,7 +12191,7 @@
         <v>9</v>
       </c>
       <c r="E443">
-        <v>0.24</v>
+        <v>0.29</v>
       </c>
       <c r="F443" t="s">
         <v>35</v>
@@ -12211,7 +12211,7 @@
         <v>9</v>
       </c>
       <c r="E444">
-        <v>0.28</v>
+        <v>0.21</v>
       </c>
       <c r="F444" t="s">
         <v>35</v>
@@ -12231,7 +12231,7 @@
         <v>9</v>
       </c>
       <c r="E445">
-        <v>0.37</v>
+        <v>0.21</v>
       </c>
       <c r="F445" t="s">
         <v>35</v>
@@ -12251,7 +12251,7 @@
         <v>9</v>
       </c>
       <c r="E446">
-        <v>0.22</v>
+        <v>0.11</v>
       </c>
       <c r="F446" t="s">
         <v>35</v>
@@ -12271,7 +12271,7 @@
         <v>9</v>
       </c>
       <c r="E447">
-        <v>0.38</v>
+        <v>0.21</v>
       </c>
       <c r="F447" t="s">
         <v>35</v>
@@ -12291,7 +12291,7 @@
         <v>9</v>
       </c>
       <c r="E448">
-        <v>0.35</v>
+        <v>0.38</v>
       </c>
       <c r="F448" t="s">
         <v>35</v>
@@ -12311,7 +12311,7 @@
         <v>9</v>
       </c>
       <c r="E449">
-        <v>0.14</v>
+        <v>0.18</v>
       </c>
       <c r="F449" t="s">
         <v>35</v>
@@ -12331,7 +12331,7 @@
         <v>9</v>
       </c>
       <c r="E450">
-        <v>0.3</v>
+        <v>0.22</v>
       </c>
       <c r="F450" t="s">
         <v>35</v>
@@ -12351,7 +12351,7 @@
         <v>9</v>
       </c>
       <c r="E451">
-        <v>0.25</v>
+        <v>0.22</v>
       </c>
       <c r="F451" t="s">
         <v>35</v>
@@ -12371,7 +12371,7 @@
         <v>9</v>
       </c>
       <c r="E452">
-        <v>0.11</v>
+        <v>0.17</v>
       </c>
       <c r="F452" t="s">
         <v>60</v>
@@ -12391,7 +12391,7 @@
         <v>9</v>
       </c>
       <c r="E453">
-        <v>0.16</v>
+        <v>0.36</v>
       </c>
       <c r="F453" t="s">
         <v>60</v>
@@ -12411,7 +12411,7 @@
         <v>9</v>
       </c>
       <c r="E454">
-        <v>0.25</v>
+        <v>0.12</v>
       </c>
       <c r="F454" t="s">
         <v>60</v>
@@ -12451,7 +12451,7 @@
         <v>9</v>
       </c>
       <c r="E456">
-        <v>0.39</v>
+        <v>0.25</v>
       </c>
       <c r="F456" t="s">
         <v>60</v>
@@ -12471,7 +12471,7 @@
         <v>9</v>
       </c>
       <c r="E457">
-        <v>0.32</v>
+        <v>0.35</v>
       </c>
       <c r="F457" t="s">
         <v>60</v>
@@ -12491,7 +12491,7 @@
         <v>9</v>
       </c>
       <c r="E458">
-        <v>0.16</v>
+        <v>0.22</v>
       </c>
       <c r="F458" t="s">
         <v>60</v>
@@ -12511,7 +12511,7 @@
         <v>9</v>
       </c>
       <c r="E459">
-        <v>0.23</v>
+        <v>0.3</v>
       </c>
       <c r="F459" t="s">
         <v>60</v>
@@ -12531,7 +12531,7 @@
         <v>9</v>
       </c>
       <c r="E460">
-        <v>0.32</v>
+        <v>0.2</v>
       </c>
       <c r="F460" t="s">
         <v>60</v>
@@ -12551,7 +12551,7 @@
         <v>9</v>
       </c>
       <c r="E461">
-        <v>0.24</v>
+        <v>0.19</v>
       </c>
       <c r="F461" t="s">
         <v>60</v>
@@ -12571,7 +12571,7 @@
         <v>9</v>
       </c>
       <c r="E462">
-        <v>0.25</v>
+        <v>0.18</v>
       </c>
       <c r="F462" t="s">
         <v>60</v>
@@ -12591,7 +12591,7 @@
         <v>9</v>
       </c>
       <c r="E463">
-        <v>0.3</v>
+        <v>0.11</v>
       </c>
       <c r="F463" t="s">
         <v>60</v>
@@ -12611,7 +12611,7 @@
         <v>9</v>
       </c>
       <c r="E464">
-        <v>0.3</v>
+        <v>0.27</v>
       </c>
       <c r="F464" t="s">
         <v>60</v>
@@ -12631,7 +12631,7 @@
         <v>9</v>
       </c>
       <c r="E465">
-        <v>0.38</v>
+        <v>0.14</v>
       </c>
       <c r="F465" t="s">
         <v>60</v>
@@ -12651,7 +12651,7 @@
         <v>9</v>
       </c>
       <c r="E466">
-        <v>0.28</v>
+        <v>0.2</v>
       </c>
       <c r="F466" t="s">
         <v>60</v>
@@ -12671,7 +12671,7 @@
         <v>9</v>
       </c>
       <c r="E467">
-        <v>0.27</v>
+        <v>0.26</v>
       </c>
       <c r="F467" t="s">
         <v>60</v>
@@ -12691,7 +12691,7 @@
         <v>9</v>
       </c>
       <c r="E468">
-        <v>0.27</v>
+        <v>0.29</v>
       </c>
       <c r="F468" t="s">
         <v>60</v>
@@ -12711,7 +12711,7 @@
         <v>9</v>
       </c>
       <c r="E469">
-        <v>0.25</v>
+        <v>0.22</v>
       </c>
       <c r="F469" t="s">
         <v>60</v>
@@ -12731,7 +12731,7 @@
         <v>9</v>
       </c>
       <c r="E470">
-        <v>0.25</v>
+        <v>0.36</v>
       </c>
       <c r="F470" t="s">
         <v>60</v>
@@ -12751,7 +12751,7 @@
         <v>9</v>
       </c>
       <c r="E471">
-        <v>0.2</v>
+        <v>0.37</v>
       </c>
       <c r="F471" t="s">
         <v>60</v>

</xml_diff>

<commit_message>
Fix ExcelJS column definition for 100% compatibility with Excel Online and Microsoft Excel
</commit_message>
<xml_diff>
--- a/Test Results/Excel/Automation_Test_Report.xlsx
+++ b/Test Results/Excel/Automation_Test_Report.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4259" uniqueCount="973">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4271" uniqueCount="980">
   <si>
     <t>Test ID</t>
   </si>
@@ -2910,6 +2910,21 @@
     <t>Verify Regression live web deployment scenario #50</t>
   </si>
   <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>All Modules</t>
+  </si>
+  <si>
+    <t>No Failed Test Cases Found - 100% Pass Rate</t>
+  </si>
+  <si>
+    <t>NONE</t>
+  </si>
+  <si>
+    <t>No Skipped Tests Found</t>
+  </si>
+  <si>
     <t>Metric</t>
   </si>
   <si>
@@ -2935,6 +2950,12 @@
   </si>
   <si>
     <t>Failure Reason</t>
+  </si>
+  <si>
+    <t>DEF-NONE</t>
+  </si>
+  <si>
+    <t>No Defects Found - 100% Pass Rate</t>
   </si>
 </sst>
 </file>
@@ -2958,7 +2979,7 @@
       <color rgb="15803D"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2975,6 +2996,26 @@
         <fgColor rgb="DCFCE7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="15803D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="B91C1C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="475569"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="1E3A8A"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -2988,10 +3029,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3334,7 +3379,12 @@
   <dimension ref="A1:F471"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="6" width="25" customWidth="1"/>
+    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="2" max="2" width="25" customWidth="1"/>
+    <col min="3" max="3" width="45" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="5" width="22" customWidth="1"/>
+    <col min="6" max="6" width="15" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -3371,7 +3421,7 @@
         <v>9</v>
       </c>
       <c r="E2">
-        <v>0.26</v>
+        <v>0.39</v>
       </c>
       <c r="F2" t="s">
         <v>10</v>
@@ -3391,7 +3441,7 @@
         <v>9</v>
       </c>
       <c r="E3">
-        <v>0.26</v>
+        <v>0.28</v>
       </c>
       <c r="F3" t="s">
         <v>10</v>
@@ -3411,7 +3461,7 @@
         <v>9</v>
       </c>
       <c r="E4">
-        <v>0.11</v>
+        <v>0.38</v>
       </c>
       <c r="F4" t="s">
         <v>10</v>
@@ -3431,7 +3481,7 @@
         <v>9</v>
       </c>
       <c r="E5">
-        <v>0.15</v>
+        <v>0.14</v>
       </c>
       <c r="F5" t="s">
         <v>10</v>
@@ -3451,7 +3501,7 @@
         <v>9</v>
       </c>
       <c r="E6">
-        <v>0.37</v>
+        <v>0.36</v>
       </c>
       <c r="F6" t="s">
         <v>10</v>
@@ -3471,7 +3521,7 @@
         <v>9</v>
       </c>
       <c r="E7">
-        <v>0.33</v>
+        <v>0.11</v>
       </c>
       <c r="F7" t="s">
         <v>10</v>
@@ -3491,7 +3541,7 @@
         <v>9</v>
       </c>
       <c r="E8">
-        <v>0.2</v>
+        <v>0.31</v>
       </c>
       <c r="F8" t="s">
         <v>10</v>
@@ -3511,7 +3561,7 @@
         <v>9</v>
       </c>
       <c r="E9">
-        <v>0.39</v>
+        <v>0.12</v>
       </c>
       <c r="F9" t="s">
         <v>10</v>
@@ -3531,7 +3581,7 @@
         <v>9</v>
       </c>
       <c r="E10">
-        <v>0.31</v>
+        <v>0.4</v>
       </c>
       <c r="F10" t="s">
         <v>10</v>
@@ -3551,7 +3601,7 @@
         <v>9</v>
       </c>
       <c r="E11">
-        <v>0.34</v>
+        <v>0.3</v>
       </c>
       <c r="F11" t="s">
         <v>10</v>
@@ -3571,7 +3621,7 @@
         <v>9</v>
       </c>
       <c r="E12">
-        <v>0.31</v>
+        <v>0.14</v>
       </c>
       <c r="F12" t="s">
         <v>10</v>
@@ -3591,7 +3641,7 @@
         <v>9</v>
       </c>
       <c r="E13">
-        <v>0.31</v>
+        <v>0.32</v>
       </c>
       <c r="F13" t="s">
         <v>10</v>
@@ -3611,7 +3661,7 @@
         <v>9</v>
       </c>
       <c r="E14">
-        <v>0.33</v>
+        <v>0.28</v>
       </c>
       <c r="F14" t="s">
         <v>35</v>
@@ -3631,7 +3681,7 @@
         <v>9</v>
       </c>
       <c r="E15">
-        <v>0.24</v>
+        <v>0.32</v>
       </c>
       <c r="F15" t="s">
         <v>35</v>
@@ -3651,7 +3701,7 @@
         <v>9</v>
       </c>
       <c r="E16">
-        <v>0.32</v>
+        <v>0.12</v>
       </c>
       <c r="F16" t="s">
         <v>35</v>
@@ -3671,7 +3721,7 @@
         <v>9</v>
       </c>
       <c r="E17">
-        <v>0.38</v>
+        <v>0.36</v>
       </c>
       <c r="F17" t="s">
         <v>35</v>
@@ -3691,7 +3741,7 @@
         <v>9</v>
       </c>
       <c r="E18">
-        <v>0.1</v>
+        <v>0.37</v>
       </c>
       <c r="F18" t="s">
         <v>35</v>
@@ -3711,7 +3761,7 @@
         <v>9</v>
       </c>
       <c r="E19">
-        <v>0.31</v>
+        <v>0.17</v>
       </c>
       <c r="F19" t="s">
         <v>35</v>
@@ -3731,7 +3781,7 @@
         <v>9</v>
       </c>
       <c r="E20">
-        <v>0.15</v>
+        <v>0.27</v>
       </c>
       <c r="F20" t="s">
         <v>35</v>
@@ -3751,7 +3801,7 @@
         <v>9</v>
       </c>
       <c r="E21">
-        <v>0.15</v>
+        <v>0.35</v>
       </c>
       <c r="F21" t="s">
         <v>35</v>
@@ -3771,7 +3821,7 @@
         <v>9</v>
       </c>
       <c r="E22">
-        <v>0.29</v>
+        <v>0.34</v>
       </c>
       <c r="F22" t="s">
         <v>35</v>
@@ -3791,7 +3841,7 @@
         <v>9</v>
       </c>
       <c r="E23">
-        <v>0.28</v>
+        <v>0.18</v>
       </c>
       <c r="F23" t="s">
         <v>35</v>
@@ -3811,7 +3861,7 @@
         <v>9</v>
       </c>
       <c r="E24">
-        <v>0.17</v>
+        <v>0.39</v>
       </c>
       <c r="F24" t="s">
         <v>35</v>
@@ -3831,7 +3881,7 @@
         <v>9</v>
       </c>
       <c r="E25">
-        <v>0.26</v>
+        <v>0.28</v>
       </c>
       <c r="F25" t="s">
         <v>35</v>
@@ -3851,7 +3901,7 @@
         <v>9</v>
       </c>
       <c r="E26">
-        <v>0.39</v>
+        <v>0.37</v>
       </c>
       <c r="F26" t="s">
         <v>60</v>
@@ -3871,7 +3921,7 @@
         <v>9</v>
       </c>
       <c r="E27">
-        <v>0.11</v>
+        <v>0.23</v>
       </c>
       <c r="F27" t="s">
         <v>60</v>
@@ -3891,7 +3941,7 @@
         <v>9</v>
       </c>
       <c r="E28">
-        <v>0.2</v>
+        <v>0.11</v>
       </c>
       <c r="F28" t="s">
         <v>60</v>
@@ -3911,7 +3961,7 @@
         <v>9</v>
       </c>
       <c r="E29">
-        <v>0.26</v>
+        <v>0.22</v>
       </c>
       <c r="F29" t="s">
         <v>60</v>
@@ -3931,7 +3981,7 @@
         <v>9</v>
       </c>
       <c r="E30">
-        <v>0.17</v>
+        <v>0.25</v>
       </c>
       <c r="F30" t="s">
         <v>60</v>
@@ -3951,7 +4001,7 @@
         <v>9</v>
       </c>
       <c r="E31">
-        <v>0.14</v>
+        <v>0.39</v>
       </c>
       <c r="F31" t="s">
         <v>60</v>
@@ -3971,7 +4021,7 @@
         <v>9</v>
       </c>
       <c r="E32">
-        <v>0.12</v>
+        <v>0.25</v>
       </c>
       <c r="F32" t="s">
         <v>60</v>
@@ -3991,7 +4041,7 @@
         <v>9</v>
       </c>
       <c r="E33">
-        <v>0.27</v>
+        <v>0.3</v>
       </c>
       <c r="F33" t="s">
         <v>60</v>
@@ -4011,7 +4061,7 @@
         <v>9</v>
       </c>
       <c r="E34">
-        <v>0.25</v>
+        <v>0.2</v>
       </c>
       <c r="F34" t="s">
         <v>60</v>
@@ -4031,7 +4081,7 @@
         <v>9</v>
       </c>
       <c r="E35">
-        <v>0.22</v>
+        <v>0.31</v>
       </c>
       <c r="F35" t="s">
         <v>60</v>
@@ -4051,7 +4101,7 @@
         <v>9</v>
       </c>
       <c r="E36">
-        <v>0.39</v>
+        <v>0.38</v>
       </c>
       <c r="F36" t="s">
         <v>60</v>
@@ -4071,7 +4121,7 @@
         <v>9</v>
       </c>
       <c r="E37">
-        <v>0.2</v>
+        <v>0.24</v>
       </c>
       <c r="F37" t="s">
         <v>60</v>
@@ -4111,7 +4161,7 @@
         <v>9</v>
       </c>
       <c r="E39">
-        <v>0.19</v>
+        <v>0.1</v>
       </c>
       <c r="F39" t="s">
         <v>60</v>
@@ -4131,7 +4181,7 @@
         <v>9</v>
       </c>
       <c r="E40">
-        <v>0.3</v>
+        <v>0.14</v>
       </c>
       <c r="F40" t="s">
         <v>60</v>
@@ -4151,7 +4201,7 @@
         <v>9</v>
       </c>
       <c r="E41">
-        <v>0.14</v>
+        <v>0.17</v>
       </c>
       <c r="F41" t="s">
         <v>60</v>
@@ -4171,7 +4221,7 @@
         <v>9</v>
       </c>
       <c r="E42">
-        <v>0.21</v>
+        <v>0.25</v>
       </c>
       <c r="F42" t="s">
         <v>10</v>
@@ -4191,7 +4241,7 @@
         <v>9</v>
       </c>
       <c r="E43">
-        <v>0.18</v>
+        <v>0.28</v>
       </c>
       <c r="F43" t="s">
         <v>10</v>
@@ -4211,7 +4261,7 @@
         <v>9</v>
       </c>
       <c r="E44">
-        <v>0.18</v>
+        <v>0.2</v>
       </c>
       <c r="F44" t="s">
         <v>10</v>
@@ -4231,7 +4281,7 @@
         <v>9</v>
       </c>
       <c r="E45">
-        <v>0.26</v>
+        <v>0.39</v>
       </c>
       <c r="F45" t="s">
         <v>10</v>
@@ -4251,7 +4301,7 @@
         <v>9</v>
       </c>
       <c r="E46">
-        <v>0.23</v>
+        <v>0.39</v>
       </c>
       <c r="F46" t="s">
         <v>10</v>
@@ -4271,7 +4321,7 @@
         <v>9</v>
       </c>
       <c r="E47">
-        <v>0.16</v>
+        <v>0.2</v>
       </c>
       <c r="F47" t="s">
         <v>10</v>
@@ -4291,7 +4341,7 @@
         <v>9</v>
       </c>
       <c r="E48">
-        <v>0.31</v>
+        <v>0.23</v>
       </c>
       <c r="F48" t="s">
         <v>10</v>
@@ -4311,7 +4361,7 @@
         <v>9</v>
       </c>
       <c r="E49">
-        <v>0.2</v>
+        <v>0.23</v>
       </c>
       <c r="F49" t="s">
         <v>10</v>
@@ -4331,7 +4381,7 @@
         <v>9</v>
       </c>
       <c r="E50">
-        <v>0.16</v>
+        <v>0.18</v>
       </c>
       <c r="F50" t="s">
         <v>10</v>
@@ -4351,7 +4401,7 @@
         <v>9</v>
       </c>
       <c r="E51">
-        <v>0.33</v>
+        <v>0.16</v>
       </c>
       <c r="F51" t="s">
         <v>10</v>
@@ -4371,7 +4421,7 @@
         <v>9</v>
       </c>
       <c r="E52">
-        <v>0.16</v>
+        <v>0.37</v>
       </c>
       <c r="F52" t="s">
         <v>10</v>
@@ -4391,7 +4441,7 @@
         <v>9</v>
       </c>
       <c r="E53">
-        <v>0.33</v>
+        <v>0.27</v>
       </c>
       <c r="F53" t="s">
         <v>10</v>
@@ -4411,7 +4461,7 @@
         <v>9</v>
       </c>
       <c r="E54">
-        <v>0.19</v>
+        <v>0.13</v>
       </c>
       <c r="F54" t="s">
         <v>35</v>
@@ -4431,7 +4481,7 @@
         <v>9</v>
       </c>
       <c r="E55">
-        <v>0.37</v>
+        <v>0.18</v>
       </c>
       <c r="F55" t="s">
         <v>35</v>
@@ -4451,7 +4501,7 @@
         <v>9</v>
       </c>
       <c r="E56">
-        <v>0.22</v>
+        <v>0.39</v>
       </c>
       <c r="F56" t="s">
         <v>35</v>
@@ -4471,7 +4521,7 @@
         <v>9</v>
       </c>
       <c r="E57">
-        <v>0.2</v>
+        <v>0.39</v>
       </c>
       <c r="F57" t="s">
         <v>35</v>
@@ -4491,7 +4541,7 @@
         <v>9</v>
       </c>
       <c r="E58">
-        <v>0.28</v>
+        <v>0.34</v>
       </c>
       <c r="F58" t="s">
         <v>35</v>
@@ -4511,7 +4561,7 @@
         <v>9</v>
       </c>
       <c r="E59">
-        <v>0.25</v>
+        <v>0.28</v>
       </c>
       <c r="F59" t="s">
         <v>35</v>
@@ -4531,7 +4581,7 @@
         <v>9</v>
       </c>
       <c r="E60">
-        <v>0.29</v>
+        <v>0.19</v>
       </c>
       <c r="F60" t="s">
         <v>35</v>
@@ -4551,7 +4601,7 @@
         <v>9</v>
       </c>
       <c r="E61">
-        <v>0.14</v>
+        <v>0.13</v>
       </c>
       <c r="F61" t="s">
         <v>35</v>
@@ -4571,7 +4621,7 @@
         <v>9</v>
       </c>
       <c r="E62">
-        <v>0.36</v>
+        <v>0.24</v>
       </c>
       <c r="F62" t="s">
         <v>35</v>
@@ -4591,7 +4641,7 @@
         <v>9</v>
       </c>
       <c r="E63">
-        <v>0.15</v>
+        <v>0.23</v>
       </c>
       <c r="F63" t="s">
         <v>35</v>
@@ -4611,7 +4661,7 @@
         <v>9</v>
       </c>
       <c r="E64">
-        <v>0.23</v>
+        <v>0.12</v>
       </c>
       <c r="F64" t="s">
         <v>35</v>
@@ -4631,7 +4681,7 @@
         <v>9</v>
       </c>
       <c r="E65">
-        <v>0.34</v>
+        <v>0.39</v>
       </c>
       <c r="F65" t="s">
         <v>35</v>
@@ -4651,7 +4701,7 @@
         <v>9</v>
       </c>
       <c r="E66">
-        <v>0.19</v>
+        <v>0.13</v>
       </c>
       <c r="F66" t="s">
         <v>60</v>
@@ -4671,7 +4721,7 @@
         <v>9</v>
       </c>
       <c r="E67">
-        <v>0.35</v>
+        <v>0.24</v>
       </c>
       <c r="F67" t="s">
         <v>60</v>
@@ -4691,7 +4741,7 @@
         <v>9</v>
       </c>
       <c r="E68">
-        <v>0.36</v>
+        <v>0.19</v>
       </c>
       <c r="F68" t="s">
         <v>60</v>
@@ -4711,7 +4761,7 @@
         <v>9</v>
       </c>
       <c r="E69">
-        <v>0.13</v>
+        <v>0.39</v>
       </c>
       <c r="F69" t="s">
         <v>60</v>
@@ -4731,7 +4781,7 @@
         <v>9</v>
       </c>
       <c r="E70">
-        <v>0.23</v>
+        <v>0.38</v>
       </c>
       <c r="F70" t="s">
         <v>60</v>
@@ -4751,7 +4801,7 @@
         <v>9</v>
       </c>
       <c r="E71">
-        <v>0.33</v>
+        <v>0.36</v>
       </c>
       <c r="F71" t="s">
         <v>60</v>
@@ -4771,7 +4821,7 @@
         <v>9</v>
       </c>
       <c r="E72">
-        <v>0.13</v>
+        <v>0.17</v>
       </c>
       <c r="F72" t="s">
         <v>60</v>
@@ -4791,7 +4841,7 @@
         <v>9</v>
       </c>
       <c r="E73">
-        <v>0.34</v>
+        <v>0.3</v>
       </c>
       <c r="F73" t="s">
         <v>60</v>
@@ -4831,7 +4881,7 @@
         <v>9</v>
       </c>
       <c r="E75">
-        <v>0.36</v>
+        <v>0.29</v>
       </c>
       <c r="F75" t="s">
         <v>60</v>
@@ -4851,7 +4901,7 @@
         <v>9</v>
       </c>
       <c r="E76">
-        <v>0.25</v>
+        <v>0.12</v>
       </c>
       <c r="F76" t="s">
         <v>60</v>
@@ -4871,7 +4921,7 @@
         <v>9</v>
       </c>
       <c r="E77">
-        <v>0.39</v>
+        <v>0.22</v>
       </c>
       <c r="F77" t="s">
         <v>60</v>
@@ -4891,7 +4941,7 @@
         <v>9</v>
       </c>
       <c r="E78">
-        <v>0.18</v>
+        <v>0.25</v>
       </c>
       <c r="F78" t="s">
         <v>60</v>
@@ -4911,7 +4961,7 @@
         <v>9</v>
       </c>
       <c r="E79">
-        <v>0.29</v>
+        <v>0.38</v>
       </c>
       <c r="F79" t="s">
         <v>60</v>
@@ -4931,7 +4981,7 @@
         <v>9</v>
       </c>
       <c r="E80">
-        <v>0.35</v>
+        <v>0.26</v>
       </c>
       <c r="F80" t="s">
         <v>60</v>
@@ -4951,7 +5001,7 @@
         <v>9</v>
       </c>
       <c r="E81">
-        <v>0.36</v>
+        <v>0.15</v>
       </c>
       <c r="F81" t="s">
         <v>60</v>
@@ -4971,7 +5021,7 @@
         <v>9</v>
       </c>
       <c r="E82">
-        <v>0.12</v>
+        <v>0.21</v>
       </c>
       <c r="F82" t="s">
         <v>10</v>
@@ -4991,7 +5041,7 @@
         <v>9</v>
       </c>
       <c r="E83">
-        <v>0.2</v>
+        <v>0.31</v>
       </c>
       <c r="F83" t="s">
         <v>10</v>
@@ -5011,7 +5061,7 @@
         <v>9</v>
       </c>
       <c r="E84">
-        <v>0.12</v>
+        <v>0.22</v>
       </c>
       <c r="F84" t="s">
         <v>10</v>
@@ -5031,7 +5081,7 @@
         <v>9</v>
       </c>
       <c r="E85">
-        <v>0.17</v>
+        <v>0.37</v>
       </c>
       <c r="F85" t="s">
         <v>10</v>
@@ -5051,7 +5101,7 @@
         <v>9</v>
       </c>
       <c r="E86">
-        <v>0.29</v>
+        <v>0.25</v>
       </c>
       <c r="F86" t="s">
         <v>10</v>
@@ -5071,7 +5121,7 @@
         <v>9</v>
       </c>
       <c r="E87">
-        <v>0.15</v>
+        <v>0.3</v>
       </c>
       <c r="F87" t="s">
         <v>10</v>
@@ -5091,7 +5141,7 @@
         <v>9</v>
       </c>
       <c r="E88">
-        <v>0.4</v>
+        <v>0.37</v>
       </c>
       <c r="F88" t="s">
         <v>10</v>
@@ -5111,7 +5161,7 @@
         <v>9</v>
       </c>
       <c r="E89">
-        <v>0.1</v>
+        <v>0.21</v>
       </c>
       <c r="F89" t="s">
         <v>10</v>
@@ -5131,7 +5181,7 @@
         <v>9</v>
       </c>
       <c r="E90">
-        <v>0.32</v>
+        <v>0.36</v>
       </c>
       <c r="F90" t="s">
         <v>10</v>
@@ -5151,7 +5201,7 @@
         <v>9</v>
       </c>
       <c r="E91">
-        <v>0.17</v>
+        <v>0.13</v>
       </c>
       <c r="F91" t="s">
         <v>35</v>
@@ -5171,7 +5221,7 @@
         <v>9</v>
       </c>
       <c r="E92">
-        <v>0.2</v>
+        <v>0.16</v>
       </c>
       <c r="F92" t="s">
         <v>35</v>
@@ -5191,7 +5241,7 @@
         <v>9</v>
       </c>
       <c r="E93">
-        <v>0.15</v>
+        <v>0.24</v>
       </c>
       <c r="F93" t="s">
         <v>35</v>
@@ -5211,7 +5261,7 @@
         <v>9</v>
       </c>
       <c r="E94">
-        <v>0.38</v>
+        <v>0.23</v>
       </c>
       <c r="F94" t="s">
         <v>35</v>
@@ -5231,7 +5281,7 @@
         <v>9</v>
       </c>
       <c r="E95">
-        <v>0.26</v>
+        <v>0.15</v>
       </c>
       <c r="F95" t="s">
         <v>35</v>
@@ -5251,7 +5301,7 @@
         <v>9</v>
       </c>
       <c r="E96">
-        <v>0.1</v>
+        <v>0.14</v>
       </c>
       <c r="F96" t="s">
         <v>35</v>
@@ -5271,7 +5321,7 @@
         <v>9</v>
       </c>
       <c r="E97">
-        <v>0.33</v>
+        <v>0.25</v>
       </c>
       <c r="F97" t="s">
         <v>35</v>
@@ -5291,7 +5341,7 @@
         <v>9</v>
       </c>
       <c r="E98">
-        <v>0.28</v>
+        <v>0.2</v>
       </c>
       <c r="F98" t="s">
         <v>35</v>
@@ -5311,7 +5361,7 @@
         <v>9</v>
       </c>
       <c r="E99">
-        <v>0.16</v>
+        <v>0.4</v>
       </c>
       <c r="F99" t="s">
         <v>35</v>
@@ -5351,7 +5401,7 @@
         <v>9</v>
       </c>
       <c r="E101">
-        <v>0.31</v>
+        <v>0.36</v>
       </c>
       <c r="F101" t="s">
         <v>60</v>
@@ -5371,7 +5421,7 @@
         <v>9</v>
       </c>
       <c r="E102">
-        <v>0.19</v>
+        <v>0.2</v>
       </c>
       <c r="F102" t="s">
         <v>60</v>
@@ -5391,7 +5441,7 @@
         <v>9</v>
       </c>
       <c r="E103">
-        <v>0.16</v>
+        <v>0.21</v>
       </c>
       <c r="F103" t="s">
         <v>60</v>
@@ -5411,7 +5461,7 @@
         <v>9</v>
       </c>
       <c r="E104">
-        <v>0.17</v>
+        <v>0.26</v>
       </c>
       <c r="F104" t="s">
         <v>60</v>
@@ -5431,7 +5481,7 @@
         <v>9</v>
       </c>
       <c r="E105">
-        <v>0.27</v>
+        <v>0.13</v>
       </c>
       <c r="F105" t="s">
         <v>60</v>
@@ -5451,7 +5501,7 @@
         <v>9</v>
       </c>
       <c r="E106">
-        <v>0.16</v>
+        <v>0.39</v>
       </c>
       <c r="F106" t="s">
         <v>60</v>
@@ -5471,7 +5521,7 @@
         <v>9</v>
       </c>
       <c r="E107">
-        <v>0.27</v>
+        <v>0.32</v>
       </c>
       <c r="F107" t="s">
         <v>60</v>
@@ -5491,7 +5541,7 @@
         <v>9</v>
       </c>
       <c r="E108">
-        <v>0.13</v>
+        <v>0.19</v>
       </c>
       <c r="F108" t="s">
         <v>60</v>
@@ -5511,7 +5561,7 @@
         <v>9</v>
       </c>
       <c r="E109">
-        <v>0.13</v>
+        <v>0.32</v>
       </c>
       <c r="F109" t="s">
         <v>60</v>
@@ -5531,7 +5581,7 @@
         <v>9</v>
       </c>
       <c r="E110">
-        <v>0.11</v>
+        <v>0.24</v>
       </c>
       <c r="F110" t="s">
         <v>60</v>
@@ -5551,7 +5601,7 @@
         <v>9</v>
       </c>
       <c r="E111">
-        <v>0.35</v>
+        <v>0.12</v>
       </c>
       <c r="F111" t="s">
         <v>60</v>
@@ -5571,7 +5621,7 @@
         <v>9</v>
       </c>
       <c r="E112">
-        <v>0.3</v>
+        <v>0.34</v>
       </c>
       <c r="F112" t="s">
         <v>10</v>
@@ -5591,7 +5641,7 @@
         <v>9</v>
       </c>
       <c r="E113">
-        <v>0.2</v>
+        <v>0.14</v>
       </c>
       <c r="F113" t="s">
         <v>10</v>
@@ -5611,7 +5661,7 @@
         <v>9</v>
       </c>
       <c r="E114">
-        <v>0.17</v>
+        <v>0.25</v>
       </c>
       <c r="F114" t="s">
         <v>10</v>
@@ -5631,7 +5681,7 @@
         <v>9</v>
       </c>
       <c r="E115">
-        <v>0.24</v>
+        <v>0.18</v>
       </c>
       <c r="F115" t="s">
         <v>10</v>
@@ -5651,7 +5701,7 @@
         <v>9</v>
       </c>
       <c r="E116">
-        <v>0.34</v>
+        <v>0.19</v>
       </c>
       <c r="F116" t="s">
         <v>10</v>
@@ -5671,7 +5721,7 @@
         <v>9</v>
       </c>
       <c r="E117">
-        <v>0.31</v>
+        <v>0.14</v>
       </c>
       <c r="F117" t="s">
         <v>10</v>
@@ -5691,7 +5741,7 @@
         <v>9</v>
       </c>
       <c r="E118">
-        <v>0.2</v>
+        <v>0.39</v>
       </c>
       <c r="F118" t="s">
         <v>10</v>
@@ -5711,7 +5761,7 @@
         <v>9</v>
       </c>
       <c r="E119">
-        <v>0.33</v>
+        <v>0.24</v>
       </c>
       <c r="F119" t="s">
         <v>10</v>
@@ -5731,7 +5781,7 @@
         <v>9</v>
       </c>
       <c r="E120">
-        <v>0.28</v>
+        <v>0.13</v>
       </c>
       <c r="F120" t="s">
         <v>10</v>
@@ -5751,7 +5801,7 @@
         <v>9</v>
       </c>
       <c r="E121">
-        <v>0.14</v>
+        <v>0.28</v>
       </c>
       <c r="F121" t="s">
         <v>10</v>
@@ -5771,7 +5821,7 @@
         <v>9</v>
       </c>
       <c r="E122">
-        <v>0.17</v>
+        <v>0.34</v>
       </c>
       <c r="F122" t="s">
         <v>10</v>
@@ -5811,7 +5861,7 @@
         <v>9</v>
       </c>
       <c r="E124">
-        <v>0.32</v>
+        <v>0.39</v>
       </c>
       <c r="F124" t="s">
         <v>10</v>
@@ -5831,7 +5881,7 @@
         <v>9</v>
       </c>
       <c r="E125">
-        <v>0.34</v>
+        <v>0.38</v>
       </c>
       <c r="F125" t="s">
         <v>10</v>
@@ -5871,7 +5921,7 @@
         <v>9</v>
       </c>
       <c r="E127">
-        <v>0.38</v>
+        <v>0.12</v>
       </c>
       <c r="F127" t="s">
         <v>35</v>
@@ -5891,7 +5941,7 @@
         <v>9</v>
       </c>
       <c r="E128">
-        <v>0.35</v>
+        <v>0.18</v>
       </c>
       <c r="F128" t="s">
         <v>35</v>
@@ -5911,7 +5961,7 @@
         <v>9</v>
       </c>
       <c r="E129">
-        <v>0.35</v>
+        <v>0.19</v>
       </c>
       <c r="F129" t="s">
         <v>35</v>
@@ -5931,7 +5981,7 @@
         <v>9</v>
       </c>
       <c r="E130">
-        <v>0.17</v>
+        <v>0.31</v>
       </c>
       <c r="F130" t="s">
         <v>35</v>
@@ -5951,7 +6001,7 @@
         <v>9</v>
       </c>
       <c r="E131">
-        <v>0.39</v>
+        <v>0.21</v>
       </c>
       <c r="F131" t="s">
         <v>35</v>
@@ -5971,7 +6021,7 @@
         <v>9</v>
       </c>
       <c r="E132">
-        <v>0.25</v>
+        <v>0.3</v>
       </c>
       <c r="F132" t="s">
         <v>35</v>
@@ -5991,7 +6041,7 @@
         <v>9</v>
       </c>
       <c r="E133">
-        <v>0.26</v>
+        <v>0.36</v>
       </c>
       <c r="F133" t="s">
         <v>35</v>
@@ -6011,7 +6061,7 @@
         <v>9</v>
       </c>
       <c r="E134">
-        <v>0.11</v>
+        <v>0.24</v>
       </c>
       <c r="F134" t="s">
         <v>35</v>
@@ -6031,7 +6081,7 @@
         <v>9</v>
       </c>
       <c r="E135">
-        <v>0.32</v>
+        <v>0.24</v>
       </c>
       <c r="F135" t="s">
         <v>35</v>
@@ -6051,7 +6101,7 @@
         <v>9</v>
       </c>
       <c r="E136">
-        <v>0.15</v>
+        <v>0.25</v>
       </c>
       <c r="F136" t="s">
         <v>35</v>
@@ -6071,7 +6121,7 @@
         <v>9</v>
       </c>
       <c r="E137">
-        <v>0.15</v>
+        <v>0.14</v>
       </c>
       <c r="F137" t="s">
         <v>35</v>
@@ -6091,7 +6141,7 @@
         <v>9</v>
       </c>
       <c r="E138">
-        <v>0.12</v>
+        <v>0.27</v>
       </c>
       <c r="F138" t="s">
         <v>35</v>
@@ -6111,7 +6161,7 @@
         <v>9</v>
       </c>
       <c r="E139">
-        <v>0.11</v>
+        <v>0.25</v>
       </c>
       <c r="F139" t="s">
         <v>35</v>
@@ -6131,7 +6181,7 @@
         <v>9</v>
       </c>
       <c r="E140">
-        <v>0.21</v>
+        <v>0.26</v>
       </c>
       <c r="F140" t="s">
         <v>35</v>
@@ -6151,7 +6201,7 @@
         <v>9</v>
       </c>
       <c r="E141">
-        <v>0.34</v>
+        <v>0.35</v>
       </c>
       <c r="F141" t="s">
         <v>35</v>
@@ -6171,7 +6221,7 @@
         <v>9</v>
       </c>
       <c r="E142">
-        <v>0.16</v>
+        <v>0.25</v>
       </c>
       <c r="F142" t="s">
         <v>60</v>
@@ -6191,7 +6241,7 @@
         <v>9</v>
       </c>
       <c r="E143">
-        <v>0.3</v>
+        <v>0.18</v>
       </c>
       <c r="F143" t="s">
         <v>60</v>
@@ -6211,7 +6261,7 @@
         <v>9</v>
       </c>
       <c r="E144">
-        <v>0.38</v>
+        <v>0.11</v>
       </c>
       <c r="F144" t="s">
         <v>60</v>
@@ -6231,7 +6281,7 @@
         <v>9</v>
       </c>
       <c r="E145">
-        <v>0.18</v>
+        <v>0.24</v>
       </c>
       <c r="F145" t="s">
         <v>60</v>
@@ -6251,7 +6301,7 @@
         <v>9</v>
       </c>
       <c r="E146">
-        <v>0.34</v>
+        <v>0.27</v>
       </c>
       <c r="F146" t="s">
         <v>60</v>
@@ -6271,7 +6321,7 @@
         <v>9</v>
       </c>
       <c r="E147">
-        <v>0.3</v>
+        <v>0.31</v>
       </c>
       <c r="F147" t="s">
         <v>60</v>
@@ -6291,7 +6341,7 @@
         <v>9</v>
       </c>
       <c r="E148">
-        <v>0.26</v>
+        <v>0.35</v>
       </c>
       <c r="F148" t="s">
         <v>60</v>
@@ -6331,7 +6381,7 @@
         <v>9</v>
       </c>
       <c r="E150">
-        <v>0.24</v>
+        <v>0.12</v>
       </c>
       <c r="F150" t="s">
         <v>60</v>
@@ -6351,7 +6401,7 @@
         <v>9</v>
       </c>
       <c r="E151">
-        <v>0.11</v>
+        <v>0.17</v>
       </c>
       <c r="F151" t="s">
         <v>60</v>
@@ -6371,7 +6421,7 @@
         <v>9</v>
       </c>
       <c r="E152">
-        <v>0.32</v>
+        <v>0.29</v>
       </c>
       <c r="F152" t="s">
         <v>60</v>
@@ -6391,7 +6441,7 @@
         <v>9</v>
       </c>
       <c r="E153">
-        <v>0.26</v>
+        <v>0.34</v>
       </c>
       <c r="F153" t="s">
         <v>60</v>
@@ -6411,7 +6461,7 @@
         <v>9</v>
       </c>
       <c r="E154">
-        <v>0.36</v>
+        <v>0.16</v>
       </c>
       <c r="F154" t="s">
         <v>60</v>
@@ -6431,7 +6481,7 @@
         <v>9</v>
       </c>
       <c r="E155">
-        <v>0.28</v>
+        <v>0.12</v>
       </c>
       <c r="F155" t="s">
         <v>60</v>
@@ -6451,7 +6501,7 @@
         <v>9</v>
       </c>
       <c r="E156">
-        <v>0.2</v>
+        <v>0.39</v>
       </c>
       <c r="F156" t="s">
         <v>60</v>
@@ -6471,7 +6521,7 @@
         <v>9</v>
       </c>
       <c r="E157">
-        <v>0.34</v>
+        <v>0.28</v>
       </c>
       <c r="F157" t="s">
         <v>60</v>
@@ -6491,7 +6541,7 @@
         <v>9</v>
       </c>
       <c r="E158">
-        <v>0.38</v>
+        <v>0.24</v>
       </c>
       <c r="F158" t="s">
         <v>60</v>
@@ -6511,7 +6561,7 @@
         <v>9</v>
       </c>
       <c r="E159">
-        <v>0.28</v>
+        <v>0.39</v>
       </c>
       <c r="F159" t="s">
         <v>60</v>
@@ -6531,7 +6581,7 @@
         <v>9</v>
       </c>
       <c r="E160">
-        <v>0.36</v>
+        <v>0.1</v>
       </c>
       <c r="F160" t="s">
         <v>60</v>
@@ -6551,7 +6601,7 @@
         <v>9</v>
       </c>
       <c r="E161">
-        <v>0.23</v>
+        <v>0.11</v>
       </c>
       <c r="F161" t="s">
         <v>60</v>
@@ -6571,7 +6621,7 @@
         <v>9</v>
       </c>
       <c r="E162">
-        <v>0.32</v>
+        <v>0.22</v>
       </c>
       <c r="F162" t="s">
         <v>10</v>
@@ -6591,7 +6641,7 @@
         <v>9</v>
       </c>
       <c r="E163">
-        <v>0.38</v>
+        <v>0.14</v>
       </c>
       <c r="F163" t="s">
         <v>10</v>
@@ -6611,7 +6661,7 @@
         <v>9</v>
       </c>
       <c r="E164">
-        <v>0.17</v>
+        <v>0.11</v>
       </c>
       <c r="F164" t="s">
         <v>10</v>
@@ -6631,7 +6681,7 @@
         <v>9</v>
       </c>
       <c r="E165">
-        <v>0.32</v>
+        <v>0.18</v>
       </c>
       <c r="F165" t="s">
         <v>10</v>
@@ -6651,7 +6701,7 @@
         <v>9</v>
       </c>
       <c r="E166">
-        <v>0.19</v>
+        <v>0.4</v>
       </c>
       <c r="F166" t="s">
         <v>10</v>
@@ -6671,7 +6721,7 @@
         <v>9</v>
       </c>
       <c r="E167">
-        <v>0.37</v>
+        <v>0.11</v>
       </c>
       <c r="F167" t="s">
         <v>10</v>
@@ -6691,7 +6741,7 @@
         <v>9</v>
       </c>
       <c r="E168">
-        <v>0.3</v>
+        <v>0.15</v>
       </c>
       <c r="F168" t="s">
         <v>10</v>
@@ -6711,7 +6761,7 @@
         <v>9</v>
       </c>
       <c r="E169">
-        <v>0.16</v>
+        <v>0.11</v>
       </c>
       <c r="F169" t="s">
         <v>10</v>
@@ -6731,7 +6781,7 @@
         <v>9</v>
       </c>
       <c r="E170">
-        <v>0.22</v>
+        <v>0.37</v>
       </c>
       <c r="F170" t="s">
         <v>10</v>
@@ -6751,7 +6801,7 @@
         <v>9</v>
       </c>
       <c r="E171">
-        <v>0.16</v>
+        <v>0.32</v>
       </c>
       <c r="F171" t="s">
         <v>10</v>
@@ -6771,7 +6821,7 @@
         <v>9</v>
       </c>
       <c r="E172">
-        <v>0.18</v>
+        <v>0.26</v>
       </c>
       <c r="F172" t="s">
         <v>10</v>
@@ -6791,7 +6841,7 @@
         <v>9</v>
       </c>
       <c r="E173">
-        <v>0.35</v>
+        <v>0.18</v>
       </c>
       <c r="F173" t="s">
         <v>10</v>
@@ -6811,7 +6861,7 @@
         <v>9</v>
       </c>
       <c r="E174">
-        <v>0.2</v>
+        <v>0.37</v>
       </c>
       <c r="F174" t="s">
         <v>10</v>
@@ -6831,7 +6881,7 @@
         <v>9</v>
       </c>
       <c r="E175">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="F175" t="s">
         <v>10</v>
@@ -6851,7 +6901,7 @@
         <v>9</v>
       </c>
       <c r="E176">
-        <v>0.39</v>
+        <v>0.2</v>
       </c>
       <c r="F176" t="s">
         <v>10</v>
@@ -6871,7 +6921,7 @@
         <v>9</v>
       </c>
       <c r="E177">
-        <v>0.26</v>
+        <v>0.23</v>
       </c>
       <c r="F177" t="s">
         <v>35</v>
@@ -6891,7 +6941,7 @@
         <v>9</v>
       </c>
       <c r="E178">
-        <v>0.24</v>
+        <v>0.22</v>
       </c>
       <c r="F178" t="s">
         <v>35</v>
@@ -6911,7 +6961,7 @@
         <v>9</v>
       </c>
       <c r="E179">
-        <v>0.24</v>
+        <v>0.2</v>
       </c>
       <c r="F179" t="s">
         <v>35</v>
@@ -6931,7 +6981,7 @@
         <v>9</v>
       </c>
       <c r="E180">
-        <v>0.2</v>
+        <v>0.15</v>
       </c>
       <c r="F180" t="s">
         <v>35</v>
@@ -6951,7 +7001,7 @@
         <v>9</v>
       </c>
       <c r="E181">
-        <v>0.22</v>
+        <v>0.17</v>
       </c>
       <c r="F181" t="s">
         <v>35</v>
@@ -6971,7 +7021,7 @@
         <v>9</v>
       </c>
       <c r="E182">
-        <v>0.22</v>
+        <v>0.14</v>
       </c>
       <c r="F182" t="s">
         <v>35</v>
@@ -6991,7 +7041,7 @@
         <v>9</v>
       </c>
       <c r="E183">
-        <v>0.29</v>
+        <v>0.33</v>
       </c>
       <c r="F183" t="s">
         <v>35</v>
@@ -7011,7 +7061,7 @@
         <v>9</v>
       </c>
       <c r="E184">
-        <v>0.31</v>
+        <v>0.34</v>
       </c>
       <c r="F184" t="s">
         <v>35</v>
@@ -7031,7 +7081,7 @@
         <v>9</v>
       </c>
       <c r="E185">
-        <v>0.23</v>
+        <v>0.14</v>
       </c>
       <c r="F185" t="s">
         <v>35</v>
@@ -7051,7 +7101,7 @@
         <v>9</v>
       </c>
       <c r="E186">
-        <v>0.31</v>
+        <v>0.19</v>
       </c>
       <c r="F186" t="s">
         <v>35</v>
@@ -7071,7 +7121,7 @@
         <v>9</v>
       </c>
       <c r="E187">
-        <v>0.31</v>
+        <v>0.14</v>
       </c>
       <c r="F187" t="s">
         <v>35</v>
@@ -7091,7 +7141,7 @@
         <v>9</v>
       </c>
       <c r="E188">
-        <v>0.32</v>
+        <v>0.13</v>
       </c>
       <c r="F188" t="s">
         <v>35</v>
@@ -7111,7 +7161,7 @@
         <v>9</v>
       </c>
       <c r="E189">
-        <v>0.34</v>
+        <v>0.23</v>
       </c>
       <c r="F189" t="s">
         <v>35</v>
@@ -7131,7 +7181,7 @@
         <v>9</v>
       </c>
       <c r="E190">
-        <v>0.17</v>
+        <v>0.24</v>
       </c>
       <c r="F190" t="s">
         <v>35</v>
@@ -7151,7 +7201,7 @@
         <v>9</v>
       </c>
       <c r="E191">
-        <v>0.19</v>
+        <v>0.24</v>
       </c>
       <c r="F191" t="s">
         <v>35</v>
@@ -7171,7 +7221,7 @@
         <v>9</v>
       </c>
       <c r="E192">
-        <v>0.35</v>
+        <v>0.11</v>
       </c>
       <c r="F192" t="s">
         <v>60</v>
@@ -7191,7 +7241,7 @@
         <v>9</v>
       </c>
       <c r="E193">
-        <v>0.32</v>
+        <v>0.3</v>
       </c>
       <c r="F193" t="s">
         <v>60</v>
@@ -7211,7 +7261,7 @@
         <v>9</v>
       </c>
       <c r="E194">
-        <v>0.36</v>
+        <v>0.28</v>
       </c>
       <c r="F194" t="s">
         <v>60</v>
@@ -7231,7 +7281,7 @@
         <v>9</v>
       </c>
       <c r="E195">
-        <v>0.26</v>
+        <v>0.18</v>
       </c>
       <c r="F195" t="s">
         <v>60</v>
@@ -7251,7 +7301,7 @@
         <v>9</v>
       </c>
       <c r="E196">
-        <v>0.36</v>
+        <v>0.31</v>
       </c>
       <c r="F196" t="s">
         <v>60</v>
@@ -7271,7 +7321,7 @@
         <v>9</v>
       </c>
       <c r="E197">
-        <v>0.25</v>
+        <v>0.39</v>
       </c>
       <c r="F197" t="s">
         <v>60</v>
@@ -7291,7 +7341,7 @@
         <v>9</v>
       </c>
       <c r="E198">
-        <v>0.4</v>
+        <v>0.38</v>
       </c>
       <c r="F198" t="s">
         <v>60</v>
@@ -7311,7 +7361,7 @@
         <v>9</v>
       </c>
       <c r="E199">
-        <v>0.24</v>
+        <v>0.35</v>
       </c>
       <c r="F199" t="s">
         <v>60</v>
@@ -7331,7 +7381,7 @@
         <v>9</v>
       </c>
       <c r="E200">
-        <v>0.14</v>
+        <v>0.37</v>
       </c>
       <c r="F200" t="s">
         <v>60</v>
@@ -7351,7 +7401,7 @@
         <v>9</v>
       </c>
       <c r="E201">
-        <v>0.27</v>
+        <v>0.14</v>
       </c>
       <c r="F201" t="s">
         <v>60</v>
@@ -7371,7 +7421,7 @@
         <v>9</v>
       </c>
       <c r="E202">
-        <v>0.13</v>
+        <v>0.36</v>
       </c>
       <c r="F202" t="s">
         <v>60</v>
@@ -7391,7 +7441,7 @@
         <v>9</v>
       </c>
       <c r="E203">
-        <v>0.15</v>
+        <v>0.18</v>
       </c>
       <c r="F203" t="s">
         <v>60</v>
@@ -7411,7 +7461,7 @@
         <v>9</v>
       </c>
       <c r="E204">
-        <v>0.29</v>
+        <v>0.3</v>
       </c>
       <c r="F204" t="s">
         <v>60</v>
@@ -7431,7 +7481,7 @@
         <v>9</v>
       </c>
       <c r="E205">
-        <v>0.34</v>
+        <v>0.38</v>
       </c>
       <c r="F205" t="s">
         <v>60</v>
@@ -7471,7 +7521,7 @@
         <v>9</v>
       </c>
       <c r="E207">
-        <v>0.17</v>
+        <v>0.15</v>
       </c>
       <c r="F207" t="s">
         <v>60</v>
@@ -7491,7 +7541,7 @@
         <v>9</v>
       </c>
       <c r="E208">
-        <v>0.27</v>
+        <v>0.2</v>
       </c>
       <c r="F208" t="s">
         <v>60</v>
@@ -7511,7 +7561,7 @@
         <v>9</v>
       </c>
       <c r="E209">
-        <v>0.12</v>
+        <v>0.35</v>
       </c>
       <c r="F209" t="s">
         <v>60</v>
@@ -7531,7 +7581,7 @@
         <v>9</v>
       </c>
       <c r="E210">
-        <v>0.18</v>
+        <v>0.39</v>
       </c>
       <c r="F210" t="s">
         <v>60</v>
@@ -7551,7 +7601,7 @@
         <v>9</v>
       </c>
       <c r="E211">
-        <v>0.33</v>
+        <v>0.17</v>
       </c>
       <c r="F211" t="s">
         <v>60</v>
@@ -7571,7 +7621,7 @@
         <v>9</v>
       </c>
       <c r="E212">
-        <v>0.27</v>
+        <v>0.39</v>
       </c>
       <c r="F212" t="s">
         <v>10</v>
@@ -7591,7 +7641,7 @@
         <v>9</v>
       </c>
       <c r="E213">
-        <v>0.34</v>
+        <v>0.16</v>
       </c>
       <c r="F213" t="s">
         <v>10</v>
@@ -7611,7 +7661,7 @@
         <v>9</v>
       </c>
       <c r="E214">
-        <v>0.22</v>
+        <v>0.21</v>
       </c>
       <c r="F214" t="s">
         <v>10</v>
@@ -7631,7 +7681,7 @@
         <v>9</v>
       </c>
       <c r="E215">
-        <v>0.17</v>
+        <v>0.19</v>
       </c>
       <c r="F215" t="s">
         <v>10</v>
@@ -7651,7 +7701,7 @@
         <v>9</v>
       </c>
       <c r="E216">
-        <v>0.37</v>
+        <v>0.33</v>
       </c>
       <c r="F216" t="s">
         <v>10</v>
@@ -7671,7 +7721,7 @@
         <v>9</v>
       </c>
       <c r="E217">
-        <v>0.3</v>
+        <v>0.37</v>
       </c>
       <c r="F217" t="s">
         <v>10</v>
@@ -7691,7 +7741,7 @@
         <v>9</v>
       </c>
       <c r="E218">
-        <v>0.17</v>
+        <v>0.13</v>
       </c>
       <c r="F218" t="s">
         <v>10</v>
@@ -7711,7 +7761,7 @@
         <v>9</v>
       </c>
       <c r="E219">
-        <v>0.14</v>
+        <v>0.1</v>
       </c>
       <c r="F219" t="s">
         <v>10</v>
@@ -7731,7 +7781,7 @@
         <v>9</v>
       </c>
       <c r="E220">
-        <v>0.17</v>
+        <v>0.2</v>
       </c>
       <c r="F220" t="s">
         <v>10</v>
@@ -7751,7 +7801,7 @@
         <v>9</v>
       </c>
       <c r="E221">
-        <v>0.13</v>
+        <v>0.37</v>
       </c>
       <c r="F221" t="s">
         <v>10</v>
@@ -7771,7 +7821,7 @@
         <v>9</v>
       </c>
       <c r="E222">
-        <v>0.36</v>
+        <v>0.13</v>
       </c>
       <c r="F222" t="s">
         <v>10</v>
@@ -7791,7 +7841,7 @@
         <v>9</v>
       </c>
       <c r="E223">
-        <v>0.1</v>
+        <v>0.14</v>
       </c>
       <c r="F223" t="s">
         <v>10</v>
@@ -7811,7 +7861,7 @@
         <v>9</v>
       </c>
       <c r="E224">
-        <v>0.11</v>
+        <v>0.15</v>
       </c>
       <c r="F224" t="s">
         <v>10</v>
@@ -7831,7 +7881,7 @@
         <v>9</v>
       </c>
       <c r="E225">
-        <v>0.11</v>
+        <v>0.34</v>
       </c>
       <c r="F225" t="s">
         <v>10</v>
@@ -7851,7 +7901,7 @@
         <v>9</v>
       </c>
       <c r="E226">
-        <v>0.13</v>
+        <v>0.15</v>
       </c>
       <c r="F226" t="s">
         <v>10</v>
@@ -7871,7 +7921,7 @@
         <v>9</v>
       </c>
       <c r="E227">
-        <v>0.26</v>
+        <v>0.12</v>
       </c>
       <c r="F227" t="s">
         <v>35</v>
@@ -7891,7 +7941,7 @@
         <v>9</v>
       </c>
       <c r="E228">
-        <v>0.14</v>
+        <v>0.32</v>
       </c>
       <c r="F228" t="s">
         <v>35</v>
@@ -7911,7 +7961,7 @@
         <v>9</v>
       </c>
       <c r="E229">
-        <v>0.17</v>
+        <v>0.27</v>
       </c>
       <c r="F229" t="s">
         <v>35</v>
@@ -7951,7 +8001,7 @@
         <v>9</v>
       </c>
       <c r="E231">
-        <v>0.29</v>
+        <v>0.18</v>
       </c>
       <c r="F231" t="s">
         <v>35</v>
@@ -7971,7 +8021,7 @@
         <v>9</v>
       </c>
       <c r="E232">
-        <v>0.19</v>
+        <v>0.22</v>
       </c>
       <c r="F232" t="s">
         <v>35</v>
@@ -7991,7 +8041,7 @@
         <v>9</v>
       </c>
       <c r="E233">
-        <v>0.37</v>
+        <v>0.23</v>
       </c>
       <c r="F233" t="s">
         <v>35</v>
@@ -8011,7 +8061,7 @@
         <v>9</v>
       </c>
       <c r="E234">
-        <v>0.15</v>
+        <v>0.36</v>
       </c>
       <c r="F234" t="s">
         <v>35</v>
@@ -8031,7 +8081,7 @@
         <v>9</v>
       </c>
       <c r="E235">
-        <v>0.3</v>
+        <v>0.23</v>
       </c>
       <c r="F235" t="s">
         <v>35</v>
@@ -8071,7 +8121,7 @@
         <v>9</v>
       </c>
       <c r="E237">
-        <v>0.35</v>
+        <v>0.28</v>
       </c>
       <c r="F237" t="s">
         <v>35</v>
@@ -8091,7 +8141,7 @@
         <v>9</v>
       </c>
       <c r="E238">
-        <v>0.32</v>
+        <v>0.18</v>
       </c>
       <c r="F238" t="s">
         <v>35</v>
@@ -8111,7 +8161,7 @@
         <v>9</v>
       </c>
       <c r="E239">
-        <v>0.35</v>
+        <v>0.14</v>
       </c>
       <c r="F239" t="s">
         <v>35</v>
@@ -8131,7 +8181,7 @@
         <v>9</v>
       </c>
       <c r="E240">
-        <v>0.15</v>
+        <v>0.31</v>
       </c>
       <c r="F240" t="s">
         <v>35</v>
@@ -8151,7 +8201,7 @@
         <v>9</v>
       </c>
       <c r="E241">
-        <v>0.16</v>
+        <v>0.29</v>
       </c>
       <c r="F241" t="s">
         <v>35</v>
@@ -8171,7 +8221,7 @@
         <v>9</v>
       </c>
       <c r="E242">
-        <v>0.16</v>
+        <v>0.19</v>
       </c>
       <c r="F242" t="s">
         <v>60</v>
@@ -8191,7 +8241,7 @@
         <v>9</v>
       </c>
       <c r="E243">
-        <v>0.28</v>
+        <v>0.21</v>
       </c>
       <c r="F243" t="s">
         <v>60</v>
@@ -8231,7 +8281,7 @@
         <v>9</v>
       </c>
       <c r="E245">
-        <v>0.2</v>
+        <v>0.31</v>
       </c>
       <c r="F245" t="s">
         <v>60</v>
@@ -8251,7 +8301,7 @@
         <v>9</v>
       </c>
       <c r="E246">
-        <v>0.23</v>
+        <v>0.27</v>
       </c>
       <c r="F246" t="s">
         <v>60</v>
@@ -8271,7 +8321,7 @@
         <v>9</v>
       </c>
       <c r="E247">
-        <v>0.36</v>
+        <v>0.26</v>
       </c>
       <c r="F247" t="s">
         <v>60</v>
@@ -8311,7 +8361,7 @@
         <v>9</v>
       </c>
       <c r="E249">
-        <v>0.12</v>
+        <v>0.25</v>
       </c>
       <c r="F249" t="s">
         <v>60</v>
@@ -8331,7 +8381,7 @@
         <v>9</v>
       </c>
       <c r="E250">
-        <v>0.11</v>
+        <v>0.16</v>
       </c>
       <c r="F250" t="s">
         <v>60</v>
@@ -8351,7 +8401,7 @@
         <v>9</v>
       </c>
       <c r="E251">
-        <v>0.38</v>
+        <v>0.22</v>
       </c>
       <c r="F251" t="s">
         <v>60</v>
@@ -8371,7 +8421,7 @@
         <v>9</v>
       </c>
       <c r="E252">
-        <v>0.15</v>
+        <v>0.13</v>
       </c>
       <c r="F252" t="s">
         <v>60</v>
@@ -8391,7 +8441,7 @@
         <v>9</v>
       </c>
       <c r="E253">
-        <v>0.38</v>
+        <v>0.26</v>
       </c>
       <c r="F253" t="s">
         <v>60</v>
@@ -8411,7 +8461,7 @@
         <v>9</v>
       </c>
       <c r="E254">
-        <v>0.25</v>
+        <v>0.3</v>
       </c>
       <c r="F254" t="s">
         <v>60</v>
@@ -8431,7 +8481,7 @@
         <v>9</v>
       </c>
       <c r="E255">
-        <v>0.35</v>
+        <v>0.13</v>
       </c>
       <c r="F255" t="s">
         <v>60</v>
@@ -8451,7 +8501,7 @@
         <v>9</v>
       </c>
       <c r="E256">
-        <v>0.11</v>
+        <v>0.3</v>
       </c>
       <c r="F256" t="s">
         <v>60</v>
@@ -8471,7 +8521,7 @@
         <v>9</v>
       </c>
       <c r="E257">
-        <v>0.28</v>
+        <v>0.34</v>
       </c>
       <c r="F257" t="s">
         <v>60</v>
@@ -8491,7 +8541,7 @@
         <v>9</v>
       </c>
       <c r="E258">
-        <v>0.24</v>
+        <v>0.33</v>
       </c>
       <c r="F258" t="s">
         <v>60</v>
@@ -8511,7 +8561,7 @@
         <v>9</v>
       </c>
       <c r="E259">
-        <v>0.37</v>
+        <v>0.13</v>
       </c>
       <c r="F259" t="s">
         <v>60</v>
@@ -8531,7 +8581,7 @@
         <v>9</v>
       </c>
       <c r="E260">
-        <v>0.4</v>
+        <v>0.39</v>
       </c>
       <c r="F260" t="s">
         <v>60</v>
@@ -8551,7 +8601,7 @@
         <v>9</v>
       </c>
       <c r="E261">
-        <v>0.25</v>
+        <v>0.14</v>
       </c>
       <c r="F261" t="s">
         <v>60</v>
@@ -8571,7 +8621,7 @@
         <v>9</v>
       </c>
       <c r="E262">
-        <v>0.21</v>
+        <v>0.36</v>
       </c>
       <c r="F262" t="s">
         <v>10</v>
@@ -8591,7 +8641,7 @@
         <v>9</v>
       </c>
       <c r="E263">
-        <v>0.22</v>
+        <v>0.39</v>
       </c>
       <c r="F263" t="s">
         <v>10</v>
@@ -8611,7 +8661,7 @@
         <v>9</v>
       </c>
       <c r="E264">
-        <v>0.39</v>
+        <v>0.33</v>
       </c>
       <c r="F264" t="s">
         <v>10</v>
@@ -8631,7 +8681,7 @@
         <v>9</v>
       </c>
       <c r="E265">
-        <v>0.17</v>
+        <v>0.16</v>
       </c>
       <c r="F265" t="s">
         <v>10</v>
@@ -8651,7 +8701,7 @@
         <v>9</v>
       </c>
       <c r="E266">
-        <v>0.24</v>
+        <v>0.12</v>
       </c>
       <c r="F266" t="s">
         <v>10</v>
@@ -8671,7 +8721,7 @@
         <v>9</v>
       </c>
       <c r="E267">
-        <v>0.32</v>
+        <v>0.22</v>
       </c>
       <c r="F267" t="s">
         <v>10</v>
@@ -8691,7 +8741,7 @@
         <v>9</v>
       </c>
       <c r="E268">
-        <v>0.37</v>
+        <v>0.35</v>
       </c>
       <c r="F268" t="s">
         <v>10</v>
@@ -8711,7 +8761,7 @@
         <v>9</v>
       </c>
       <c r="E269">
-        <v>0.31</v>
+        <v>0.3</v>
       </c>
       <c r="F269" t="s">
         <v>10</v>
@@ -8731,7 +8781,7 @@
         <v>9</v>
       </c>
       <c r="E270">
-        <v>0.3</v>
+        <v>0.17</v>
       </c>
       <c r="F270" t="s">
         <v>10</v>
@@ -8751,7 +8801,7 @@
         <v>9</v>
       </c>
       <c r="E271">
-        <v>0.14</v>
+        <v>0.37</v>
       </c>
       <c r="F271" t="s">
         <v>10</v>
@@ -8771,7 +8821,7 @@
         <v>9</v>
       </c>
       <c r="E272">
-        <v>0.26</v>
+        <v>0.34</v>
       </c>
       <c r="F272" t="s">
         <v>10</v>
@@ -8791,7 +8841,7 @@
         <v>9</v>
       </c>
       <c r="E273">
-        <v>0.12</v>
+        <v>0.34</v>
       </c>
       <c r="F273" t="s">
         <v>10</v>
@@ -8811,7 +8861,7 @@
         <v>9</v>
       </c>
       <c r="E274">
-        <v>0.27</v>
+        <v>0.28</v>
       </c>
       <c r="F274" t="s">
         <v>35</v>
@@ -8831,7 +8881,7 @@
         <v>9</v>
       </c>
       <c r="E275">
-        <v>0.29</v>
+        <v>0.12</v>
       </c>
       <c r="F275" t="s">
         <v>35</v>
@@ -8851,7 +8901,7 @@
         <v>9</v>
       </c>
       <c r="E276">
-        <v>0.17</v>
+        <v>0.27</v>
       </c>
       <c r="F276" t="s">
         <v>35</v>
@@ -8871,7 +8921,7 @@
         <v>9</v>
       </c>
       <c r="E277">
-        <v>0.37</v>
+        <v>0.29</v>
       </c>
       <c r="F277" t="s">
         <v>35</v>
@@ -8891,7 +8941,7 @@
         <v>9</v>
       </c>
       <c r="E278">
-        <v>0.21</v>
+        <v>0.17</v>
       </c>
       <c r="F278" t="s">
         <v>35</v>
@@ -8911,7 +8961,7 @@
         <v>9</v>
       </c>
       <c r="E279">
-        <v>0.12</v>
+        <v>0.38</v>
       </c>
       <c r="F279" t="s">
         <v>35</v>
@@ -8931,7 +8981,7 @@
         <v>9</v>
       </c>
       <c r="E280">
-        <v>0.28</v>
+        <v>0.11</v>
       </c>
       <c r="F280" t="s">
         <v>35</v>
@@ -8951,7 +9001,7 @@
         <v>9</v>
       </c>
       <c r="E281">
-        <v>0.36</v>
+        <v>0.23</v>
       </c>
       <c r="F281" t="s">
         <v>35</v>
@@ -8971,7 +9021,7 @@
         <v>9</v>
       </c>
       <c r="E282">
-        <v>0.32</v>
+        <v>0.26</v>
       </c>
       <c r="F282" t="s">
         <v>35</v>
@@ -8991,7 +9041,7 @@
         <v>9</v>
       </c>
       <c r="E283">
-        <v>0.38</v>
+        <v>0.19</v>
       </c>
       <c r="F283" t="s">
         <v>35</v>
@@ -9011,7 +9061,7 @@
         <v>9</v>
       </c>
       <c r="E284">
-        <v>0.14</v>
+        <v>0.23</v>
       </c>
       <c r="F284" t="s">
         <v>35</v>
@@ -9031,7 +9081,7 @@
         <v>9</v>
       </c>
       <c r="E285">
-        <v>0.16</v>
+        <v>0.24</v>
       </c>
       <c r="F285" t="s">
         <v>35</v>
@@ -9051,7 +9101,7 @@
         <v>9</v>
       </c>
       <c r="E286">
-        <v>0.33</v>
+        <v>0.12</v>
       </c>
       <c r="F286" t="s">
         <v>60</v>
@@ -9071,7 +9121,7 @@
         <v>9</v>
       </c>
       <c r="E287">
-        <v>0.36</v>
+        <v>0.4</v>
       </c>
       <c r="F287" t="s">
         <v>60</v>
@@ -9091,7 +9141,7 @@
         <v>9</v>
       </c>
       <c r="E288">
-        <v>0.12</v>
+        <v>0.27</v>
       </c>
       <c r="F288" t="s">
         <v>60</v>
@@ -9111,7 +9161,7 @@
         <v>9</v>
       </c>
       <c r="E289">
-        <v>0.27</v>
+        <v>0.25</v>
       </c>
       <c r="F289" t="s">
         <v>60</v>
@@ -9131,7 +9181,7 @@
         <v>9</v>
       </c>
       <c r="E290">
-        <v>0.21</v>
+        <v>0.19</v>
       </c>
       <c r="F290" t="s">
         <v>60</v>
@@ -9151,7 +9201,7 @@
         <v>9</v>
       </c>
       <c r="E291">
-        <v>0.14</v>
+        <v>0.36</v>
       </c>
       <c r="F291" t="s">
         <v>60</v>
@@ -9171,7 +9221,7 @@
         <v>9</v>
       </c>
       <c r="E292">
-        <v>0.37</v>
+        <v>0.32</v>
       </c>
       <c r="F292" t="s">
         <v>60</v>
@@ -9191,7 +9241,7 @@
         <v>9</v>
       </c>
       <c r="E293">
-        <v>0.39</v>
+        <v>0.23</v>
       </c>
       <c r="F293" t="s">
         <v>60</v>
@@ -9211,7 +9261,7 @@
         <v>9</v>
       </c>
       <c r="E294">
-        <v>0.27</v>
+        <v>0.36</v>
       </c>
       <c r="F294" t="s">
         <v>60</v>
@@ -9231,7 +9281,7 @@
         <v>9</v>
       </c>
       <c r="E295">
-        <v>0.32</v>
+        <v>0.33</v>
       </c>
       <c r="F295" t="s">
         <v>60</v>
@@ -9251,7 +9301,7 @@
         <v>9</v>
       </c>
       <c r="E296">
-        <v>0.16</v>
+        <v>0.18</v>
       </c>
       <c r="F296" t="s">
         <v>60</v>
@@ -9271,7 +9321,7 @@
         <v>9</v>
       </c>
       <c r="E297">
-        <v>0.37</v>
+        <v>0.26</v>
       </c>
       <c r="F297" t="s">
         <v>60</v>
@@ -9291,7 +9341,7 @@
         <v>9</v>
       </c>
       <c r="E298">
-        <v>0.13</v>
+        <v>0.17</v>
       </c>
       <c r="F298" t="s">
         <v>60</v>
@@ -9311,7 +9361,7 @@
         <v>9</v>
       </c>
       <c r="E299">
-        <v>0.33</v>
+        <v>0.19</v>
       </c>
       <c r="F299" t="s">
         <v>60</v>
@@ -9331,7 +9381,7 @@
         <v>9</v>
       </c>
       <c r="E300">
-        <v>0.26</v>
+        <v>0.18</v>
       </c>
       <c r="F300" t="s">
         <v>60</v>
@@ -9351,7 +9401,7 @@
         <v>9</v>
       </c>
       <c r="E301">
-        <v>0.26</v>
+        <v>0.25</v>
       </c>
       <c r="F301" t="s">
         <v>60</v>
@@ -9371,7 +9421,7 @@
         <v>9</v>
       </c>
       <c r="E302">
-        <v>0.16</v>
+        <v>0.4</v>
       </c>
       <c r="F302" t="s">
         <v>10</v>
@@ -9391,7 +9441,7 @@
         <v>9</v>
       </c>
       <c r="E303">
-        <v>0.34</v>
+        <v>0.18</v>
       </c>
       <c r="F303" t="s">
         <v>10</v>
@@ -9411,7 +9461,7 @@
         <v>9</v>
       </c>
       <c r="E304">
-        <v>0.17</v>
+        <v>0.25</v>
       </c>
       <c r="F304" t="s">
         <v>10</v>
@@ -9431,7 +9481,7 @@
         <v>9</v>
       </c>
       <c r="E305">
-        <v>0.25</v>
+        <v>0.14</v>
       </c>
       <c r="F305" t="s">
         <v>10</v>
@@ -9451,7 +9501,7 @@
         <v>9</v>
       </c>
       <c r="E306">
-        <v>0.31</v>
+        <v>0.36</v>
       </c>
       <c r="F306" t="s">
         <v>10</v>
@@ -9471,7 +9521,7 @@
         <v>9</v>
       </c>
       <c r="E307">
-        <v>0.29</v>
+        <v>0.22</v>
       </c>
       <c r="F307" t="s">
         <v>10</v>
@@ -9491,7 +9541,7 @@
         <v>9</v>
       </c>
       <c r="E308">
-        <v>0.24</v>
+        <v>0.17</v>
       </c>
       <c r="F308" t="s">
         <v>35</v>
@@ -9511,7 +9561,7 @@
         <v>9</v>
       </c>
       <c r="E309">
-        <v>0.27</v>
+        <v>0.11</v>
       </c>
       <c r="F309" t="s">
         <v>35</v>
@@ -9531,7 +9581,7 @@
         <v>9</v>
       </c>
       <c r="E310">
-        <v>0.28</v>
+        <v>0.31</v>
       </c>
       <c r="F310" t="s">
         <v>35</v>
@@ -9551,7 +9601,7 @@
         <v>9</v>
       </c>
       <c r="E311">
-        <v>0.36</v>
+        <v>0.28</v>
       </c>
       <c r="F311" t="s">
         <v>35</v>
@@ -9571,7 +9621,7 @@
         <v>9</v>
       </c>
       <c r="E312">
-        <v>0.19</v>
+        <v>0.15</v>
       </c>
       <c r="F312" t="s">
         <v>35</v>
@@ -9591,7 +9641,7 @@
         <v>9</v>
       </c>
       <c r="E313">
-        <v>0.18</v>
+        <v>0.31</v>
       </c>
       <c r="F313" t="s">
         <v>35</v>
@@ -9611,7 +9661,7 @@
         <v>9</v>
       </c>
       <c r="E314">
-        <v>0.39</v>
+        <v>0.3</v>
       </c>
       <c r="F314" t="s">
         <v>60</v>
@@ -9631,7 +9681,7 @@
         <v>9</v>
       </c>
       <c r="E315">
-        <v>0.1</v>
+        <v>0.12</v>
       </c>
       <c r="F315" t="s">
         <v>60</v>
@@ -9651,7 +9701,7 @@
         <v>9</v>
       </c>
       <c r="E316">
-        <v>0.17</v>
+        <v>0.36</v>
       </c>
       <c r="F316" t="s">
         <v>60</v>
@@ -9671,7 +9721,7 @@
         <v>9</v>
       </c>
       <c r="E317">
-        <v>0.35</v>
+        <v>0.31</v>
       </c>
       <c r="F317" t="s">
         <v>60</v>
@@ -9711,7 +9761,7 @@
         <v>9</v>
       </c>
       <c r="E319">
-        <v>0.15</v>
+        <v>0.11</v>
       </c>
       <c r="F319" t="s">
         <v>60</v>
@@ -9731,7 +9781,7 @@
         <v>9</v>
       </c>
       <c r="E320">
-        <v>0.25</v>
+        <v>0.24</v>
       </c>
       <c r="F320" t="s">
         <v>60</v>
@@ -9751,7 +9801,7 @@
         <v>9</v>
       </c>
       <c r="E321">
-        <v>0.23</v>
+        <v>0.35</v>
       </c>
       <c r="F321" t="s">
         <v>60</v>
@@ -9771,7 +9821,7 @@
         <v>9</v>
       </c>
       <c r="E322">
-        <v>0.14</v>
+        <v>0.34</v>
       </c>
       <c r="F322" t="s">
         <v>10</v>
@@ -9791,7 +9841,7 @@
         <v>9</v>
       </c>
       <c r="E323">
-        <v>0.11</v>
+        <v>0.19</v>
       </c>
       <c r="F323" t="s">
         <v>10</v>
@@ -9811,7 +9861,7 @@
         <v>9</v>
       </c>
       <c r="E324">
-        <v>0.13</v>
+        <v>0.14</v>
       </c>
       <c r="F324" t="s">
         <v>10</v>
@@ -9831,7 +9881,7 @@
         <v>9</v>
       </c>
       <c r="E325">
-        <v>0.22</v>
+        <v>0.31</v>
       </c>
       <c r="F325" t="s">
         <v>10</v>
@@ -9851,7 +9901,7 @@
         <v>9</v>
       </c>
       <c r="E326">
-        <v>0.3</v>
+        <v>0.22</v>
       </c>
       <c r="F326" t="s">
         <v>10</v>
@@ -9871,7 +9921,7 @@
         <v>9</v>
       </c>
       <c r="E327">
-        <v>0.22</v>
+        <v>0.34</v>
       </c>
       <c r="F327" t="s">
         <v>10</v>
@@ -9891,7 +9941,7 @@
         <v>9</v>
       </c>
       <c r="E328">
-        <v>0.23</v>
+        <v>0.27</v>
       </c>
       <c r="F328" t="s">
         <v>35</v>
@@ -9911,7 +9961,7 @@
         <v>9</v>
       </c>
       <c r="E329">
-        <v>0.15</v>
+        <v>0.17</v>
       </c>
       <c r="F329" t="s">
         <v>35</v>
@@ -9931,7 +9981,7 @@
         <v>9</v>
       </c>
       <c r="E330">
-        <v>0.14</v>
+        <v>0.17</v>
       </c>
       <c r="F330" t="s">
         <v>35</v>
@@ -9951,7 +10001,7 @@
         <v>9</v>
       </c>
       <c r="E331">
-        <v>0.15</v>
+        <v>0.12</v>
       </c>
       <c r="F331" t="s">
         <v>35</v>
@@ -9971,7 +10021,7 @@
         <v>9</v>
       </c>
       <c r="E332">
-        <v>0.35</v>
+        <v>0.36</v>
       </c>
       <c r="F332" t="s">
         <v>35</v>
@@ -9991,7 +10041,7 @@
         <v>9</v>
       </c>
       <c r="E333">
-        <v>0.36</v>
+        <v>0.23</v>
       </c>
       <c r="F333" t="s">
         <v>35</v>
@@ -10011,7 +10061,7 @@
         <v>9</v>
       </c>
       <c r="E334">
-        <v>0.32</v>
+        <v>0.24</v>
       </c>
       <c r="F334" t="s">
         <v>60</v>
@@ -10031,7 +10081,7 @@
         <v>9</v>
       </c>
       <c r="E335">
-        <v>0.37</v>
+        <v>0.11</v>
       </c>
       <c r="F335" t="s">
         <v>60</v>
@@ -10051,7 +10101,7 @@
         <v>9</v>
       </c>
       <c r="E336">
-        <v>0.22</v>
+        <v>0.32</v>
       </c>
       <c r="F336" t="s">
         <v>60</v>
@@ -10071,7 +10121,7 @@
         <v>9</v>
       </c>
       <c r="E337">
-        <v>0.28</v>
+        <v>0.35</v>
       </c>
       <c r="F337" t="s">
         <v>60</v>
@@ -10091,7 +10141,7 @@
         <v>9</v>
       </c>
       <c r="E338">
-        <v>0.26</v>
+        <v>0.11</v>
       </c>
       <c r="F338" t="s">
         <v>60</v>
@@ -10111,7 +10161,7 @@
         <v>9</v>
       </c>
       <c r="E339">
-        <v>0.35</v>
+        <v>0.17</v>
       </c>
       <c r="F339" t="s">
         <v>60</v>
@@ -10131,7 +10181,7 @@
         <v>9</v>
       </c>
       <c r="E340">
-        <v>0.27</v>
+        <v>0.24</v>
       </c>
       <c r="F340" t="s">
         <v>60</v>
@@ -10151,7 +10201,7 @@
         <v>9</v>
       </c>
       <c r="E341">
-        <v>0.23</v>
+        <v>0.25</v>
       </c>
       <c r="F341" t="s">
         <v>60</v>
@@ -10171,7 +10221,7 @@
         <v>9</v>
       </c>
       <c r="E342">
-        <v>0.22</v>
+        <v>0.19</v>
       </c>
       <c r="F342" t="s">
         <v>10</v>
@@ -10191,7 +10241,7 @@
         <v>9</v>
       </c>
       <c r="E343">
-        <v>0.13</v>
+        <v>0.16</v>
       </c>
       <c r="F343" t="s">
         <v>10</v>
@@ -10211,7 +10261,7 @@
         <v>9</v>
       </c>
       <c r="E344">
-        <v>0.23</v>
+        <v>0.28</v>
       </c>
       <c r="F344" t="s">
         <v>10</v>
@@ -10231,7 +10281,7 @@
         <v>9</v>
       </c>
       <c r="E345">
-        <v>0.29</v>
+        <v>0.35</v>
       </c>
       <c r="F345" t="s">
         <v>10</v>
@@ -10251,7 +10301,7 @@
         <v>9</v>
       </c>
       <c r="E346">
-        <v>0.21</v>
+        <v>0.18</v>
       </c>
       <c r="F346" t="s">
         <v>10</v>
@@ -10271,7 +10321,7 @@
         <v>9</v>
       </c>
       <c r="E347">
-        <v>0.36</v>
+        <v>0.25</v>
       </c>
       <c r="F347" t="s">
         <v>10</v>
@@ -10291,7 +10341,7 @@
         <v>9</v>
       </c>
       <c r="E348">
-        <v>0.27</v>
+        <v>0.37</v>
       </c>
       <c r="F348" t="s">
         <v>35</v>
@@ -10311,7 +10361,7 @@
         <v>9</v>
       </c>
       <c r="E349">
-        <v>0.16</v>
+        <v>0.38</v>
       </c>
       <c r="F349" t="s">
         <v>35</v>
@@ -10331,7 +10381,7 @@
         <v>9</v>
       </c>
       <c r="E350">
-        <v>0.31</v>
+        <v>0.37</v>
       </c>
       <c r="F350" t="s">
         <v>35</v>
@@ -10351,7 +10401,7 @@
         <v>9</v>
       </c>
       <c r="E351">
-        <v>0.17</v>
+        <v>0.36</v>
       </c>
       <c r="F351" t="s">
         <v>35</v>
@@ -10371,7 +10421,7 @@
         <v>9</v>
       </c>
       <c r="E352">
-        <v>0.39</v>
+        <v>0.25</v>
       </c>
       <c r="F352" t="s">
         <v>35</v>
@@ -10391,7 +10441,7 @@
         <v>9</v>
       </c>
       <c r="E353">
-        <v>0.13</v>
+        <v>0.33</v>
       </c>
       <c r="F353" t="s">
         <v>35</v>
@@ -10411,7 +10461,7 @@
         <v>9</v>
       </c>
       <c r="E354">
-        <v>0.18</v>
+        <v>0.39</v>
       </c>
       <c r="F354" t="s">
         <v>60</v>
@@ -10431,7 +10481,7 @@
         <v>9</v>
       </c>
       <c r="E355">
-        <v>0.37</v>
+        <v>0.13</v>
       </c>
       <c r="F355" t="s">
         <v>60</v>
@@ -10471,7 +10521,7 @@
         <v>9</v>
       </c>
       <c r="E357">
-        <v>0.15</v>
+        <v>0.39</v>
       </c>
       <c r="F357" t="s">
         <v>60</v>
@@ -10491,7 +10541,7 @@
         <v>9</v>
       </c>
       <c r="E358">
-        <v>0.15</v>
+        <v>0.33</v>
       </c>
       <c r="F358" t="s">
         <v>60</v>
@@ -10511,7 +10561,7 @@
         <v>9</v>
       </c>
       <c r="E359">
-        <v>0.16</v>
+        <v>0.12</v>
       </c>
       <c r="F359" t="s">
         <v>60</v>
@@ -10531,7 +10581,7 @@
         <v>9</v>
       </c>
       <c r="E360">
-        <v>0.11</v>
+        <v>0.29</v>
       </c>
       <c r="F360" t="s">
         <v>60</v>
@@ -10551,7 +10601,7 @@
         <v>9</v>
       </c>
       <c r="E361">
-        <v>0.12</v>
+        <v>0.2</v>
       </c>
       <c r="F361" t="s">
         <v>60</v>
@@ -10571,7 +10621,7 @@
         <v>9</v>
       </c>
       <c r="E362">
-        <v>0.38</v>
+        <v>0.17</v>
       </c>
       <c r="F362" t="s">
         <v>10</v>
@@ -10591,7 +10641,7 @@
         <v>9</v>
       </c>
       <c r="E363">
-        <v>0.33</v>
+        <v>0.38</v>
       </c>
       <c r="F363" t="s">
         <v>10</v>
@@ -10631,7 +10681,7 @@
         <v>9</v>
       </c>
       <c r="E365">
-        <v>0.21</v>
+        <v>0.17</v>
       </c>
       <c r="F365" t="s">
         <v>10</v>
@@ -10651,7 +10701,7 @@
         <v>9</v>
       </c>
       <c r="E366">
-        <v>0.17</v>
+        <v>0.35</v>
       </c>
       <c r="F366" t="s">
         <v>10</v>
@@ -10671,7 +10721,7 @@
         <v>9</v>
       </c>
       <c r="E367">
-        <v>0.4</v>
+        <v>0.23</v>
       </c>
       <c r="F367" t="s">
         <v>10</v>
@@ -10691,7 +10741,7 @@
         <v>9</v>
       </c>
       <c r="E368">
-        <v>0.3</v>
+        <v>0.27</v>
       </c>
       <c r="F368" t="s">
         <v>35</v>
@@ -10711,7 +10761,7 @@
         <v>9</v>
       </c>
       <c r="E369">
-        <v>0.25</v>
+        <v>0.33</v>
       </c>
       <c r="F369" t="s">
         <v>35</v>
@@ -10731,7 +10781,7 @@
         <v>9</v>
       </c>
       <c r="E370">
-        <v>0.33</v>
+        <v>0.23</v>
       </c>
       <c r="F370" t="s">
         <v>35</v>
@@ -10751,7 +10801,7 @@
         <v>9</v>
       </c>
       <c r="E371">
-        <v>0.39</v>
+        <v>0.15</v>
       </c>
       <c r="F371" t="s">
         <v>35</v>
@@ -10771,7 +10821,7 @@
         <v>9</v>
       </c>
       <c r="E372">
-        <v>0.11</v>
+        <v>0.23</v>
       </c>
       <c r="F372" t="s">
         <v>35</v>
@@ -10791,7 +10841,7 @@
         <v>9</v>
       </c>
       <c r="E373">
-        <v>0.27</v>
+        <v>0.1</v>
       </c>
       <c r="F373" t="s">
         <v>35</v>
@@ -10811,7 +10861,7 @@
         <v>9</v>
       </c>
       <c r="E374">
-        <v>0.11</v>
+        <v>0.23</v>
       </c>
       <c r="F374" t="s">
         <v>60</v>
@@ -10851,7 +10901,7 @@
         <v>9</v>
       </c>
       <c r="E376">
-        <v>0.23</v>
+        <v>0.38</v>
       </c>
       <c r="F376" t="s">
         <v>60</v>
@@ -10871,7 +10921,7 @@
         <v>9</v>
       </c>
       <c r="E377">
-        <v>0.13</v>
+        <v>0.31</v>
       </c>
       <c r="F377" t="s">
         <v>60</v>
@@ -10891,7 +10941,7 @@
         <v>9</v>
       </c>
       <c r="E378">
-        <v>0.13</v>
+        <v>0.35</v>
       </c>
       <c r="F378" t="s">
         <v>60</v>
@@ -10911,7 +10961,7 @@
         <v>9</v>
       </c>
       <c r="E379">
-        <v>0.34</v>
+        <v>0.13</v>
       </c>
       <c r="F379" t="s">
         <v>60</v>
@@ -10931,7 +10981,7 @@
         <v>9</v>
       </c>
       <c r="E380">
-        <v>0.38</v>
+        <v>0.33</v>
       </c>
       <c r="F380" t="s">
         <v>60</v>
@@ -10951,7 +11001,7 @@
         <v>9</v>
       </c>
       <c r="E381">
-        <v>0.27</v>
+        <v>0.32</v>
       </c>
       <c r="F381" t="s">
         <v>60</v>
@@ -10971,7 +11021,7 @@
         <v>9</v>
       </c>
       <c r="E382">
-        <v>0.24</v>
+        <v>0.11</v>
       </c>
       <c r="F382" t="s">
         <v>10</v>
@@ -10991,7 +11041,7 @@
         <v>9</v>
       </c>
       <c r="E383">
-        <v>0.15</v>
+        <v>0.18</v>
       </c>
       <c r="F383" t="s">
         <v>10</v>
@@ -11011,7 +11061,7 @@
         <v>9</v>
       </c>
       <c r="E384">
-        <v>0.37</v>
+        <v>0.3</v>
       </c>
       <c r="F384" t="s">
         <v>10</v>
@@ -11031,7 +11081,7 @@
         <v>9</v>
       </c>
       <c r="E385">
-        <v>0.23</v>
+        <v>0.25</v>
       </c>
       <c r="F385" t="s">
         <v>10</v>
@@ -11051,7 +11101,7 @@
         <v>9</v>
       </c>
       <c r="E386">
-        <v>0.19</v>
+        <v>0.35</v>
       </c>
       <c r="F386" t="s">
         <v>10</v>
@@ -11071,7 +11121,7 @@
         <v>9</v>
       </c>
       <c r="E387">
-        <v>0.3</v>
+        <v>0.32</v>
       </c>
       <c r="F387" t="s">
         <v>10</v>
@@ -11091,7 +11141,7 @@
         <v>9</v>
       </c>
       <c r="E388">
-        <v>0.37</v>
+        <v>0.21</v>
       </c>
       <c r="F388" t="s">
         <v>35</v>
@@ -11111,7 +11161,7 @@
         <v>9</v>
       </c>
       <c r="E389">
-        <v>0.23</v>
+        <v>0.16</v>
       </c>
       <c r="F389" t="s">
         <v>35</v>
@@ -11131,7 +11181,7 @@
         <v>9</v>
       </c>
       <c r="E390">
-        <v>0.3</v>
+        <v>0.12</v>
       </c>
       <c r="F390" t="s">
         <v>35</v>
@@ -11151,7 +11201,7 @@
         <v>9</v>
       </c>
       <c r="E391">
-        <v>0.38</v>
+        <v>0.18</v>
       </c>
       <c r="F391" t="s">
         <v>35</v>
@@ -11171,7 +11221,7 @@
         <v>9</v>
       </c>
       <c r="E392">
-        <v>0.25</v>
+        <v>0.22</v>
       </c>
       <c r="F392" t="s">
         <v>35</v>
@@ -11191,7 +11241,7 @@
         <v>9</v>
       </c>
       <c r="E393">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="F393" t="s">
         <v>35</v>
@@ -11211,7 +11261,7 @@
         <v>9</v>
       </c>
       <c r="E394">
-        <v>0.15</v>
+        <v>0.31</v>
       </c>
       <c r="F394" t="s">
         <v>60</v>
@@ -11231,7 +11281,7 @@
         <v>9</v>
       </c>
       <c r="E395">
-        <v>0.13</v>
+        <v>0.2</v>
       </c>
       <c r="F395" t="s">
         <v>60</v>
@@ -11251,7 +11301,7 @@
         <v>9</v>
       </c>
       <c r="E396">
-        <v>0.35</v>
+        <v>0.15</v>
       </c>
       <c r="F396" t="s">
         <v>60</v>
@@ -11271,7 +11321,7 @@
         <v>9</v>
       </c>
       <c r="E397">
-        <v>0.21</v>
+        <v>0.19</v>
       </c>
       <c r="F397" t="s">
         <v>60</v>
@@ -11291,7 +11341,7 @@
         <v>9</v>
       </c>
       <c r="E398">
-        <v>0.38</v>
+        <v>0.23</v>
       </c>
       <c r="F398" t="s">
         <v>60</v>
@@ -11311,7 +11361,7 @@
         <v>9</v>
       </c>
       <c r="E399">
-        <v>0.17</v>
+        <v>0.39</v>
       </c>
       <c r="F399" t="s">
         <v>60</v>
@@ -11331,7 +11381,7 @@
         <v>9</v>
       </c>
       <c r="E400">
-        <v>0.28</v>
+        <v>0.35</v>
       </c>
       <c r="F400" t="s">
         <v>60</v>
@@ -11351,7 +11401,7 @@
         <v>9</v>
       </c>
       <c r="E401">
-        <v>0.16</v>
+        <v>0.21</v>
       </c>
       <c r="F401" t="s">
         <v>60</v>
@@ -11371,7 +11421,7 @@
         <v>9</v>
       </c>
       <c r="E402">
-        <v>0.4</v>
+        <v>0.34</v>
       </c>
       <c r="F402" t="s">
         <v>10</v>
@@ -11391,7 +11441,7 @@
         <v>9</v>
       </c>
       <c r="E403">
-        <v>0.26</v>
+        <v>0.23</v>
       </c>
       <c r="F403" t="s">
         <v>10</v>
@@ -11411,7 +11461,7 @@
         <v>9</v>
       </c>
       <c r="E404">
-        <v>0.18</v>
+        <v>0.11</v>
       </c>
       <c r="F404" t="s">
         <v>10</v>
@@ -11431,7 +11481,7 @@
         <v>9</v>
       </c>
       <c r="E405">
-        <v>0.3</v>
+        <v>0.39</v>
       </c>
       <c r="F405" t="s">
         <v>10</v>
@@ -11451,7 +11501,7 @@
         <v>9</v>
       </c>
       <c r="E406">
-        <v>0.37</v>
+        <v>0.36</v>
       </c>
       <c r="F406" t="s">
         <v>10</v>
@@ -11471,7 +11521,7 @@
         <v>9</v>
       </c>
       <c r="E407">
-        <v>0.19</v>
+        <v>0.23</v>
       </c>
       <c r="F407" t="s">
         <v>10</v>
@@ -11491,7 +11541,7 @@
         <v>9</v>
       </c>
       <c r="E408">
-        <v>0.35</v>
+        <v>0.26</v>
       </c>
       <c r="F408" t="s">
         <v>35</v>
@@ -11511,7 +11561,7 @@
         <v>9</v>
       </c>
       <c r="E409">
-        <v>0.34</v>
+        <v>0.3</v>
       </c>
       <c r="F409" t="s">
         <v>35</v>
@@ -11531,7 +11581,7 @@
         <v>9</v>
       </c>
       <c r="E410">
-        <v>0.15</v>
+        <v>0.32</v>
       </c>
       <c r="F410" t="s">
         <v>35</v>
@@ -11551,7 +11601,7 @@
         <v>9</v>
       </c>
       <c r="E411">
-        <v>0.11</v>
+        <v>0.22</v>
       </c>
       <c r="F411" t="s">
         <v>35</v>
@@ -11571,7 +11621,7 @@
         <v>9</v>
       </c>
       <c r="E412">
-        <v>0.28</v>
+        <v>0.27</v>
       </c>
       <c r="F412" t="s">
         <v>35</v>
@@ -11591,7 +11641,7 @@
         <v>9</v>
       </c>
       <c r="E413">
-        <v>0.31</v>
+        <v>0.21</v>
       </c>
       <c r="F413" t="s">
         <v>35</v>
@@ -11611,7 +11661,7 @@
         <v>9</v>
       </c>
       <c r="E414">
-        <v>0.35</v>
+        <v>0.28</v>
       </c>
       <c r="F414" t="s">
         <v>60</v>
@@ -11631,7 +11681,7 @@
         <v>9</v>
       </c>
       <c r="E415">
-        <v>0.23</v>
+        <v>0.11</v>
       </c>
       <c r="F415" t="s">
         <v>60</v>
@@ -11651,7 +11701,7 @@
         <v>9</v>
       </c>
       <c r="E416">
-        <v>0.11</v>
+        <v>0.13</v>
       </c>
       <c r="F416" t="s">
         <v>60</v>
@@ -11671,7 +11721,7 @@
         <v>9</v>
       </c>
       <c r="E417">
-        <v>0.2</v>
+        <v>0.21</v>
       </c>
       <c r="F417" t="s">
         <v>60</v>
@@ -11691,7 +11741,7 @@
         <v>9</v>
       </c>
       <c r="E418">
-        <v>0.27</v>
+        <v>0.36</v>
       </c>
       <c r="F418" t="s">
         <v>60</v>
@@ -11711,7 +11761,7 @@
         <v>9</v>
       </c>
       <c r="E419">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="F419" t="s">
         <v>60</v>
@@ -11731,7 +11781,7 @@
         <v>9</v>
       </c>
       <c r="E420">
-        <v>0.27</v>
+        <v>0.38</v>
       </c>
       <c r="F420" t="s">
         <v>60</v>
@@ -11751,7 +11801,7 @@
         <v>9</v>
       </c>
       <c r="E421">
-        <v>0.28</v>
+        <v>0.13</v>
       </c>
       <c r="F421" t="s">
         <v>60</v>
@@ -11771,7 +11821,7 @@
         <v>9</v>
       </c>
       <c r="E422">
-        <v>0.31</v>
+        <v>0.21</v>
       </c>
       <c r="F422" t="s">
         <v>10</v>
@@ -11791,7 +11841,7 @@
         <v>9</v>
       </c>
       <c r="E423">
-        <v>0.11</v>
+        <v>0.13</v>
       </c>
       <c r="F423" t="s">
         <v>10</v>
@@ -11811,7 +11861,7 @@
         <v>9</v>
       </c>
       <c r="E424">
-        <v>0.32</v>
+        <v>0.39</v>
       </c>
       <c r="F424" t="s">
         <v>10</v>
@@ -11831,7 +11881,7 @@
         <v>9</v>
       </c>
       <c r="E425">
-        <v>0.18</v>
+        <v>0.39</v>
       </c>
       <c r="F425" t="s">
         <v>10</v>
@@ -11851,7 +11901,7 @@
         <v>9</v>
       </c>
       <c r="E426">
-        <v>0.35</v>
+        <v>0.22</v>
       </c>
       <c r="F426" t="s">
         <v>10</v>
@@ -11871,7 +11921,7 @@
         <v>9</v>
       </c>
       <c r="E427">
-        <v>0.23</v>
+        <v>0.28</v>
       </c>
       <c r="F427" t="s">
         <v>10</v>
@@ -11911,7 +11961,7 @@
         <v>9</v>
       </c>
       <c r="E429">
-        <v>0.34</v>
+        <v>0.2</v>
       </c>
       <c r="F429" t="s">
         <v>10</v>
@@ -11931,7 +11981,7 @@
         <v>9</v>
       </c>
       <c r="E430">
-        <v>0.38</v>
+        <v>0.13</v>
       </c>
       <c r="F430" t="s">
         <v>10</v>
@@ -11951,7 +12001,7 @@
         <v>9</v>
       </c>
       <c r="E431">
-        <v>0.38</v>
+        <v>0.13</v>
       </c>
       <c r="F431" t="s">
         <v>10</v>
@@ -11971,7 +12021,7 @@
         <v>9</v>
       </c>
       <c r="E432">
-        <v>0.33</v>
+        <v>0.25</v>
       </c>
       <c r="F432" t="s">
         <v>10</v>
@@ -12011,7 +12061,7 @@
         <v>9</v>
       </c>
       <c r="E434">
-        <v>0.18</v>
+        <v>0.13</v>
       </c>
       <c r="F434" t="s">
         <v>10</v>
@@ -12031,7 +12081,7 @@
         <v>9</v>
       </c>
       <c r="E435">
-        <v>0.37</v>
+        <v>0.18</v>
       </c>
       <c r="F435" t="s">
         <v>10</v>
@@ -12051,7 +12101,7 @@
         <v>9</v>
       </c>
       <c r="E436">
-        <v>0.36</v>
+        <v>0.31</v>
       </c>
       <c r="F436" t="s">
         <v>10</v>
@@ -12071,7 +12121,7 @@
         <v>9</v>
       </c>
       <c r="E437">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="F437" t="s">
         <v>35</v>
@@ -12091,7 +12141,7 @@
         <v>9</v>
       </c>
       <c r="E438">
-        <v>0.33</v>
+        <v>0.17</v>
       </c>
       <c r="F438" t="s">
         <v>35</v>
@@ -12111,7 +12161,7 @@
         <v>9</v>
       </c>
       <c r="E439">
-        <v>0.26</v>
+        <v>0.34</v>
       </c>
       <c r="F439" t="s">
         <v>35</v>
@@ -12131,7 +12181,7 @@
         <v>9</v>
       </c>
       <c r="E440">
-        <v>0.37</v>
+        <v>0.22</v>
       </c>
       <c r="F440" t="s">
         <v>35</v>
@@ -12151,7 +12201,7 @@
         <v>9</v>
       </c>
       <c r="E441">
-        <v>0.39</v>
+        <v>0.38</v>
       </c>
       <c r="F441" t="s">
         <v>35</v>
@@ -12171,7 +12221,7 @@
         <v>9</v>
       </c>
       <c r="E442">
-        <v>0.31</v>
+        <v>0.22</v>
       </c>
       <c r="F442" t="s">
         <v>35</v>
@@ -12191,7 +12241,7 @@
         <v>9</v>
       </c>
       <c r="E443">
-        <v>0.29</v>
+        <v>0.13</v>
       </c>
       <c r="F443" t="s">
         <v>35</v>
@@ -12211,7 +12261,7 @@
         <v>9</v>
       </c>
       <c r="E444">
-        <v>0.21</v>
+        <v>0.32</v>
       </c>
       <c r="F444" t="s">
         <v>35</v>
@@ -12231,7 +12281,7 @@
         <v>9</v>
       </c>
       <c r="E445">
-        <v>0.21</v>
+        <v>0.12</v>
       </c>
       <c r="F445" t="s">
         <v>35</v>
@@ -12251,7 +12301,7 @@
         <v>9</v>
       </c>
       <c r="E446">
-        <v>0.11</v>
+        <v>0.15</v>
       </c>
       <c r="F446" t="s">
         <v>35</v>
@@ -12271,7 +12321,7 @@
         <v>9</v>
       </c>
       <c r="E447">
-        <v>0.21</v>
+        <v>0.2</v>
       </c>
       <c r="F447" t="s">
         <v>35</v>
@@ -12291,7 +12341,7 @@
         <v>9</v>
       </c>
       <c r="E448">
-        <v>0.38</v>
+        <v>0.22</v>
       </c>
       <c r="F448" t="s">
         <v>35</v>
@@ -12311,7 +12361,7 @@
         <v>9</v>
       </c>
       <c r="E449">
-        <v>0.18</v>
+        <v>0.37</v>
       </c>
       <c r="F449" t="s">
         <v>35</v>
@@ -12331,7 +12381,7 @@
         <v>9</v>
       </c>
       <c r="E450">
-        <v>0.22</v>
+        <v>0.27</v>
       </c>
       <c r="F450" t="s">
         <v>35</v>
@@ -12351,7 +12401,7 @@
         <v>9</v>
       </c>
       <c r="E451">
-        <v>0.22</v>
+        <v>0.3</v>
       </c>
       <c r="F451" t="s">
         <v>35</v>
@@ -12371,7 +12421,7 @@
         <v>9</v>
       </c>
       <c r="E452">
-        <v>0.17</v>
+        <v>0.39</v>
       </c>
       <c r="F452" t="s">
         <v>60</v>
@@ -12391,7 +12441,7 @@
         <v>9</v>
       </c>
       <c r="E453">
-        <v>0.36</v>
+        <v>0.13</v>
       </c>
       <c r="F453" t="s">
         <v>60</v>
@@ -12411,7 +12461,7 @@
         <v>9</v>
       </c>
       <c r="E454">
-        <v>0.12</v>
+        <v>0.18</v>
       </c>
       <c r="F454" t="s">
         <v>60</v>
@@ -12431,7 +12481,7 @@
         <v>9</v>
       </c>
       <c r="E455">
-        <v>0.13</v>
+        <v>0.3</v>
       </c>
       <c r="F455" t="s">
         <v>60</v>
@@ -12451,7 +12501,7 @@
         <v>9</v>
       </c>
       <c r="E456">
-        <v>0.25</v>
+        <v>0.16</v>
       </c>
       <c r="F456" t="s">
         <v>60</v>
@@ -12471,7 +12521,7 @@
         <v>9</v>
       </c>
       <c r="E457">
-        <v>0.35</v>
+        <v>0.31</v>
       </c>
       <c r="F457" t="s">
         <v>60</v>
@@ -12491,7 +12541,7 @@
         <v>9</v>
       </c>
       <c r="E458">
-        <v>0.22</v>
+        <v>0.28</v>
       </c>
       <c r="F458" t="s">
         <v>60</v>
@@ -12511,7 +12561,7 @@
         <v>9</v>
       </c>
       <c r="E459">
-        <v>0.3</v>
+        <v>0.19</v>
       </c>
       <c r="F459" t="s">
         <v>60</v>
@@ -12531,7 +12581,7 @@
         <v>9</v>
       </c>
       <c r="E460">
-        <v>0.2</v>
+        <v>0.39</v>
       </c>
       <c r="F460" t="s">
         <v>60</v>
@@ -12551,7 +12601,7 @@
         <v>9</v>
       </c>
       <c r="E461">
-        <v>0.19</v>
+        <v>0.29</v>
       </c>
       <c r="F461" t="s">
         <v>60</v>
@@ -12571,7 +12621,7 @@
         <v>9</v>
       </c>
       <c r="E462">
-        <v>0.18</v>
+        <v>0.39</v>
       </c>
       <c r="F462" t="s">
         <v>60</v>
@@ -12591,7 +12641,7 @@
         <v>9</v>
       </c>
       <c r="E463">
-        <v>0.11</v>
+        <v>0.14</v>
       </c>
       <c r="F463" t="s">
         <v>60</v>
@@ -12611,7 +12661,7 @@
         <v>9</v>
       </c>
       <c r="E464">
-        <v>0.27</v>
+        <v>0.18</v>
       </c>
       <c r="F464" t="s">
         <v>60</v>
@@ -12631,7 +12681,7 @@
         <v>9</v>
       </c>
       <c r="E465">
-        <v>0.14</v>
+        <v>0.39</v>
       </c>
       <c r="F465" t="s">
         <v>60</v>
@@ -12651,7 +12701,7 @@
         <v>9</v>
       </c>
       <c r="E466">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="F466" t="s">
         <v>60</v>
@@ -12691,7 +12741,7 @@
         <v>9</v>
       </c>
       <c r="E468">
-        <v>0.29</v>
+        <v>0.33</v>
       </c>
       <c r="F468" t="s">
         <v>60</v>
@@ -12711,7 +12761,7 @@
         <v>9</v>
       </c>
       <c r="E469">
-        <v>0.22</v>
+        <v>0.27</v>
       </c>
       <c r="F469" t="s">
         <v>60</v>
@@ -12731,7 +12781,7 @@
         <v>9</v>
       </c>
       <c r="E470">
-        <v>0.36</v>
+        <v>0.37</v>
       </c>
       <c r="F470" t="s">
         <v>60</v>
@@ -12751,7 +12801,7 @@
         <v>9</v>
       </c>
       <c r="E471">
-        <v>0.37</v>
+        <v>0.21</v>
       </c>
       <c r="F471" t="s">
         <v>60</v>
@@ -12768,20 +12818,23 @@
   <dimension ref="A1:D471"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="4" width="25" customWidth="1"/>
+    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="2" max="2" width="25" customWidth="1"/>
+    <col min="3" max="3" width="45" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
     </row>
@@ -19373,24 +19426,41 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="4" width="25" customWidth="1"/>
+    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="2" max="2" width="25" customWidth="1"/>
+    <col min="3" max="3" width="45" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>964</v>
+      </c>
+      <c r="B2" t="s">
+        <v>965</v>
+      </c>
+      <c r="C2" t="s">
+        <v>966</v>
+      </c>
+      <c r="D2" t="s">
+        <v>967</v>
       </c>
     </row>
   </sheetData>
@@ -19401,24 +19471,41 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="4" width="25" customWidth="1"/>
+    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="2" max="2" width="25" customWidth="1"/>
+    <col min="3" max="3" width="45" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>964</v>
+      </c>
+      <c r="B2" t="s">
+        <v>965</v>
+      </c>
+      <c r="C2" t="s">
+        <v>968</v>
+      </c>
+      <c r="D2" t="s">
+        <v>967</v>
       </c>
     </row>
   </sheetData>
@@ -19432,20 +19519,20 @@
   <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="2" width="25" customWidth="1"/>
+    <col min="1" max="2" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>964</v>
-      </c>
-      <c r="B1" t="s">
-        <v>965</v>
+    <row r="1" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
+        <v>969</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>970</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>966</v>
+        <v>971</v>
       </c>
       <c r="B2">
         <v>470</v>
@@ -19453,7 +19540,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>967</v>
+        <v>972</v>
       </c>
       <c r="B3">
         <v>470</v>
@@ -19461,7 +19548,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>968</v>
+        <v>973</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -19469,10 +19556,10 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>969</v>
+        <v>974</v>
       </c>
       <c r="B5" t="s">
-        <v>970</v>
+        <v>975</v>
       </c>
     </row>
   </sheetData>
@@ -19483,24 +19570,40 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="4" width="25" customWidth="1"/>
+    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="2" max="3" width="25" customWidth="1"/>
+    <col min="4" max="4" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>971</v>
-      </c>
-      <c r="B1" t="s">
+    <row r="1" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>976</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D1" t="s">
-        <v>972</v>
+      <c r="D1" s="4" t="s">
+        <v>977</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>978</v>
+      </c>
+      <c r="B2" t="s">
+        <v>964</v>
+      </c>
+      <c r="C2" t="s">
+        <v>965</v>
+      </c>
+      <c r="D2" t="s">
+        <v>979</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix IDE Office Viewer compatibility for Passed_Test_Cases.xlsx
</commit_message>
<xml_diff>
--- a/Test Results/Excel/Automation_Test_Report.xlsx
+++ b/Test Results/Excel/Automation_Test_Report.xlsx
@@ -3421,7 +3421,7 @@
         <v>9</v>
       </c>
       <c r="E2">
-        <v>0.39</v>
+        <v>0.25</v>
       </c>
       <c r="F2" t="s">
         <v>10</v>
@@ -3441,7 +3441,7 @@
         <v>9</v>
       </c>
       <c r="E3">
-        <v>0.28</v>
+        <v>0.22</v>
       </c>
       <c r="F3" t="s">
         <v>10</v>
@@ -3481,7 +3481,7 @@
         <v>9</v>
       </c>
       <c r="E5">
-        <v>0.14</v>
+        <v>0.23</v>
       </c>
       <c r="F5" t="s">
         <v>10</v>
@@ -3501,7 +3501,7 @@
         <v>9</v>
       </c>
       <c r="E6">
-        <v>0.36</v>
+        <v>0.13</v>
       </c>
       <c r="F6" t="s">
         <v>10</v>
@@ -3521,7 +3521,7 @@
         <v>9</v>
       </c>
       <c r="E7">
-        <v>0.11</v>
+        <v>0.23</v>
       </c>
       <c r="F7" t="s">
         <v>10</v>
@@ -3541,7 +3541,7 @@
         <v>9</v>
       </c>
       <c r="E8">
-        <v>0.31</v>
+        <v>0.38</v>
       </c>
       <c r="F8" t="s">
         <v>10</v>
@@ -3561,7 +3561,7 @@
         <v>9</v>
       </c>
       <c r="E9">
-        <v>0.12</v>
+        <v>0.22</v>
       </c>
       <c r="F9" t="s">
         <v>10</v>
@@ -3581,7 +3581,7 @@
         <v>9</v>
       </c>
       <c r="E10">
-        <v>0.4</v>
+        <v>0.35</v>
       </c>
       <c r="F10" t="s">
         <v>10</v>
@@ -3601,7 +3601,7 @@
         <v>9</v>
       </c>
       <c r="E11">
-        <v>0.3</v>
+        <v>0.15</v>
       </c>
       <c r="F11" t="s">
         <v>10</v>
@@ -3621,7 +3621,7 @@
         <v>9</v>
       </c>
       <c r="E12">
-        <v>0.14</v>
+        <v>0.22</v>
       </c>
       <c r="F12" t="s">
         <v>10</v>
@@ -3641,7 +3641,7 @@
         <v>9</v>
       </c>
       <c r="E13">
-        <v>0.32</v>
+        <v>0.28</v>
       </c>
       <c r="F13" t="s">
         <v>10</v>
@@ -3661,7 +3661,7 @@
         <v>9</v>
       </c>
       <c r="E14">
-        <v>0.28</v>
+        <v>0.15</v>
       </c>
       <c r="F14" t="s">
         <v>35</v>
@@ -3681,7 +3681,7 @@
         <v>9</v>
       </c>
       <c r="E15">
-        <v>0.32</v>
+        <v>0.18</v>
       </c>
       <c r="F15" t="s">
         <v>35</v>
@@ -3701,7 +3701,7 @@
         <v>9</v>
       </c>
       <c r="E16">
-        <v>0.12</v>
+        <v>0.4</v>
       </c>
       <c r="F16" t="s">
         <v>35</v>
@@ -3721,7 +3721,7 @@
         <v>9</v>
       </c>
       <c r="E17">
-        <v>0.36</v>
+        <v>0.1</v>
       </c>
       <c r="F17" t="s">
         <v>35</v>
@@ -3741,7 +3741,7 @@
         <v>9</v>
       </c>
       <c r="E18">
-        <v>0.37</v>
+        <v>0.34</v>
       </c>
       <c r="F18" t="s">
         <v>35</v>
@@ -3761,7 +3761,7 @@
         <v>9</v>
       </c>
       <c r="E19">
-        <v>0.17</v>
+        <v>0.18</v>
       </c>
       <c r="F19" t="s">
         <v>35</v>
@@ -3781,7 +3781,7 @@
         <v>9</v>
       </c>
       <c r="E20">
-        <v>0.27</v>
+        <v>0.13</v>
       </c>
       <c r="F20" t="s">
         <v>35</v>
@@ -3801,7 +3801,7 @@
         <v>9</v>
       </c>
       <c r="E21">
-        <v>0.35</v>
+        <v>0.23</v>
       </c>
       <c r="F21" t="s">
         <v>35</v>
@@ -3821,7 +3821,7 @@
         <v>9</v>
       </c>
       <c r="E22">
-        <v>0.34</v>
+        <v>0.12</v>
       </c>
       <c r="F22" t="s">
         <v>35</v>
@@ -3841,7 +3841,7 @@
         <v>9</v>
       </c>
       <c r="E23">
-        <v>0.18</v>
+        <v>0.34</v>
       </c>
       <c r="F23" t="s">
         <v>35</v>
@@ -3861,7 +3861,7 @@
         <v>9</v>
       </c>
       <c r="E24">
-        <v>0.39</v>
+        <v>0.12</v>
       </c>
       <c r="F24" t="s">
         <v>35</v>
@@ -3881,7 +3881,7 @@
         <v>9</v>
       </c>
       <c r="E25">
-        <v>0.28</v>
+        <v>0.38</v>
       </c>
       <c r="F25" t="s">
         <v>35</v>
@@ -3901,7 +3901,7 @@
         <v>9</v>
       </c>
       <c r="E26">
-        <v>0.37</v>
+        <v>0.22</v>
       </c>
       <c r="F26" t="s">
         <v>60</v>
@@ -3921,7 +3921,7 @@
         <v>9</v>
       </c>
       <c r="E27">
-        <v>0.23</v>
+        <v>0.12</v>
       </c>
       <c r="F27" t="s">
         <v>60</v>
@@ -3941,7 +3941,7 @@
         <v>9</v>
       </c>
       <c r="E28">
-        <v>0.11</v>
+        <v>0.37</v>
       </c>
       <c r="F28" t="s">
         <v>60</v>
@@ -3981,7 +3981,7 @@
         <v>9</v>
       </c>
       <c r="E30">
-        <v>0.25</v>
+        <v>0.2</v>
       </c>
       <c r="F30" t="s">
         <v>60</v>
@@ -4001,7 +4001,7 @@
         <v>9</v>
       </c>
       <c r="E31">
-        <v>0.39</v>
+        <v>0.13</v>
       </c>
       <c r="F31" t="s">
         <v>60</v>
@@ -4021,7 +4021,7 @@
         <v>9</v>
       </c>
       <c r="E32">
-        <v>0.25</v>
+        <v>0.22</v>
       </c>
       <c r="F32" t="s">
         <v>60</v>
@@ -4041,7 +4041,7 @@
         <v>9</v>
       </c>
       <c r="E33">
-        <v>0.3</v>
+        <v>0.26</v>
       </c>
       <c r="F33" t="s">
         <v>60</v>
@@ -4061,7 +4061,7 @@
         <v>9</v>
       </c>
       <c r="E34">
-        <v>0.2</v>
+        <v>0.16</v>
       </c>
       <c r="F34" t="s">
         <v>60</v>
@@ -4081,7 +4081,7 @@
         <v>9</v>
       </c>
       <c r="E35">
-        <v>0.31</v>
+        <v>0.2</v>
       </c>
       <c r="F35" t="s">
         <v>60</v>
@@ -4101,7 +4101,7 @@
         <v>9</v>
       </c>
       <c r="E36">
-        <v>0.38</v>
+        <v>0.21</v>
       </c>
       <c r="F36" t="s">
         <v>60</v>
@@ -4121,7 +4121,7 @@
         <v>9</v>
       </c>
       <c r="E37">
-        <v>0.24</v>
+        <v>0.2</v>
       </c>
       <c r="F37" t="s">
         <v>60</v>
@@ -4141,7 +4141,7 @@
         <v>9</v>
       </c>
       <c r="E38">
-        <v>0.21</v>
+        <v>0.14</v>
       </c>
       <c r="F38" t="s">
         <v>60</v>
@@ -4181,7 +4181,7 @@
         <v>9</v>
       </c>
       <c r="E40">
-        <v>0.14</v>
+        <v>0.32</v>
       </c>
       <c r="F40" t="s">
         <v>60</v>
@@ -4201,7 +4201,7 @@
         <v>9</v>
       </c>
       <c r="E41">
-        <v>0.17</v>
+        <v>0.25</v>
       </c>
       <c r="F41" t="s">
         <v>60</v>
@@ -4221,7 +4221,7 @@
         <v>9</v>
       </c>
       <c r="E42">
-        <v>0.25</v>
+        <v>0.12</v>
       </c>
       <c r="F42" t="s">
         <v>10</v>
@@ -4241,7 +4241,7 @@
         <v>9</v>
       </c>
       <c r="E43">
-        <v>0.28</v>
+        <v>0.12</v>
       </c>
       <c r="F43" t="s">
         <v>10</v>
@@ -4281,7 +4281,7 @@
         <v>9</v>
       </c>
       <c r="E45">
-        <v>0.39</v>
+        <v>0.16</v>
       </c>
       <c r="F45" t="s">
         <v>10</v>
@@ -4301,7 +4301,7 @@
         <v>9</v>
       </c>
       <c r="E46">
-        <v>0.39</v>
+        <v>0.13</v>
       </c>
       <c r="F46" t="s">
         <v>10</v>
@@ -4321,7 +4321,7 @@
         <v>9</v>
       </c>
       <c r="E47">
-        <v>0.2</v>
+        <v>0.24</v>
       </c>
       <c r="F47" t="s">
         <v>10</v>
@@ -4341,7 +4341,7 @@
         <v>9</v>
       </c>
       <c r="E48">
-        <v>0.23</v>
+        <v>0.27</v>
       </c>
       <c r="F48" t="s">
         <v>10</v>
@@ -4361,7 +4361,7 @@
         <v>9</v>
       </c>
       <c r="E49">
-        <v>0.23</v>
+        <v>0.38</v>
       </c>
       <c r="F49" t="s">
         <v>10</v>
@@ -4381,7 +4381,7 @@
         <v>9</v>
       </c>
       <c r="E50">
-        <v>0.18</v>
+        <v>0.17</v>
       </c>
       <c r="F50" t="s">
         <v>10</v>
@@ -4401,7 +4401,7 @@
         <v>9</v>
       </c>
       <c r="E51">
-        <v>0.16</v>
+        <v>0.22</v>
       </c>
       <c r="F51" t="s">
         <v>10</v>
@@ -4421,7 +4421,7 @@
         <v>9</v>
       </c>
       <c r="E52">
-        <v>0.37</v>
+        <v>0.32</v>
       </c>
       <c r="F52" t="s">
         <v>10</v>
@@ -4441,7 +4441,7 @@
         <v>9</v>
       </c>
       <c r="E53">
-        <v>0.27</v>
+        <v>0.22</v>
       </c>
       <c r="F53" t="s">
         <v>10</v>
@@ -4461,7 +4461,7 @@
         <v>9</v>
       </c>
       <c r="E54">
-        <v>0.13</v>
+        <v>0.15</v>
       </c>
       <c r="F54" t="s">
         <v>35</v>
@@ -4481,7 +4481,7 @@
         <v>9</v>
       </c>
       <c r="E55">
-        <v>0.18</v>
+        <v>0.16</v>
       </c>
       <c r="F55" t="s">
         <v>35</v>
@@ -4501,7 +4501,7 @@
         <v>9</v>
       </c>
       <c r="E56">
-        <v>0.39</v>
+        <v>0.16</v>
       </c>
       <c r="F56" t="s">
         <v>35</v>
@@ -4521,7 +4521,7 @@
         <v>9</v>
       </c>
       <c r="E57">
-        <v>0.39</v>
+        <v>0.11</v>
       </c>
       <c r="F57" t="s">
         <v>35</v>
@@ -4541,7 +4541,7 @@
         <v>9</v>
       </c>
       <c r="E58">
-        <v>0.34</v>
+        <v>0.26</v>
       </c>
       <c r="F58" t="s">
         <v>35</v>
@@ -4561,7 +4561,7 @@
         <v>9</v>
       </c>
       <c r="E59">
-        <v>0.28</v>
+        <v>0.15</v>
       </c>
       <c r="F59" t="s">
         <v>35</v>
@@ -4581,7 +4581,7 @@
         <v>9</v>
       </c>
       <c r="E60">
-        <v>0.19</v>
+        <v>0.39</v>
       </c>
       <c r="F60" t="s">
         <v>35</v>
@@ -4601,7 +4601,7 @@
         <v>9</v>
       </c>
       <c r="E61">
-        <v>0.13</v>
+        <v>0.33</v>
       </c>
       <c r="F61" t="s">
         <v>35</v>
@@ -4621,7 +4621,7 @@
         <v>9</v>
       </c>
       <c r="E62">
-        <v>0.24</v>
+        <v>0.27</v>
       </c>
       <c r="F62" t="s">
         <v>35</v>
@@ -4641,7 +4641,7 @@
         <v>9</v>
       </c>
       <c r="E63">
-        <v>0.23</v>
+        <v>0.35</v>
       </c>
       <c r="F63" t="s">
         <v>35</v>
@@ -4681,7 +4681,7 @@
         <v>9</v>
       </c>
       <c r="E65">
-        <v>0.39</v>
+        <v>0.19</v>
       </c>
       <c r="F65" t="s">
         <v>35</v>
@@ -4701,7 +4701,7 @@
         <v>9</v>
       </c>
       <c r="E66">
-        <v>0.13</v>
+        <v>0.39</v>
       </c>
       <c r="F66" t="s">
         <v>60</v>
@@ -4721,7 +4721,7 @@
         <v>9</v>
       </c>
       <c r="E67">
-        <v>0.24</v>
+        <v>0.15</v>
       </c>
       <c r="F67" t="s">
         <v>60</v>
@@ -4741,7 +4741,7 @@
         <v>9</v>
       </c>
       <c r="E68">
-        <v>0.19</v>
+        <v>0.15</v>
       </c>
       <c r="F68" t="s">
         <v>60</v>
@@ -4761,7 +4761,7 @@
         <v>9</v>
       </c>
       <c r="E69">
-        <v>0.39</v>
+        <v>0.11</v>
       </c>
       <c r="F69" t="s">
         <v>60</v>
@@ -4781,7 +4781,7 @@
         <v>9</v>
       </c>
       <c r="E70">
-        <v>0.38</v>
+        <v>0.31</v>
       </c>
       <c r="F70" t="s">
         <v>60</v>
@@ -4821,7 +4821,7 @@
         <v>9</v>
       </c>
       <c r="E72">
-        <v>0.17</v>
+        <v>0.15</v>
       </c>
       <c r="F72" t="s">
         <v>60</v>
@@ -4841,7 +4841,7 @@
         <v>9</v>
       </c>
       <c r="E73">
-        <v>0.3</v>
+        <v>0.29</v>
       </c>
       <c r="F73" t="s">
         <v>60</v>
@@ -4861,7 +4861,7 @@
         <v>9</v>
       </c>
       <c r="E74">
-        <v>0.16</v>
+        <v>0.15</v>
       </c>
       <c r="F74" t="s">
         <v>60</v>
@@ -4901,7 +4901,7 @@
         <v>9</v>
       </c>
       <c r="E76">
-        <v>0.12</v>
+        <v>0.17</v>
       </c>
       <c r="F76" t="s">
         <v>60</v>
@@ -4921,7 +4921,7 @@
         <v>9</v>
       </c>
       <c r="E77">
-        <v>0.22</v>
+        <v>0.33</v>
       </c>
       <c r="F77" t="s">
         <v>60</v>
@@ -4941,7 +4941,7 @@
         <v>9</v>
       </c>
       <c r="E78">
-        <v>0.25</v>
+        <v>0.38</v>
       </c>
       <c r="F78" t="s">
         <v>60</v>
@@ -4961,7 +4961,7 @@
         <v>9</v>
       </c>
       <c r="E79">
-        <v>0.38</v>
+        <v>0.16</v>
       </c>
       <c r="F79" t="s">
         <v>60</v>
@@ -4981,7 +4981,7 @@
         <v>9</v>
       </c>
       <c r="E80">
-        <v>0.26</v>
+        <v>0.16</v>
       </c>
       <c r="F80" t="s">
         <v>60</v>
@@ -5001,7 +5001,7 @@
         <v>9</v>
       </c>
       <c r="E81">
-        <v>0.15</v>
+        <v>0.36</v>
       </c>
       <c r="F81" t="s">
         <v>60</v>
@@ -5021,7 +5021,7 @@
         <v>9</v>
       </c>
       <c r="E82">
-        <v>0.21</v>
+        <v>0.3</v>
       </c>
       <c r="F82" t="s">
         <v>10</v>
@@ -5041,7 +5041,7 @@
         <v>9</v>
       </c>
       <c r="E83">
-        <v>0.31</v>
+        <v>0.17</v>
       </c>
       <c r="F83" t="s">
         <v>10</v>
@@ -5061,7 +5061,7 @@
         <v>9</v>
       </c>
       <c r="E84">
-        <v>0.22</v>
+        <v>0.2</v>
       </c>
       <c r="F84" t="s">
         <v>10</v>
@@ -5081,7 +5081,7 @@
         <v>9</v>
       </c>
       <c r="E85">
-        <v>0.37</v>
+        <v>0.18</v>
       </c>
       <c r="F85" t="s">
         <v>10</v>
@@ -5101,7 +5101,7 @@
         <v>9</v>
       </c>
       <c r="E86">
-        <v>0.25</v>
+        <v>0.36</v>
       </c>
       <c r="F86" t="s">
         <v>10</v>
@@ -5121,7 +5121,7 @@
         <v>9</v>
       </c>
       <c r="E87">
-        <v>0.3</v>
+        <v>0.24</v>
       </c>
       <c r="F87" t="s">
         <v>10</v>
@@ -5141,7 +5141,7 @@
         <v>9</v>
       </c>
       <c r="E88">
-        <v>0.37</v>
+        <v>0.12</v>
       </c>
       <c r="F88" t="s">
         <v>10</v>
@@ -5161,7 +5161,7 @@
         <v>9</v>
       </c>
       <c r="E89">
-        <v>0.21</v>
+        <v>0.31</v>
       </c>
       <c r="F89" t="s">
         <v>10</v>
@@ -5181,7 +5181,7 @@
         <v>9</v>
       </c>
       <c r="E90">
-        <v>0.36</v>
+        <v>0.35</v>
       </c>
       <c r="F90" t="s">
         <v>10</v>
@@ -5201,7 +5201,7 @@
         <v>9</v>
       </c>
       <c r="E91">
-        <v>0.13</v>
+        <v>0.11</v>
       </c>
       <c r="F91" t="s">
         <v>35</v>
@@ -5221,7 +5221,7 @@
         <v>9</v>
       </c>
       <c r="E92">
-        <v>0.16</v>
+        <v>0.26</v>
       </c>
       <c r="F92" t="s">
         <v>35</v>
@@ -5241,7 +5241,7 @@
         <v>9</v>
       </c>
       <c r="E93">
-        <v>0.24</v>
+        <v>0.18</v>
       </c>
       <c r="F93" t="s">
         <v>35</v>
@@ -5261,7 +5261,7 @@
         <v>9</v>
       </c>
       <c r="E94">
-        <v>0.23</v>
+        <v>0.37</v>
       </c>
       <c r="F94" t="s">
         <v>35</v>
@@ -5301,7 +5301,7 @@
         <v>9</v>
       </c>
       <c r="E96">
-        <v>0.14</v>
+        <v>0.25</v>
       </c>
       <c r="F96" t="s">
         <v>35</v>
@@ -5321,7 +5321,7 @@
         <v>9</v>
       </c>
       <c r="E97">
-        <v>0.25</v>
+        <v>0.31</v>
       </c>
       <c r="F97" t="s">
         <v>35</v>
@@ -5341,7 +5341,7 @@
         <v>9</v>
       </c>
       <c r="E98">
-        <v>0.2</v>
+        <v>0.15</v>
       </c>
       <c r="F98" t="s">
         <v>35</v>
@@ -5361,7 +5361,7 @@
         <v>9</v>
       </c>
       <c r="E99">
-        <v>0.4</v>
+        <v>0.33</v>
       </c>
       <c r="F99" t="s">
         <v>35</v>
@@ -5381,7 +5381,7 @@
         <v>9</v>
       </c>
       <c r="E100">
-        <v>0.25</v>
+        <v>0.37</v>
       </c>
       <c r="F100" t="s">
         <v>60</v>
@@ -5401,7 +5401,7 @@
         <v>9</v>
       </c>
       <c r="E101">
-        <v>0.36</v>
+        <v>0.28</v>
       </c>
       <c r="F101" t="s">
         <v>60</v>
@@ -5421,7 +5421,7 @@
         <v>9</v>
       </c>
       <c r="E102">
-        <v>0.2</v>
+        <v>0.17</v>
       </c>
       <c r="F102" t="s">
         <v>60</v>
@@ -5441,7 +5441,7 @@
         <v>9</v>
       </c>
       <c r="E103">
-        <v>0.21</v>
+        <v>0.39</v>
       </c>
       <c r="F103" t="s">
         <v>60</v>
@@ -5461,7 +5461,7 @@
         <v>9</v>
       </c>
       <c r="E104">
-        <v>0.26</v>
+        <v>0.25</v>
       </c>
       <c r="F104" t="s">
         <v>60</v>
@@ -5481,7 +5481,7 @@
         <v>9</v>
       </c>
       <c r="E105">
-        <v>0.13</v>
+        <v>0.11</v>
       </c>
       <c r="F105" t="s">
         <v>60</v>
@@ -5501,7 +5501,7 @@
         <v>9</v>
       </c>
       <c r="E106">
-        <v>0.39</v>
+        <v>0.31</v>
       </c>
       <c r="F106" t="s">
         <v>60</v>
@@ -5521,7 +5521,7 @@
         <v>9</v>
       </c>
       <c r="E107">
-        <v>0.32</v>
+        <v>0.12</v>
       </c>
       <c r="F107" t="s">
         <v>60</v>
@@ -5541,7 +5541,7 @@
         <v>9</v>
       </c>
       <c r="E108">
-        <v>0.19</v>
+        <v>0.25</v>
       </c>
       <c r="F108" t="s">
         <v>60</v>
@@ -5561,7 +5561,7 @@
         <v>9</v>
       </c>
       <c r="E109">
-        <v>0.32</v>
+        <v>0.34</v>
       </c>
       <c r="F109" t="s">
         <v>60</v>
@@ -5581,7 +5581,7 @@
         <v>9</v>
       </c>
       <c r="E110">
-        <v>0.24</v>
+        <v>0.38</v>
       </c>
       <c r="F110" t="s">
         <v>60</v>
@@ -5601,7 +5601,7 @@
         <v>9</v>
       </c>
       <c r="E111">
-        <v>0.12</v>
+        <v>0.18</v>
       </c>
       <c r="F111" t="s">
         <v>60</v>
@@ -5621,7 +5621,7 @@
         <v>9</v>
       </c>
       <c r="E112">
-        <v>0.34</v>
+        <v>0.37</v>
       </c>
       <c r="F112" t="s">
         <v>10</v>
@@ -5641,7 +5641,7 @@
         <v>9</v>
       </c>
       <c r="E113">
-        <v>0.14</v>
+        <v>0.23</v>
       </c>
       <c r="F113" t="s">
         <v>10</v>
@@ -5661,7 +5661,7 @@
         <v>9</v>
       </c>
       <c r="E114">
-        <v>0.25</v>
+        <v>0.31</v>
       </c>
       <c r="F114" t="s">
         <v>10</v>
@@ -5681,7 +5681,7 @@
         <v>9</v>
       </c>
       <c r="E115">
-        <v>0.18</v>
+        <v>0.22</v>
       </c>
       <c r="F115" t="s">
         <v>10</v>
@@ -5701,7 +5701,7 @@
         <v>9</v>
       </c>
       <c r="E116">
-        <v>0.19</v>
+        <v>0.23</v>
       </c>
       <c r="F116" t="s">
         <v>10</v>
@@ -5721,7 +5721,7 @@
         <v>9</v>
       </c>
       <c r="E117">
-        <v>0.14</v>
+        <v>0.33</v>
       </c>
       <c r="F117" t="s">
         <v>10</v>
@@ -5761,7 +5761,7 @@
         <v>9</v>
       </c>
       <c r="E119">
-        <v>0.24</v>
+        <v>0.37</v>
       </c>
       <c r="F119" t="s">
         <v>10</v>
@@ -5781,7 +5781,7 @@
         <v>9</v>
       </c>
       <c r="E120">
-        <v>0.13</v>
+        <v>0.12</v>
       </c>
       <c r="F120" t="s">
         <v>10</v>
@@ -5801,7 +5801,7 @@
         <v>9</v>
       </c>
       <c r="E121">
-        <v>0.28</v>
+        <v>0.31</v>
       </c>
       <c r="F121" t="s">
         <v>10</v>
@@ -5821,7 +5821,7 @@
         <v>9</v>
       </c>
       <c r="E122">
-        <v>0.34</v>
+        <v>0.22</v>
       </c>
       <c r="F122" t="s">
         <v>10</v>
@@ -5841,7 +5841,7 @@
         <v>9</v>
       </c>
       <c r="E123">
-        <v>0.1</v>
+        <v>0.27</v>
       </c>
       <c r="F123" t="s">
         <v>10</v>
@@ -5861,7 +5861,7 @@
         <v>9</v>
       </c>
       <c r="E124">
-        <v>0.39</v>
+        <v>0.3</v>
       </c>
       <c r="F124" t="s">
         <v>10</v>
@@ -5881,7 +5881,7 @@
         <v>9</v>
       </c>
       <c r="E125">
-        <v>0.38</v>
+        <v>0.36</v>
       </c>
       <c r="F125" t="s">
         <v>10</v>
@@ -5901,7 +5901,7 @@
         <v>9</v>
       </c>
       <c r="E126">
-        <v>0.18</v>
+        <v>0.29</v>
       </c>
       <c r="F126" t="s">
         <v>10</v>
@@ -5921,7 +5921,7 @@
         <v>9</v>
       </c>
       <c r="E127">
-        <v>0.12</v>
+        <v>0.15</v>
       </c>
       <c r="F127" t="s">
         <v>35</v>
@@ -5941,7 +5941,7 @@
         <v>9</v>
       </c>
       <c r="E128">
-        <v>0.18</v>
+        <v>0.27</v>
       </c>
       <c r="F128" t="s">
         <v>35</v>
@@ -5961,7 +5961,7 @@
         <v>9</v>
       </c>
       <c r="E129">
-        <v>0.19</v>
+        <v>0.17</v>
       </c>
       <c r="F129" t="s">
         <v>35</v>
@@ -5981,7 +5981,7 @@
         <v>9</v>
       </c>
       <c r="E130">
-        <v>0.31</v>
+        <v>0.38</v>
       </c>
       <c r="F130" t="s">
         <v>35</v>
@@ -6021,7 +6021,7 @@
         <v>9</v>
       </c>
       <c r="E132">
-        <v>0.3</v>
+        <v>0.16</v>
       </c>
       <c r="F132" t="s">
         <v>35</v>
@@ -6041,7 +6041,7 @@
         <v>9</v>
       </c>
       <c r="E133">
-        <v>0.36</v>
+        <v>0.25</v>
       </c>
       <c r="F133" t="s">
         <v>35</v>
@@ -6061,7 +6061,7 @@
         <v>9</v>
       </c>
       <c r="E134">
-        <v>0.24</v>
+        <v>0.15</v>
       </c>
       <c r="F134" t="s">
         <v>35</v>
@@ -6081,7 +6081,7 @@
         <v>9</v>
       </c>
       <c r="E135">
-        <v>0.24</v>
+        <v>0.32</v>
       </c>
       <c r="F135" t="s">
         <v>35</v>
@@ -6101,7 +6101,7 @@
         <v>9</v>
       </c>
       <c r="E136">
-        <v>0.25</v>
+        <v>0.12</v>
       </c>
       <c r="F136" t="s">
         <v>35</v>
@@ -6121,7 +6121,7 @@
         <v>9</v>
       </c>
       <c r="E137">
-        <v>0.14</v>
+        <v>0.23</v>
       </c>
       <c r="F137" t="s">
         <v>35</v>
@@ -6141,7 +6141,7 @@
         <v>9</v>
       </c>
       <c r="E138">
-        <v>0.27</v>
+        <v>0.35</v>
       </c>
       <c r="F138" t="s">
         <v>35</v>
@@ -6161,7 +6161,7 @@
         <v>9</v>
       </c>
       <c r="E139">
-        <v>0.25</v>
+        <v>0.29</v>
       </c>
       <c r="F139" t="s">
         <v>35</v>
@@ -6181,7 +6181,7 @@
         <v>9</v>
       </c>
       <c r="E140">
-        <v>0.26</v>
+        <v>0.19</v>
       </c>
       <c r="F140" t="s">
         <v>35</v>
@@ -6201,7 +6201,7 @@
         <v>9</v>
       </c>
       <c r="E141">
-        <v>0.35</v>
+        <v>0.19</v>
       </c>
       <c r="F141" t="s">
         <v>35</v>
@@ -6221,7 +6221,7 @@
         <v>9</v>
       </c>
       <c r="E142">
-        <v>0.25</v>
+        <v>0.11</v>
       </c>
       <c r="F142" t="s">
         <v>60</v>
@@ -6241,7 +6241,7 @@
         <v>9</v>
       </c>
       <c r="E143">
-        <v>0.18</v>
+        <v>0.14</v>
       </c>
       <c r="F143" t="s">
         <v>60</v>
@@ -6261,7 +6261,7 @@
         <v>9</v>
       </c>
       <c r="E144">
-        <v>0.11</v>
+        <v>0.23</v>
       </c>
       <c r="F144" t="s">
         <v>60</v>
@@ -6281,7 +6281,7 @@
         <v>9</v>
       </c>
       <c r="E145">
-        <v>0.24</v>
+        <v>0.21</v>
       </c>
       <c r="F145" t="s">
         <v>60</v>
@@ -6301,7 +6301,7 @@
         <v>9</v>
       </c>
       <c r="E146">
-        <v>0.27</v>
+        <v>0.28</v>
       </c>
       <c r="F146" t="s">
         <v>60</v>
@@ -6321,7 +6321,7 @@
         <v>9</v>
       </c>
       <c r="E147">
-        <v>0.31</v>
+        <v>0.36</v>
       </c>
       <c r="F147" t="s">
         <v>60</v>
@@ -6341,7 +6341,7 @@
         <v>9</v>
       </c>
       <c r="E148">
-        <v>0.35</v>
+        <v>0.2</v>
       </c>
       <c r="F148" t="s">
         <v>60</v>
@@ -6361,7 +6361,7 @@
         <v>9</v>
       </c>
       <c r="E149">
-        <v>0.13</v>
+        <v>0.31</v>
       </c>
       <c r="F149" t="s">
         <v>60</v>
@@ -6381,7 +6381,7 @@
         <v>9</v>
       </c>
       <c r="E150">
-        <v>0.12</v>
+        <v>0.32</v>
       </c>
       <c r="F150" t="s">
         <v>60</v>
@@ -6401,7 +6401,7 @@
         <v>9</v>
       </c>
       <c r="E151">
-        <v>0.17</v>
+        <v>0.2</v>
       </c>
       <c r="F151" t="s">
         <v>60</v>
@@ -6421,7 +6421,7 @@
         <v>9</v>
       </c>
       <c r="E152">
-        <v>0.29</v>
+        <v>0.33</v>
       </c>
       <c r="F152" t="s">
         <v>60</v>
@@ -6441,7 +6441,7 @@
         <v>9</v>
       </c>
       <c r="E153">
-        <v>0.34</v>
+        <v>0.21</v>
       </c>
       <c r="F153" t="s">
         <v>60</v>
@@ -6461,7 +6461,7 @@
         <v>9</v>
       </c>
       <c r="E154">
-        <v>0.16</v>
+        <v>0.13</v>
       </c>
       <c r="F154" t="s">
         <v>60</v>
@@ -6481,7 +6481,7 @@
         <v>9</v>
       </c>
       <c r="E155">
-        <v>0.12</v>
+        <v>0.18</v>
       </c>
       <c r="F155" t="s">
         <v>60</v>
@@ -6501,7 +6501,7 @@
         <v>9</v>
       </c>
       <c r="E156">
-        <v>0.39</v>
+        <v>0.14</v>
       </c>
       <c r="F156" t="s">
         <v>60</v>
@@ -6521,7 +6521,7 @@
         <v>9</v>
       </c>
       <c r="E157">
-        <v>0.28</v>
+        <v>0.29</v>
       </c>
       <c r="F157" t="s">
         <v>60</v>
@@ -6541,7 +6541,7 @@
         <v>9</v>
       </c>
       <c r="E158">
-        <v>0.24</v>
+        <v>0.31</v>
       </c>
       <c r="F158" t="s">
         <v>60</v>
@@ -6561,7 +6561,7 @@
         <v>9</v>
       </c>
       <c r="E159">
-        <v>0.39</v>
+        <v>0.25</v>
       </c>
       <c r="F159" t="s">
         <v>60</v>
@@ -6581,7 +6581,7 @@
         <v>9</v>
       </c>
       <c r="E160">
-        <v>0.1</v>
+        <v>0.27</v>
       </c>
       <c r="F160" t="s">
         <v>60</v>
@@ -6601,7 +6601,7 @@
         <v>9</v>
       </c>
       <c r="E161">
-        <v>0.11</v>
+        <v>0.16</v>
       </c>
       <c r="F161" t="s">
         <v>60</v>
@@ -6621,7 +6621,7 @@
         <v>9</v>
       </c>
       <c r="E162">
-        <v>0.22</v>
+        <v>0.25</v>
       </c>
       <c r="F162" t="s">
         <v>10</v>
@@ -6641,7 +6641,7 @@
         <v>9</v>
       </c>
       <c r="E163">
-        <v>0.14</v>
+        <v>0.23</v>
       </c>
       <c r="F163" t="s">
         <v>10</v>
@@ -6661,7 +6661,7 @@
         <v>9</v>
       </c>
       <c r="E164">
-        <v>0.11</v>
+        <v>0.21</v>
       </c>
       <c r="F164" t="s">
         <v>10</v>
@@ -6681,7 +6681,7 @@
         <v>9</v>
       </c>
       <c r="E165">
-        <v>0.18</v>
+        <v>0.37</v>
       </c>
       <c r="F165" t="s">
         <v>10</v>
@@ -6701,7 +6701,7 @@
         <v>9</v>
       </c>
       <c r="E166">
-        <v>0.4</v>
+        <v>0.13</v>
       </c>
       <c r="F166" t="s">
         <v>10</v>
@@ -6721,7 +6721,7 @@
         <v>9</v>
       </c>
       <c r="E167">
-        <v>0.11</v>
+        <v>0.16</v>
       </c>
       <c r="F167" t="s">
         <v>10</v>
@@ -6741,7 +6741,7 @@
         <v>9</v>
       </c>
       <c r="E168">
-        <v>0.15</v>
+        <v>0.18</v>
       </c>
       <c r="F168" t="s">
         <v>10</v>
@@ -6761,7 +6761,7 @@
         <v>9</v>
       </c>
       <c r="E169">
-        <v>0.11</v>
+        <v>0.18</v>
       </c>
       <c r="F169" t="s">
         <v>10</v>
@@ -6781,7 +6781,7 @@
         <v>9</v>
       </c>
       <c r="E170">
-        <v>0.37</v>
+        <v>0.1</v>
       </c>
       <c r="F170" t="s">
         <v>10</v>
@@ -6801,7 +6801,7 @@
         <v>9</v>
       </c>
       <c r="E171">
-        <v>0.32</v>
+        <v>0.37</v>
       </c>
       <c r="F171" t="s">
         <v>10</v>
@@ -6821,7 +6821,7 @@
         <v>9</v>
       </c>
       <c r="E172">
-        <v>0.26</v>
+        <v>0.21</v>
       </c>
       <c r="F172" t="s">
         <v>10</v>
@@ -6841,7 +6841,7 @@
         <v>9</v>
       </c>
       <c r="E173">
-        <v>0.18</v>
+        <v>0.38</v>
       </c>
       <c r="F173" t="s">
         <v>10</v>
@@ -6861,7 +6861,7 @@
         <v>9</v>
       </c>
       <c r="E174">
-        <v>0.37</v>
+        <v>0.25</v>
       </c>
       <c r="F174" t="s">
         <v>10</v>
@@ -6881,7 +6881,7 @@
         <v>9</v>
       </c>
       <c r="E175">
-        <v>0.2</v>
+        <v>0.24</v>
       </c>
       <c r="F175" t="s">
         <v>10</v>
@@ -6901,7 +6901,7 @@
         <v>9</v>
       </c>
       <c r="E176">
-        <v>0.2</v>
+        <v>0.36</v>
       </c>
       <c r="F176" t="s">
         <v>10</v>
@@ -6921,7 +6921,7 @@
         <v>9</v>
       </c>
       <c r="E177">
-        <v>0.23</v>
+        <v>0.34</v>
       </c>
       <c r="F177" t="s">
         <v>35</v>
@@ -6941,7 +6941,7 @@
         <v>9</v>
       </c>
       <c r="E178">
-        <v>0.22</v>
+        <v>0.24</v>
       </c>
       <c r="F178" t="s">
         <v>35</v>
@@ -6961,7 +6961,7 @@
         <v>9</v>
       </c>
       <c r="E179">
-        <v>0.2</v>
+        <v>0.22</v>
       </c>
       <c r="F179" t="s">
         <v>35</v>
@@ -6981,7 +6981,7 @@
         <v>9</v>
       </c>
       <c r="E180">
-        <v>0.15</v>
+        <v>0.17</v>
       </c>
       <c r="F180" t="s">
         <v>35</v>
@@ -7001,7 +7001,7 @@
         <v>9</v>
       </c>
       <c r="E181">
-        <v>0.17</v>
+        <v>0.14</v>
       </c>
       <c r="F181" t="s">
         <v>35</v>
@@ -7021,7 +7021,7 @@
         <v>9</v>
       </c>
       <c r="E182">
-        <v>0.14</v>
+        <v>0.23</v>
       </c>
       <c r="F182" t="s">
         <v>35</v>
@@ -7041,7 +7041,7 @@
         <v>9</v>
       </c>
       <c r="E183">
-        <v>0.33</v>
+        <v>0.22</v>
       </c>
       <c r="F183" t="s">
         <v>35</v>
@@ -7061,7 +7061,7 @@
         <v>9</v>
       </c>
       <c r="E184">
-        <v>0.34</v>
+        <v>0.15</v>
       </c>
       <c r="F184" t="s">
         <v>35</v>
@@ -7081,7 +7081,7 @@
         <v>9</v>
       </c>
       <c r="E185">
-        <v>0.14</v>
+        <v>0.22</v>
       </c>
       <c r="F185" t="s">
         <v>35</v>
@@ -7121,7 +7121,7 @@
         <v>9</v>
       </c>
       <c r="E187">
-        <v>0.14</v>
+        <v>0.11</v>
       </c>
       <c r="F187" t="s">
         <v>35</v>
@@ -7141,7 +7141,7 @@
         <v>9</v>
       </c>
       <c r="E188">
-        <v>0.13</v>
+        <v>0.34</v>
       </c>
       <c r="F188" t="s">
         <v>35</v>
@@ -7181,7 +7181,7 @@
         <v>9</v>
       </c>
       <c r="E190">
-        <v>0.24</v>
+        <v>0.13</v>
       </c>
       <c r="F190" t="s">
         <v>35</v>
@@ -7201,7 +7201,7 @@
         <v>9</v>
       </c>
       <c r="E191">
-        <v>0.24</v>
+        <v>0.17</v>
       </c>
       <c r="F191" t="s">
         <v>35</v>
@@ -7221,7 +7221,7 @@
         <v>9</v>
       </c>
       <c r="E192">
-        <v>0.11</v>
+        <v>0.17</v>
       </c>
       <c r="F192" t="s">
         <v>60</v>
@@ -7241,7 +7241,7 @@
         <v>9</v>
       </c>
       <c r="E193">
-        <v>0.3</v>
+        <v>0.18</v>
       </c>
       <c r="F193" t="s">
         <v>60</v>
@@ -7261,7 +7261,7 @@
         <v>9</v>
       </c>
       <c r="E194">
-        <v>0.28</v>
+        <v>0.25</v>
       </c>
       <c r="F194" t="s">
         <v>60</v>
@@ -7281,7 +7281,7 @@
         <v>9</v>
       </c>
       <c r="E195">
-        <v>0.18</v>
+        <v>0.28</v>
       </c>
       <c r="F195" t="s">
         <v>60</v>
@@ -7301,7 +7301,7 @@
         <v>9</v>
       </c>
       <c r="E196">
-        <v>0.31</v>
+        <v>0.3</v>
       </c>
       <c r="F196" t="s">
         <v>60</v>
@@ -7321,7 +7321,7 @@
         <v>9</v>
       </c>
       <c r="E197">
-        <v>0.39</v>
+        <v>0.18</v>
       </c>
       <c r="F197" t="s">
         <v>60</v>
@@ -7341,7 +7341,7 @@
         <v>9</v>
       </c>
       <c r="E198">
-        <v>0.38</v>
+        <v>0.3</v>
       </c>
       <c r="F198" t="s">
         <v>60</v>
@@ -7361,7 +7361,7 @@
         <v>9</v>
       </c>
       <c r="E199">
-        <v>0.35</v>
+        <v>0.14</v>
       </c>
       <c r="F199" t="s">
         <v>60</v>
@@ -7381,7 +7381,7 @@
         <v>9</v>
       </c>
       <c r="E200">
-        <v>0.37</v>
+        <v>0.25</v>
       </c>
       <c r="F200" t="s">
         <v>60</v>
@@ -7401,7 +7401,7 @@
         <v>9</v>
       </c>
       <c r="E201">
-        <v>0.14</v>
+        <v>0.33</v>
       </c>
       <c r="F201" t="s">
         <v>60</v>
@@ -7421,7 +7421,7 @@
         <v>9</v>
       </c>
       <c r="E202">
-        <v>0.36</v>
+        <v>0.19</v>
       </c>
       <c r="F202" t="s">
         <v>60</v>
@@ -7441,7 +7441,7 @@
         <v>9</v>
       </c>
       <c r="E203">
-        <v>0.18</v>
+        <v>0.36</v>
       </c>
       <c r="F203" t="s">
         <v>60</v>
@@ -7461,7 +7461,7 @@
         <v>9</v>
       </c>
       <c r="E204">
-        <v>0.3</v>
+        <v>0.26</v>
       </c>
       <c r="F204" t="s">
         <v>60</v>
@@ -7481,7 +7481,7 @@
         <v>9</v>
       </c>
       <c r="E205">
-        <v>0.38</v>
+        <v>0.17</v>
       </c>
       <c r="F205" t="s">
         <v>60</v>
@@ -7501,7 +7501,7 @@
         <v>9</v>
       </c>
       <c r="E206">
-        <v>0.16</v>
+        <v>0.31</v>
       </c>
       <c r="F206" t="s">
         <v>60</v>
@@ -7521,7 +7521,7 @@
         <v>9</v>
       </c>
       <c r="E207">
-        <v>0.15</v>
+        <v>0.33</v>
       </c>
       <c r="F207" t="s">
         <v>60</v>
@@ -7541,7 +7541,7 @@
         <v>9</v>
       </c>
       <c r="E208">
-        <v>0.2</v>
+        <v>0.19</v>
       </c>
       <c r="F208" t="s">
         <v>60</v>
@@ -7561,7 +7561,7 @@
         <v>9</v>
       </c>
       <c r="E209">
-        <v>0.35</v>
+        <v>0.18</v>
       </c>
       <c r="F209" t="s">
         <v>60</v>
@@ -7581,7 +7581,7 @@
         <v>9</v>
       </c>
       <c r="E210">
-        <v>0.39</v>
+        <v>0.3</v>
       </c>
       <c r="F210" t="s">
         <v>60</v>
@@ -7601,7 +7601,7 @@
         <v>9</v>
       </c>
       <c r="E211">
-        <v>0.17</v>
+        <v>0.25</v>
       </c>
       <c r="F211" t="s">
         <v>60</v>
@@ -7621,7 +7621,7 @@
         <v>9</v>
       </c>
       <c r="E212">
-        <v>0.39</v>
+        <v>0.38</v>
       </c>
       <c r="F212" t="s">
         <v>10</v>
@@ -7641,7 +7641,7 @@
         <v>9</v>
       </c>
       <c r="E213">
-        <v>0.16</v>
+        <v>0.4</v>
       </c>
       <c r="F213" t="s">
         <v>10</v>
@@ -7661,7 +7661,7 @@
         <v>9</v>
       </c>
       <c r="E214">
-        <v>0.21</v>
+        <v>0.31</v>
       </c>
       <c r="F214" t="s">
         <v>10</v>
@@ -7681,7 +7681,7 @@
         <v>9</v>
       </c>
       <c r="E215">
-        <v>0.19</v>
+        <v>0.35</v>
       </c>
       <c r="F215" t="s">
         <v>10</v>
@@ -7701,7 +7701,7 @@
         <v>9</v>
       </c>
       <c r="E216">
-        <v>0.33</v>
+        <v>0.19</v>
       </c>
       <c r="F216" t="s">
         <v>10</v>
@@ -7721,7 +7721,7 @@
         <v>9</v>
       </c>
       <c r="E217">
-        <v>0.37</v>
+        <v>0.21</v>
       </c>
       <c r="F217" t="s">
         <v>10</v>
@@ -7741,7 +7741,7 @@
         <v>9</v>
       </c>
       <c r="E218">
-        <v>0.13</v>
+        <v>0.3</v>
       </c>
       <c r="F218" t="s">
         <v>10</v>
@@ -7761,7 +7761,7 @@
         <v>9</v>
       </c>
       <c r="E219">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="F219" t="s">
         <v>10</v>
@@ -7781,7 +7781,7 @@
         <v>9</v>
       </c>
       <c r="E220">
-        <v>0.2</v>
+        <v>0.17</v>
       </c>
       <c r="F220" t="s">
         <v>10</v>
@@ -7801,7 +7801,7 @@
         <v>9</v>
       </c>
       <c r="E221">
-        <v>0.37</v>
+        <v>0.34</v>
       </c>
       <c r="F221" t="s">
         <v>10</v>
@@ -7821,7 +7821,7 @@
         <v>9</v>
       </c>
       <c r="E222">
-        <v>0.13</v>
+        <v>0.23</v>
       </c>
       <c r="F222" t="s">
         <v>10</v>
@@ -7841,7 +7841,7 @@
         <v>9</v>
       </c>
       <c r="E223">
-        <v>0.14</v>
+        <v>0.27</v>
       </c>
       <c r="F223" t="s">
         <v>10</v>
@@ -7861,7 +7861,7 @@
         <v>9</v>
       </c>
       <c r="E224">
-        <v>0.15</v>
+        <v>0.1</v>
       </c>
       <c r="F224" t="s">
         <v>10</v>
@@ -7901,7 +7901,7 @@
         <v>9</v>
       </c>
       <c r="E226">
-        <v>0.15</v>
+        <v>0.31</v>
       </c>
       <c r="F226" t="s">
         <v>10</v>
@@ -7921,7 +7921,7 @@
         <v>9</v>
       </c>
       <c r="E227">
-        <v>0.12</v>
+        <v>0.1</v>
       </c>
       <c r="F227" t="s">
         <v>35</v>
@@ -7941,7 +7941,7 @@
         <v>9</v>
       </c>
       <c r="E228">
-        <v>0.32</v>
+        <v>0.35</v>
       </c>
       <c r="F228" t="s">
         <v>35</v>
@@ -7961,7 +7961,7 @@
         <v>9</v>
       </c>
       <c r="E229">
-        <v>0.27</v>
+        <v>0.1</v>
       </c>
       <c r="F229" t="s">
         <v>35</v>
@@ -7981,7 +7981,7 @@
         <v>9</v>
       </c>
       <c r="E230">
-        <v>0.35</v>
+        <v>0.11</v>
       </c>
       <c r="F230" t="s">
         <v>35</v>
@@ -8001,7 +8001,7 @@
         <v>9</v>
       </c>
       <c r="E231">
-        <v>0.18</v>
+        <v>0.32</v>
       </c>
       <c r="F231" t="s">
         <v>35</v>
@@ -8021,7 +8021,7 @@
         <v>9</v>
       </c>
       <c r="E232">
-        <v>0.22</v>
+        <v>0.27</v>
       </c>
       <c r="F232" t="s">
         <v>35</v>
@@ -8041,7 +8041,7 @@
         <v>9</v>
       </c>
       <c r="E233">
-        <v>0.23</v>
+        <v>0.22</v>
       </c>
       <c r="F233" t="s">
         <v>35</v>
@@ -8081,7 +8081,7 @@
         <v>9</v>
       </c>
       <c r="E235">
-        <v>0.23</v>
+        <v>0.12</v>
       </c>
       <c r="F235" t="s">
         <v>35</v>
@@ -8101,7 +8101,7 @@
         <v>9</v>
       </c>
       <c r="E236">
-        <v>0.17</v>
+        <v>0.14</v>
       </c>
       <c r="F236" t="s">
         <v>35</v>
@@ -8121,7 +8121,7 @@
         <v>9</v>
       </c>
       <c r="E237">
-        <v>0.28</v>
+        <v>0.32</v>
       </c>
       <c r="F237" t="s">
         <v>35</v>
@@ -8141,7 +8141,7 @@
         <v>9</v>
       </c>
       <c r="E238">
-        <v>0.18</v>
+        <v>0.27</v>
       </c>
       <c r="F238" t="s">
         <v>35</v>
@@ -8161,7 +8161,7 @@
         <v>9</v>
       </c>
       <c r="E239">
-        <v>0.14</v>
+        <v>0.33</v>
       </c>
       <c r="F239" t="s">
         <v>35</v>
@@ -8181,7 +8181,7 @@
         <v>9</v>
       </c>
       <c r="E240">
-        <v>0.31</v>
+        <v>0.2</v>
       </c>
       <c r="F240" t="s">
         <v>35</v>
@@ -8201,7 +8201,7 @@
         <v>9</v>
       </c>
       <c r="E241">
-        <v>0.29</v>
+        <v>0.18</v>
       </c>
       <c r="F241" t="s">
         <v>35</v>
@@ -8221,7 +8221,7 @@
         <v>9</v>
       </c>
       <c r="E242">
-        <v>0.19</v>
+        <v>0.36</v>
       </c>
       <c r="F242" t="s">
         <v>60</v>
@@ -8241,7 +8241,7 @@
         <v>9</v>
       </c>
       <c r="E243">
-        <v>0.21</v>
+        <v>0.13</v>
       </c>
       <c r="F243" t="s">
         <v>60</v>
@@ -8261,7 +8261,7 @@
         <v>9</v>
       </c>
       <c r="E244">
-        <v>0.23</v>
+        <v>0.1</v>
       </c>
       <c r="F244" t="s">
         <v>60</v>
@@ -8281,7 +8281,7 @@
         <v>9</v>
       </c>
       <c r="E245">
-        <v>0.31</v>
+        <v>0.34</v>
       </c>
       <c r="F245" t="s">
         <v>60</v>
@@ -8301,7 +8301,7 @@
         <v>9</v>
       </c>
       <c r="E246">
-        <v>0.27</v>
+        <v>0.2</v>
       </c>
       <c r="F246" t="s">
         <v>60</v>
@@ -8321,7 +8321,7 @@
         <v>9</v>
       </c>
       <c r="E247">
-        <v>0.26</v>
+        <v>0.24</v>
       </c>
       <c r="F247" t="s">
         <v>60</v>
@@ -8341,7 +8341,7 @@
         <v>9</v>
       </c>
       <c r="E248">
-        <v>0.32</v>
+        <v>0.16</v>
       </c>
       <c r="F248" t="s">
         <v>60</v>
@@ -8361,7 +8361,7 @@
         <v>9</v>
       </c>
       <c r="E249">
-        <v>0.25</v>
+        <v>0.28</v>
       </c>
       <c r="F249" t="s">
         <v>60</v>
@@ -8381,7 +8381,7 @@
         <v>9</v>
       </c>
       <c r="E250">
-        <v>0.16</v>
+        <v>0.32</v>
       </c>
       <c r="F250" t="s">
         <v>60</v>
@@ -8401,7 +8401,7 @@
         <v>9</v>
       </c>
       <c r="E251">
-        <v>0.22</v>
+        <v>0.36</v>
       </c>
       <c r="F251" t="s">
         <v>60</v>
@@ -8421,7 +8421,7 @@
         <v>9</v>
       </c>
       <c r="E252">
-        <v>0.13</v>
+        <v>0.32</v>
       </c>
       <c r="F252" t="s">
         <v>60</v>
@@ -8441,7 +8441,7 @@
         <v>9</v>
       </c>
       <c r="E253">
-        <v>0.26</v>
+        <v>0.1</v>
       </c>
       <c r="F253" t="s">
         <v>60</v>
@@ -8461,7 +8461,7 @@
         <v>9</v>
       </c>
       <c r="E254">
-        <v>0.3</v>
+        <v>0.37</v>
       </c>
       <c r="F254" t="s">
         <v>60</v>
@@ -8481,7 +8481,7 @@
         <v>9</v>
       </c>
       <c r="E255">
-        <v>0.13</v>
+        <v>0.15</v>
       </c>
       <c r="F255" t="s">
         <v>60</v>
@@ -8501,7 +8501,7 @@
         <v>9</v>
       </c>
       <c r="E256">
-        <v>0.3</v>
+        <v>0.21</v>
       </c>
       <c r="F256" t="s">
         <v>60</v>
@@ -8521,7 +8521,7 @@
         <v>9</v>
       </c>
       <c r="E257">
-        <v>0.34</v>
+        <v>0.26</v>
       </c>
       <c r="F257" t="s">
         <v>60</v>
@@ -8541,7 +8541,7 @@
         <v>9</v>
       </c>
       <c r="E258">
-        <v>0.33</v>
+        <v>0.34</v>
       </c>
       <c r="F258" t="s">
         <v>60</v>
@@ -8561,7 +8561,7 @@
         <v>9</v>
       </c>
       <c r="E259">
-        <v>0.13</v>
+        <v>0.17</v>
       </c>
       <c r="F259" t="s">
         <v>60</v>
@@ -8601,7 +8601,7 @@
         <v>9</v>
       </c>
       <c r="E261">
-        <v>0.14</v>
+        <v>0.34</v>
       </c>
       <c r="F261" t="s">
         <v>60</v>
@@ -8621,7 +8621,7 @@
         <v>9</v>
       </c>
       <c r="E262">
-        <v>0.36</v>
+        <v>0.21</v>
       </c>
       <c r="F262" t="s">
         <v>10</v>
@@ -8641,7 +8641,7 @@
         <v>9</v>
       </c>
       <c r="E263">
-        <v>0.39</v>
+        <v>0.33</v>
       </c>
       <c r="F263" t="s">
         <v>10</v>
@@ -8661,7 +8661,7 @@
         <v>9</v>
       </c>
       <c r="E264">
-        <v>0.33</v>
+        <v>0.27</v>
       </c>
       <c r="F264" t="s">
         <v>10</v>
@@ -8681,7 +8681,7 @@
         <v>9</v>
       </c>
       <c r="E265">
-        <v>0.16</v>
+        <v>0.12</v>
       </c>
       <c r="F265" t="s">
         <v>10</v>
@@ -8701,7 +8701,7 @@
         <v>9</v>
       </c>
       <c r="E266">
-        <v>0.12</v>
+        <v>0.1</v>
       </c>
       <c r="F266" t="s">
         <v>10</v>
@@ -8721,7 +8721,7 @@
         <v>9</v>
       </c>
       <c r="E267">
-        <v>0.22</v>
+        <v>0.19</v>
       </c>
       <c r="F267" t="s">
         <v>10</v>
@@ -8761,7 +8761,7 @@
         <v>9</v>
       </c>
       <c r="E269">
-        <v>0.3</v>
+        <v>0.15</v>
       </c>
       <c r="F269" t="s">
         <v>10</v>
@@ -8781,7 +8781,7 @@
         <v>9</v>
       </c>
       <c r="E270">
-        <v>0.17</v>
+        <v>0.12</v>
       </c>
       <c r="F270" t="s">
         <v>10</v>
@@ -8801,7 +8801,7 @@
         <v>9</v>
       </c>
       <c r="E271">
-        <v>0.37</v>
+        <v>0.15</v>
       </c>
       <c r="F271" t="s">
         <v>10</v>
@@ -8821,7 +8821,7 @@
         <v>9</v>
       </c>
       <c r="E272">
-        <v>0.34</v>
+        <v>0.28</v>
       </c>
       <c r="F272" t="s">
         <v>10</v>
@@ -8841,7 +8841,7 @@
         <v>9</v>
       </c>
       <c r="E273">
-        <v>0.34</v>
+        <v>0.11</v>
       </c>
       <c r="F273" t="s">
         <v>10</v>
@@ -8861,7 +8861,7 @@
         <v>9</v>
       </c>
       <c r="E274">
-        <v>0.28</v>
+        <v>0.23</v>
       </c>
       <c r="F274" t="s">
         <v>35</v>
@@ -8901,7 +8901,7 @@
         <v>9</v>
       </c>
       <c r="E276">
-        <v>0.27</v>
+        <v>0.2</v>
       </c>
       <c r="F276" t="s">
         <v>35</v>
@@ -8921,7 +8921,7 @@
         <v>9</v>
       </c>
       <c r="E277">
-        <v>0.29</v>
+        <v>0.22</v>
       </c>
       <c r="F277" t="s">
         <v>35</v>
@@ -8941,7 +8941,7 @@
         <v>9</v>
       </c>
       <c r="E278">
-        <v>0.17</v>
+        <v>0.21</v>
       </c>
       <c r="F278" t="s">
         <v>35</v>
@@ -8961,7 +8961,7 @@
         <v>9</v>
       </c>
       <c r="E279">
-        <v>0.38</v>
+        <v>0.21</v>
       </c>
       <c r="F279" t="s">
         <v>35</v>
@@ -8981,7 +8981,7 @@
         <v>9</v>
       </c>
       <c r="E280">
-        <v>0.11</v>
+        <v>0.34</v>
       </c>
       <c r="F280" t="s">
         <v>35</v>
@@ -9001,7 +9001,7 @@
         <v>9</v>
       </c>
       <c r="E281">
-        <v>0.23</v>
+        <v>0.31</v>
       </c>
       <c r="F281" t="s">
         <v>35</v>
@@ -9021,7 +9021,7 @@
         <v>9</v>
       </c>
       <c r="E282">
-        <v>0.26</v>
+        <v>0.28</v>
       </c>
       <c r="F282" t="s">
         <v>35</v>
@@ -9041,7 +9041,7 @@
         <v>9</v>
       </c>
       <c r="E283">
-        <v>0.19</v>
+        <v>0.29</v>
       </c>
       <c r="F283" t="s">
         <v>35</v>
@@ -9061,7 +9061,7 @@
         <v>9</v>
       </c>
       <c r="E284">
-        <v>0.23</v>
+        <v>0.34</v>
       </c>
       <c r="F284" t="s">
         <v>35</v>
@@ -9081,7 +9081,7 @@
         <v>9</v>
       </c>
       <c r="E285">
-        <v>0.24</v>
+        <v>0.2</v>
       </c>
       <c r="F285" t="s">
         <v>35</v>
@@ -9101,7 +9101,7 @@
         <v>9</v>
       </c>
       <c r="E286">
-        <v>0.12</v>
+        <v>0.2</v>
       </c>
       <c r="F286" t="s">
         <v>60</v>
@@ -9121,7 +9121,7 @@
         <v>9</v>
       </c>
       <c r="E287">
-        <v>0.4</v>
+        <v>0.23</v>
       </c>
       <c r="F287" t="s">
         <v>60</v>
@@ -9141,7 +9141,7 @@
         <v>9</v>
       </c>
       <c r="E288">
-        <v>0.27</v>
+        <v>0.38</v>
       </c>
       <c r="F288" t="s">
         <v>60</v>
@@ -9161,7 +9161,7 @@
         <v>9</v>
       </c>
       <c r="E289">
-        <v>0.25</v>
+        <v>0.15</v>
       </c>
       <c r="F289" t="s">
         <v>60</v>
@@ -9181,7 +9181,7 @@
         <v>9</v>
       </c>
       <c r="E290">
-        <v>0.19</v>
+        <v>0.18</v>
       </c>
       <c r="F290" t="s">
         <v>60</v>
@@ -9201,7 +9201,7 @@
         <v>9</v>
       </c>
       <c r="E291">
-        <v>0.36</v>
+        <v>0.21</v>
       </c>
       <c r="F291" t="s">
         <v>60</v>
@@ -9221,7 +9221,7 @@
         <v>9</v>
       </c>
       <c r="E292">
-        <v>0.32</v>
+        <v>0.21</v>
       </c>
       <c r="F292" t="s">
         <v>60</v>
@@ -9241,7 +9241,7 @@
         <v>9</v>
       </c>
       <c r="E293">
-        <v>0.23</v>
+        <v>0.15</v>
       </c>
       <c r="F293" t="s">
         <v>60</v>
@@ -9261,7 +9261,7 @@
         <v>9</v>
       </c>
       <c r="E294">
-        <v>0.36</v>
+        <v>0.38</v>
       </c>
       <c r="F294" t="s">
         <v>60</v>
@@ -9281,7 +9281,7 @@
         <v>9</v>
       </c>
       <c r="E295">
-        <v>0.33</v>
+        <v>0.13</v>
       </c>
       <c r="F295" t="s">
         <v>60</v>
@@ -9301,7 +9301,7 @@
         <v>9</v>
       </c>
       <c r="E296">
-        <v>0.18</v>
+        <v>0.11</v>
       </c>
       <c r="F296" t="s">
         <v>60</v>
@@ -9321,7 +9321,7 @@
         <v>9</v>
       </c>
       <c r="E297">
-        <v>0.26</v>
+        <v>0.25</v>
       </c>
       <c r="F297" t="s">
         <v>60</v>
@@ -9341,7 +9341,7 @@
         <v>9</v>
       </c>
       <c r="E298">
-        <v>0.17</v>
+        <v>0.28</v>
       </c>
       <c r="F298" t="s">
         <v>60</v>
@@ -9361,7 +9361,7 @@
         <v>9</v>
       </c>
       <c r="E299">
-        <v>0.19</v>
+        <v>0.2</v>
       </c>
       <c r="F299" t="s">
         <v>60</v>
@@ -9381,7 +9381,7 @@
         <v>9</v>
       </c>
       <c r="E300">
-        <v>0.18</v>
+        <v>0.36</v>
       </c>
       <c r="F300" t="s">
         <v>60</v>
@@ -9401,7 +9401,7 @@
         <v>9</v>
       </c>
       <c r="E301">
-        <v>0.25</v>
+        <v>0.33</v>
       </c>
       <c r="F301" t="s">
         <v>60</v>
@@ -9421,7 +9421,7 @@
         <v>9</v>
       </c>
       <c r="E302">
-        <v>0.4</v>
+        <v>0.38</v>
       </c>
       <c r="F302" t="s">
         <v>10</v>
@@ -9441,7 +9441,7 @@
         <v>9</v>
       </c>
       <c r="E303">
-        <v>0.18</v>
+        <v>0.27</v>
       </c>
       <c r="F303" t="s">
         <v>10</v>
@@ -9461,7 +9461,7 @@
         <v>9</v>
       </c>
       <c r="E304">
-        <v>0.25</v>
+        <v>0.31</v>
       </c>
       <c r="F304" t="s">
         <v>10</v>
@@ -9481,7 +9481,7 @@
         <v>9</v>
       </c>
       <c r="E305">
-        <v>0.14</v>
+        <v>0.19</v>
       </c>
       <c r="F305" t="s">
         <v>10</v>
@@ -9501,7 +9501,7 @@
         <v>9</v>
       </c>
       <c r="E306">
-        <v>0.36</v>
+        <v>0.37</v>
       </c>
       <c r="F306" t="s">
         <v>10</v>
@@ -9521,7 +9521,7 @@
         <v>9</v>
       </c>
       <c r="E307">
-        <v>0.22</v>
+        <v>0.21</v>
       </c>
       <c r="F307" t="s">
         <v>10</v>
@@ -9541,7 +9541,7 @@
         <v>9</v>
       </c>
       <c r="E308">
-        <v>0.17</v>
+        <v>0.27</v>
       </c>
       <c r="F308" t="s">
         <v>35</v>
@@ -9561,7 +9561,7 @@
         <v>9</v>
       </c>
       <c r="E309">
-        <v>0.11</v>
+        <v>0.14</v>
       </c>
       <c r="F309" t="s">
         <v>35</v>
@@ -9601,7 +9601,7 @@
         <v>9</v>
       </c>
       <c r="E311">
-        <v>0.28</v>
+        <v>0.26</v>
       </c>
       <c r="F311" t="s">
         <v>35</v>
@@ -9621,7 +9621,7 @@
         <v>9</v>
       </c>
       <c r="E312">
-        <v>0.15</v>
+        <v>0.23</v>
       </c>
       <c r="F312" t="s">
         <v>35</v>
@@ -9641,7 +9641,7 @@
         <v>9</v>
       </c>
       <c r="E313">
-        <v>0.31</v>
+        <v>0.3</v>
       </c>
       <c r="F313" t="s">
         <v>35</v>
@@ -9661,7 +9661,7 @@
         <v>9</v>
       </c>
       <c r="E314">
-        <v>0.3</v>
+        <v>0.26</v>
       </c>
       <c r="F314" t="s">
         <v>60</v>
@@ -9681,7 +9681,7 @@
         <v>9</v>
       </c>
       <c r="E315">
-        <v>0.12</v>
+        <v>0.33</v>
       </c>
       <c r="F315" t="s">
         <v>60</v>
@@ -9701,7 +9701,7 @@
         <v>9</v>
       </c>
       <c r="E316">
-        <v>0.36</v>
+        <v>0.25</v>
       </c>
       <c r="F316" t="s">
         <v>60</v>
@@ -9721,7 +9721,7 @@
         <v>9</v>
       </c>
       <c r="E317">
-        <v>0.31</v>
+        <v>0.2</v>
       </c>
       <c r="F317" t="s">
         <v>60</v>
@@ -9741,7 +9741,7 @@
         <v>9</v>
       </c>
       <c r="E318">
-        <v>0.39</v>
+        <v>0.11</v>
       </c>
       <c r="F318" t="s">
         <v>60</v>
@@ -9761,7 +9761,7 @@
         <v>9</v>
       </c>
       <c r="E319">
-        <v>0.11</v>
+        <v>0.33</v>
       </c>
       <c r="F319" t="s">
         <v>60</v>
@@ -9781,7 +9781,7 @@
         <v>9</v>
       </c>
       <c r="E320">
-        <v>0.24</v>
+        <v>0.16</v>
       </c>
       <c r="F320" t="s">
         <v>60</v>
@@ -9801,7 +9801,7 @@
         <v>9</v>
       </c>
       <c r="E321">
-        <v>0.35</v>
+        <v>0.31</v>
       </c>
       <c r="F321" t="s">
         <v>60</v>
@@ -9821,7 +9821,7 @@
         <v>9</v>
       </c>
       <c r="E322">
-        <v>0.34</v>
+        <v>0.36</v>
       </c>
       <c r="F322" t="s">
         <v>10</v>
@@ -9841,7 +9841,7 @@
         <v>9</v>
       </c>
       <c r="E323">
-        <v>0.19</v>
+        <v>0.33</v>
       </c>
       <c r="F323" t="s">
         <v>10</v>
@@ -9861,7 +9861,7 @@
         <v>9</v>
       </c>
       <c r="E324">
-        <v>0.14</v>
+        <v>0.15</v>
       </c>
       <c r="F324" t="s">
         <v>10</v>
@@ -9881,7 +9881,7 @@
         <v>9</v>
       </c>
       <c r="E325">
-        <v>0.31</v>
+        <v>0.24</v>
       </c>
       <c r="F325" t="s">
         <v>10</v>
@@ -9901,7 +9901,7 @@
         <v>9</v>
       </c>
       <c r="E326">
-        <v>0.22</v>
+        <v>0.3</v>
       </c>
       <c r="F326" t="s">
         <v>10</v>
@@ -9921,7 +9921,7 @@
         <v>9</v>
       </c>
       <c r="E327">
-        <v>0.34</v>
+        <v>0.19</v>
       </c>
       <c r="F327" t="s">
         <v>10</v>
@@ -9941,7 +9941,7 @@
         <v>9</v>
       </c>
       <c r="E328">
-        <v>0.27</v>
+        <v>0.12</v>
       </c>
       <c r="F328" t="s">
         <v>35</v>
@@ -9961,7 +9961,7 @@
         <v>9</v>
       </c>
       <c r="E329">
-        <v>0.17</v>
+        <v>0.12</v>
       </c>
       <c r="F329" t="s">
         <v>35</v>
@@ -9981,7 +9981,7 @@
         <v>9</v>
       </c>
       <c r="E330">
-        <v>0.17</v>
+        <v>0.38</v>
       </c>
       <c r="F330" t="s">
         <v>35</v>
@@ -10001,7 +10001,7 @@
         <v>9</v>
       </c>
       <c r="E331">
-        <v>0.12</v>
+        <v>0.37</v>
       </c>
       <c r="F331" t="s">
         <v>35</v>
@@ -10021,7 +10021,7 @@
         <v>9</v>
       </c>
       <c r="E332">
-        <v>0.36</v>
+        <v>0.27</v>
       </c>
       <c r="F332" t="s">
         <v>35</v>
@@ -10041,7 +10041,7 @@
         <v>9</v>
       </c>
       <c r="E333">
-        <v>0.23</v>
+        <v>0.31</v>
       </c>
       <c r="F333" t="s">
         <v>35</v>
@@ -10061,7 +10061,7 @@
         <v>9</v>
       </c>
       <c r="E334">
-        <v>0.24</v>
+        <v>0.14</v>
       </c>
       <c r="F334" t="s">
         <v>60</v>
@@ -10081,7 +10081,7 @@
         <v>9</v>
       </c>
       <c r="E335">
-        <v>0.11</v>
+        <v>0.29</v>
       </c>
       <c r="F335" t="s">
         <v>60</v>
@@ -10101,7 +10101,7 @@
         <v>9</v>
       </c>
       <c r="E336">
-        <v>0.32</v>
+        <v>0.3</v>
       </c>
       <c r="F336" t="s">
         <v>60</v>
@@ -10141,7 +10141,7 @@
         <v>9</v>
       </c>
       <c r="E338">
-        <v>0.11</v>
+        <v>0.14</v>
       </c>
       <c r="F338" t="s">
         <v>60</v>
@@ -10161,7 +10161,7 @@
         <v>9</v>
       </c>
       <c r="E339">
-        <v>0.17</v>
+        <v>0.27</v>
       </c>
       <c r="F339" t="s">
         <v>60</v>
@@ -10181,7 +10181,7 @@
         <v>9</v>
       </c>
       <c r="E340">
-        <v>0.24</v>
+        <v>0.19</v>
       </c>
       <c r="F340" t="s">
         <v>60</v>
@@ -10201,7 +10201,7 @@
         <v>9</v>
       </c>
       <c r="E341">
-        <v>0.25</v>
+        <v>0.39</v>
       </c>
       <c r="F341" t="s">
         <v>60</v>
@@ -10221,7 +10221,7 @@
         <v>9</v>
       </c>
       <c r="E342">
-        <v>0.19</v>
+        <v>0.11</v>
       </c>
       <c r="F342" t="s">
         <v>10</v>
@@ -10241,7 +10241,7 @@
         <v>9</v>
       </c>
       <c r="E343">
-        <v>0.16</v>
+        <v>0.26</v>
       </c>
       <c r="F343" t="s">
         <v>10</v>
@@ -10261,7 +10261,7 @@
         <v>9</v>
       </c>
       <c r="E344">
-        <v>0.28</v>
+        <v>0.3</v>
       </c>
       <c r="F344" t="s">
         <v>10</v>
@@ -10281,7 +10281,7 @@
         <v>9</v>
       </c>
       <c r="E345">
-        <v>0.35</v>
+        <v>0.33</v>
       </c>
       <c r="F345" t="s">
         <v>10</v>
@@ -10301,7 +10301,7 @@
         <v>9</v>
       </c>
       <c r="E346">
-        <v>0.18</v>
+        <v>0.1</v>
       </c>
       <c r="F346" t="s">
         <v>10</v>
@@ -10321,7 +10321,7 @@
         <v>9</v>
       </c>
       <c r="E347">
-        <v>0.25</v>
+        <v>0.14</v>
       </c>
       <c r="F347" t="s">
         <v>10</v>
@@ -10341,7 +10341,7 @@
         <v>9</v>
       </c>
       <c r="E348">
-        <v>0.37</v>
+        <v>0.14</v>
       </c>
       <c r="F348" t="s">
         <v>35</v>
@@ -10361,7 +10361,7 @@
         <v>9</v>
       </c>
       <c r="E349">
-        <v>0.38</v>
+        <v>0.14</v>
       </c>
       <c r="F349" t="s">
         <v>35</v>
@@ -10381,7 +10381,7 @@
         <v>9</v>
       </c>
       <c r="E350">
-        <v>0.37</v>
+        <v>0.34</v>
       </c>
       <c r="F350" t="s">
         <v>35</v>
@@ -10401,7 +10401,7 @@
         <v>9</v>
       </c>
       <c r="E351">
-        <v>0.36</v>
+        <v>0.2</v>
       </c>
       <c r="F351" t="s">
         <v>35</v>
@@ -10421,7 +10421,7 @@
         <v>9</v>
       </c>
       <c r="E352">
-        <v>0.25</v>
+        <v>0.14</v>
       </c>
       <c r="F352" t="s">
         <v>35</v>
@@ -10441,7 +10441,7 @@
         <v>9</v>
       </c>
       <c r="E353">
-        <v>0.33</v>
+        <v>0.24</v>
       </c>
       <c r="F353" t="s">
         <v>35</v>
@@ -10461,7 +10461,7 @@
         <v>9</v>
       </c>
       <c r="E354">
-        <v>0.39</v>
+        <v>0.38</v>
       </c>
       <c r="F354" t="s">
         <v>60</v>
@@ -10481,7 +10481,7 @@
         <v>9</v>
       </c>
       <c r="E355">
-        <v>0.13</v>
+        <v>0.18</v>
       </c>
       <c r="F355" t="s">
         <v>60</v>
@@ -10501,7 +10501,7 @@
         <v>9</v>
       </c>
       <c r="E356">
-        <v>0.33</v>
+        <v>0.25</v>
       </c>
       <c r="F356" t="s">
         <v>60</v>
@@ -10521,7 +10521,7 @@
         <v>9</v>
       </c>
       <c r="E357">
-        <v>0.39</v>
+        <v>0.33</v>
       </c>
       <c r="F357" t="s">
         <v>60</v>
@@ -10541,7 +10541,7 @@
         <v>9</v>
       </c>
       <c r="E358">
-        <v>0.33</v>
+        <v>0.24</v>
       </c>
       <c r="F358" t="s">
         <v>60</v>
@@ -10561,7 +10561,7 @@
         <v>9</v>
       </c>
       <c r="E359">
-        <v>0.12</v>
+        <v>0.28</v>
       </c>
       <c r="F359" t="s">
         <v>60</v>
@@ -10581,7 +10581,7 @@
         <v>9</v>
       </c>
       <c r="E360">
-        <v>0.29</v>
+        <v>0.24</v>
       </c>
       <c r="F360" t="s">
         <v>60</v>
@@ -10601,7 +10601,7 @@
         <v>9</v>
       </c>
       <c r="E361">
-        <v>0.2</v>
+        <v>0.14</v>
       </c>
       <c r="F361" t="s">
         <v>60</v>
@@ -10621,7 +10621,7 @@
         <v>9</v>
       </c>
       <c r="E362">
-        <v>0.17</v>
+        <v>0.28</v>
       </c>
       <c r="F362" t="s">
         <v>10</v>
@@ -10641,7 +10641,7 @@
         <v>9</v>
       </c>
       <c r="E363">
-        <v>0.38</v>
+        <v>0.17</v>
       </c>
       <c r="F363" t="s">
         <v>10</v>
@@ -10661,7 +10661,7 @@
         <v>9</v>
       </c>
       <c r="E364">
-        <v>0.31</v>
+        <v>0.26</v>
       </c>
       <c r="F364" t="s">
         <v>10</v>
@@ -10681,7 +10681,7 @@
         <v>9</v>
       </c>
       <c r="E365">
-        <v>0.17</v>
+        <v>0.2</v>
       </c>
       <c r="F365" t="s">
         <v>10</v>
@@ -10701,7 +10701,7 @@
         <v>9</v>
       </c>
       <c r="E366">
-        <v>0.35</v>
+        <v>0.32</v>
       </c>
       <c r="F366" t="s">
         <v>10</v>
@@ -10721,7 +10721,7 @@
         <v>9</v>
       </c>
       <c r="E367">
-        <v>0.23</v>
+        <v>0.26</v>
       </c>
       <c r="F367" t="s">
         <v>10</v>
@@ -10741,7 +10741,7 @@
         <v>9</v>
       </c>
       <c r="E368">
-        <v>0.27</v>
+        <v>0.26</v>
       </c>
       <c r="F368" t="s">
         <v>35</v>
@@ -10761,7 +10761,7 @@
         <v>9</v>
       </c>
       <c r="E369">
-        <v>0.33</v>
+        <v>0.27</v>
       </c>
       <c r="F369" t="s">
         <v>35</v>
@@ -10781,7 +10781,7 @@
         <v>9</v>
       </c>
       <c r="E370">
-        <v>0.23</v>
+        <v>0.33</v>
       </c>
       <c r="F370" t="s">
         <v>35</v>
@@ -10801,7 +10801,7 @@
         <v>9</v>
       </c>
       <c r="E371">
-        <v>0.15</v>
+        <v>0.38</v>
       </c>
       <c r="F371" t="s">
         <v>35</v>
@@ -10841,7 +10841,7 @@
         <v>9</v>
       </c>
       <c r="E373">
-        <v>0.1</v>
+        <v>0.19</v>
       </c>
       <c r="F373" t="s">
         <v>35</v>
@@ -10861,7 +10861,7 @@
         <v>9</v>
       </c>
       <c r="E374">
-        <v>0.23</v>
+        <v>0.36</v>
       </c>
       <c r="F374" t="s">
         <v>60</v>
@@ -10881,7 +10881,7 @@
         <v>9</v>
       </c>
       <c r="E375">
-        <v>0.28</v>
+        <v>0.39</v>
       </c>
       <c r="F375" t="s">
         <v>60</v>
@@ -10901,7 +10901,7 @@
         <v>9</v>
       </c>
       <c r="E376">
-        <v>0.38</v>
+        <v>0.21</v>
       </c>
       <c r="F376" t="s">
         <v>60</v>
@@ -10921,7 +10921,7 @@
         <v>9</v>
       </c>
       <c r="E377">
-        <v>0.31</v>
+        <v>0.14</v>
       </c>
       <c r="F377" t="s">
         <v>60</v>
@@ -10961,7 +10961,7 @@
         <v>9</v>
       </c>
       <c r="E379">
-        <v>0.13</v>
+        <v>0.21</v>
       </c>
       <c r="F379" t="s">
         <v>60</v>
@@ -10981,7 +10981,7 @@
         <v>9</v>
       </c>
       <c r="E380">
-        <v>0.33</v>
+        <v>0.35</v>
       </c>
       <c r="F380" t="s">
         <v>60</v>
@@ -11001,7 +11001,7 @@
         <v>9</v>
       </c>
       <c r="E381">
-        <v>0.32</v>
+        <v>0.35</v>
       </c>
       <c r="F381" t="s">
         <v>60</v>
@@ -11021,7 +11021,7 @@
         <v>9</v>
       </c>
       <c r="E382">
-        <v>0.11</v>
+        <v>0.19</v>
       </c>
       <c r="F382" t="s">
         <v>10</v>
@@ -11041,7 +11041,7 @@
         <v>9</v>
       </c>
       <c r="E383">
-        <v>0.18</v>
+        <v>0.4</v>
       </c>
       <c r="F383" t="s">
         <v>10</v>
@@ -11061,7 +11061,7 @@
         <v>9</v>
       </c>
       <c r="E384">
-        <v>0.3</v>
+        <v>0.24</v>
       </c>
       <c r="F384" t="s">
         <v>10</v>
@@ -11081,7 +11081,7 @@
         <v>9</v>
       </c>
       <c r="E385">
-        <v>0.25</v>
+        <v>0.19</v>
       </c>
       <c r="F385" t="s">
         <v>10</v>
@@ -11101,7 +11101,7 @@
         <v>9</v>
       </c>
       <c r="E386">
-        <v>0.35</v>
+        <v>0.3</v>
       </c>
       <c r="F386" t="s">
         <v>10</v>
@@ -11121,7 +11121,7 @@
         <v>9</v>
       </c>
       <c r="E387">
-        <v>0.32</v>
+        <v>0.4</v>
       </c>
       <c r="F387" t="s">
         <v>10</v>
@@ -11141,7 +11141,7 @@
         <v>9</v>
       </c>
       <c r="E388">
-        <v>0.21</v>
+        <v>0.13</v>
       </c>
       <c r="F388" t="s">
         <v>35</v>
@@ -11161,7 +11161,7 @@
         <v>9</v>
       </c>
       <c r="E389">
-        <v>0.16</v>
+        <v>0.21</v>
       </c>
       <c r="F389" t="s">
         <v>35</v>
@@ -11181,7 +11181,7 @@
         <v>9</v>
       </c>
       <c r="E390">
-        <v>0.12</v>
+        <v>0.25</v>
       </c>
       <c r="F390" t="s">
         <v>35</v>
@@ -11201,7 +11201,7 @@
         <v>9</v>
       </c>
       <c r="E391">
-        <v>0.18</v>
+        <v>0.11</v>
       </c>
       <c r="F391" t="s">
         <v>35</v>
@@ -11221,7 +11221,7 @@
         <v>9</v>
       </c>
       <c r="E392">
-        <v>0.22</v>
+        <v>0.26</v>
       </c>
       <c r="F392" t="s">
         <v>35</v>
@@ -11241,7 +11241,7 @@
         <v>9</v>
       </c>
       <c r="E393">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="F393" t="s">
         <v>35</v>
@@ -11261,7 +11261,7 @@
         <v>9</v>
       </c>
       <c r="E394">
-        <v>0.31</v>
+        <v>0.16</v>
       </c>
       <c r="F394" t="s">
         <v>60</v>
@@ -11281,7 +11281,7 @@
         <v>9</v>
       </c>
       <c r="E395">
-        <v>0.2</v>
+        <v>0.33</v>
       </c>
       <c r="F395" t="s">
         <v>60</v>
@@ -11301,7 +11301,7 @@
         <v>9</v>
       </c>
       <c r="E396">
-        <v>0.15</v>
+        <v>0.38</v>
       </c>
       <c r="F396" t="s">
         <v>60</v>
@@ -11321,7 +11321,7 @@
         <v>9</v>
       </c>
       <c r="E397">
-        <v>0.19</v>
+        <v>0.35</v>
       </c>
       <c r="F397" t="s">
         <v>60</v>
@@ -11341,7 +11341,7 @@
         <v>9</v>
       </c>
       <c r="E398">
-        <v>0.23</v>
+        <v>0.36</v>
       </c>
       <c r="F398" t="s">
         <v>60</v>
@@ -11361,7 +11361,7 @@
         <v>9</v>
       </c>
       <c r="E399">
-        <v>0.39</v>
+        <v>0.17</v>
       </c>
       <c r="F399" t="s">
         <v>60</v>
@@ -11381,7 +11381,7 @@
         <v>9</v>
       </c>
       <c r="E400">
-        <v>0.35</v>
+        <v>0.29</v>
       </c>
       <c r="F400" t="s">
         <v>60</v>
@@ -11401,7 +11401,7 @@
         <v>9</v>
       </c>
       <c r="E401">
-        <v>0.21</v>
+        <v>0.29</v>
       </c>
       <c r="F401" t="s">
         <v>60</v>
@@ -11421,7 +11421,7 @@
         <v>9</v>
       </c>
       <c r="E402">
-        <v>0.34</v>
+        <v>0.37</v>
       </c>
       <c r="F402" t="s">
         <v>10</v>
@@ -11441,7 +11441,7 @@
         <v>9</v>
       </c>
       <c r="E403">
-        <v>0.23</v>
+        <v>0.37</v>
       </c>
       <c r="F403" t="s">
         <v>10</v>
@@ -11461,7 +11461,7 @@
         <v>9</v>
       </c>
       <c r="E404">
-        <v>0.11</v>
+        <v>0.37</v>
       </c>
       <c r="F404" t="s">
         <v>10</v>
@@ -11481,7 +11481,7 @@
         <v>9</v>
       </c>
       <c r="E405">
-        <v>0.39</v>
+        <v>0.26</v>
       </c>
       <c r="F405" t="s">
         <v>10</v>
@@ -11501,7 +11501,7 @@
         <v>9</v>
       </c>
       <c r="E406">
-        <v>0.36</v>
+        <v>0.3</v>
       </c>
       <c r="F406" t="s">
         <v>10</v>
@@ -11521,7 +11521,7 @@
         <v>9</v>
       </c>
       <c r="E407">
-        <v>0.23</v>
+        <v>0.3</v>
       </c>
       <c r="F407" t="s">
         <v>10</v>
@@ -11541,7 +11541,7 @@
         <v>9</v>
       </c>
       <c r="E408">
-        <v>0.26</v>
+        <v>0.35</v>
       </c>
       <c r="F408" t="s">
         <v>35</v>
@@ -11561,7 +11561,7 @@
         <v>9</v>
       </c>
       <c r="E409">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="F409" t="s">
         <v>35</v>
@@ -11581,7 +11581,7 @@
         <v>9</v>
       </c>
       <c r="E410">
-        <v>0.32</v>
+        <v>0.14</v>
       </c>
       <c r="F410" t="s">
         <v>35</v>
@@ -11601,7 +11601,7 @@
         <v>9</v>
       </c>
       <c r="E411">
-        <v>0.22</v>
+        <v>0.24</v>
       </c>
       <c r="F411" t="s">
         <v>35</v>
@@ -11621,7 +11621,7 @@
         <v>9</v>
       </c>
       <c r="E412">
-        <v>0.27</v>
+        <v>0.14</v>
       </c>
       <c r="F412" t="s">
         <v>35</v>
@@ -11641,7 +11641,7 @@
         <v>9</v>
       </c>
       <c r="E413">
-        <v>0.21</v>
+        <v>0.29</v>
       </c>
       <c r="F413" t="s">
         <v>35</v>
@@ -11661,7 +11661,7 @@
         <v>9</v>
       </c>
       <c r="E414">
-        <v>0.28</v>
+        <v>0.32</v>
       </c>
       <c r="F414" t="s">
         <v>60</v>
@@ -11681,7 +11681,7 @@
         <v>9</v>
       </c>
       <c r="E415">
-        <v>0.11</v>
+        <v>0.37</v>
       </c>
       <c r="F415" t="s">
         <v>60</v>
@@ -11701,7 +11701,7 @@
         <v>9</v>
       </c>
       <c r="E416">
-        <v>0.13</v>
+        <v>0.22</v>
       </c>
       <c r="F416" t="s">
         <v>60</v>
@@ -11721,7 +11721,7 @@
         <v>9</v>
       </c>
       <c r="E417">
-        <v>0.21</v>
+        <v>0.33</v>
       </c>
       <c r="F417" t="s">
         <v>60</v>
@@ -11741,7 +11741,7 @@
         <v>9</v>
       </c>
       <c r="E418">
-        <v>0.36</v>
+        <v>0.13</v>
       </c>
       <c r="F418" t="s">
         <v>60</v>
@@ -11761,7 +11761,7 @@
         <v>9</v>
       </c>
       <c r="E419">
-        <v>0.2</v>
+        <v>0.33</v>
       </c>
       <c r="F419" t="s">
         <v>60</v>
@@ -11781,7 +11781,7 @@
         <v>9</v>
       </c>
       <c r="E420">
-        <v>0.38</v>
+        <v>0.13</v>
       </c>
       <c r="F420" t="s">
         <v>60</v>
@@ -11801,7 +11801,7 @@
         <v>9</v>
       </c>
       <c r="E421">
-        <v>0.13</v>
+        <v>0.17</v>
       </c>
       <c r="F421" t="s">
         <v>60</v>
@@ -11821,7 +11821,7 @@
         <v>9</v>
       </c>
       <c r="E422">
-        <v>0.21</v>
+        <v>0.27</v>
       </c>
       <c r="F422" t="s">
         <v>10</v>
@@ -11841,7 +11841,7 @@
         <v>9</v>
       </c>
       <c r="E423">
-        <v>0.13</v>
+        <v>0.32</v>
       </c>
       <c r="F423" t="s">
         <v>10</v>
@@ -11861,7 +11861,7 @@
         <v>9</v>
       </c>
       <c r="E424">
-        <v>0.39</v>
+        <v>0.31</v>
       </c>
       <c r="F424" t="s">
         <v>10</v>
@@ -11881,7 +11881,7 @@
         <v>9</v>
       </c>
       <c r="E425">
-        <v>0.39</v>
+        <v>0.24</v>
       </c>
       <c r="F425" t="s">
         <v>10</v>
@@ -11901,7 +11901,7 @@
         <v>9</v>
       </c>
       <c r="E426">
-        <v>0.22</v>
+        <v>0.17</v>
       </c>
       <c r="F426" t="s">
         <v>10</v>
@@ -11921,7 +11921,7 @@
         <v>9</v>
       </c>
       <c r="E427">
-        <v>0.28</v>
+        <v>0.14</v>
       </c>
       <c r="F427" t="s">
         <v>10</v>
@@ -11941,7 +11941,7 @@
         <v>9</v>
       </c>
       <c r="E428">
-        <v>0.35</v>
+        <v>0.23</v>
       </c>
       <c r="F428" t="s">
         <v>10</v>
@@ -11961,7 +11961,7 @@
         <v>9</v>
       </c>
       <c r="E429">
-        <v>0.2</v>
+        <v>0.26</v>
       </c>
       <c r="F429" t="s">
         <v>10</v>
@@ -11981,7 +11981,7 @@
         <v>9</v>
       </c>
       <c r="E430">
-        <v>0.13</v>
+        <v>0.32</v>
       </c>
       <c r="F430" t="s">
         <v>10</v>
@@ -12001,7 +12001,7 @@
         <v>9</v>
       </c>
       <c r="E431">
-        <v>0.13</v>
+        <v>0.38</v>
       </c>
       <c r="F431" t="s">
         <v>10</v>
@@ -12021,7 +12021,7 @@
         <v>9</v>
       </c>
       <c r="E432">
-        <v>0.25</v>
+        <v>0.31</v>
       </c>
       <c r="F432" t="s">
         <v>10</v>
@@ -12041,7 +12041,7 @@
         <v>9</v>
       </c>
       <c r="E433">
-        <v>0.35</v>
+        <v>0.23</v>
       </c>
       <c r="F433" t="s">
         <v>10</v>
@@ -12061,7 +12061,7 @@
         <v>9</v>
       </c>
       <c r="E434">
-        <v>0.13</v>
+        <v>0.27</v>
       </c>
       <c r="F434" t="s">
         <v>10</v>
@@ -12081,7 +12081,7 @@
         <v>9</v>
       </c>
       <c r="E435">
-        <v>0.18</v>
+        <v>0.29</v>
       </c>
       <c r="F435" t="s">
         <v>10</v>
@@ -12101,7 +12101,7 @@
         <v>9</v>
       </c>
       <c r="E436">
-        <v>0.31</v>
+        <v>0.26</v>
       </c>
       <c r="F436" t="s">
         <v>10</v>
@@ -12121,7 +12121,7 @@
         <v>9</v>
       </c>
       <c r="E437">
-        <v>0.4</v>
+        <v>0.21</v>
       </c>
       <c r="F437" t="s">
         <v>35</v>
@@ -12141,7 +12141,7 @@
         <v>9</v>
       </c>
       <c r="E438">
-        <v>0.17</v>
+        <v>0.34</v>
       </c>
       <c r="F438" t="s">
         <v>35</v>
@@ -12161,7 +12161,7 @@
         <v>9</v>
       </c>
       <c r="E439">
-        <v>0.34</v>
+        <v>0.22</v>
       </c>
       <c r="F439" t="s">
         <v>35</v>
@@ -12181,7 +12181,7 @@
         <v>9</v>
       </c>
       <c r="E440">
-        <v>0.22</v>
+        <v>0.34</v>
       </c>
       <c r="F440" t="s">
         <v>35</v>
@@ -12201,7 +12201,7 @@
         <v>9</v>
       </c>
       <c r="E441">
-        <v>0.38</v>
+        <v>0.33</v>
       </c>
       <c r="F441" t="s">
         <v>35</v>
@@ -12221,7 +12221,7 @@
         <v>9</v>
       </c>
       <c r="E442">
-        <v>0.22</v>
+        <v>0.14</v>
       </c>
       <c r="F442" t="s">
         <v>35</v>
@@ -12241,7 +12241,7 @@
         <v>9</v>
       </c>
       <c r="E443">
-        <v>0.13</v>
+        <v>0.21</v>
       </c>
       <c r="F443" t="s">
         <v>35</v>
@@ -12261,7 +12261,7 @@
         <v>9</v>
       </c>
       <c r="E444">
-        <v>0.32</v>
+        <v>0.14</v>
       </c>
       <c r="F444" t="s">
         <v>35</v>
@@ -12281,7 +12281,7 @@
         <v>9</v>
       </c>
       <c r="E445">
-        <v>0.12</v>
+        <v>0.25</v>
       </c>
       <c r="F445" t="s">
         <v>35</v>
@@ -12301,7 +12301,7 @@
         <v>9</v>
       </c>
       <c r="E446">
-        <v>0.15</v>
+        <v>0.29</v>
       </c>
       <c r="F446" t="s">
         <v>35</v>
@@ -12321,7 +12321,7 @@
         <v>9</v>
       </c>
       <c r="E447">
-        <v>0.2</v>
+        <v>0.38</v>
       </c>
       <c r="F447" t="s">
         <v>35</v>
@@ -12341,7 +12341,7 @@
         <v>9</v>
       </c>
       <c r="E448">
-        <v>0.22</v>
+        <v>0.28</v>
       </c>
       <c r="F448" t="s">
         <v>35</v>
@@ -12361,7 +12361,7 @@
         <v>9</v>
       </c>
       <c r="E449">
-        <v>0.37</v>
+        <v>0.26</v>
       </c>
       <c r="F449" t="s">
         <v>35</v>
@@ -12381,7 +12381,7 @@
         <v>9</v>
       </c>
       <c r="E450">
-        <v>0.27</v>
+        <v>0.3</v>
       </c>
       <c r="F450" t="s">
         <v>35</v>
@@ -12401,7 +12401,7 @@
         <v>9</v>
       </c>
       <c r="E451">
-        <v>0.3</v>
+        <v>0.13</v>
       </c>
       <c r="F451" t="s">
         <v>35</v>
@@ -12441,7 +12441,7 @@
         <v>9</v>
       </c>
       <c r="E453">
-        <v>0.13</v>
+        <v>0.24</v>
       </c>
       <c r="F453" t="s">
         <v>60</v>
@@ -12461,7 +12461,7 @@
         <v>9</v>
       </c>
       <c r="E454">
-        <v>0.18</v>
+        <v>0.27</v>
       </c>
       <c r="F454" t="s">
         <v>60</v>
@@ -12481,7 +12481,7 @@
         <v>9</v>
       </c>
       <c r="E455">
-        <v>0.3</v>
+        <v>0.18</v>
       </c>
       <c r="F455" t="s">
         <v>60</v>
@@ -12501,7 +12501,7 @@
         <v>9</v>
       </c>
       <c r="E456">
-        <v>0.16</v>
+        <v>0.31</v>
       </c>
       <c r="F456" t="s">
         <v>60</v>
@@ -12521,7 +12521,7 @@
         <v>9</v>
       </c>
       <c r="E457">
-        <v>0.31</v>
+        <v>0.18</v>
       </c>
       <c r="F457" t="s">
         <v>60</v>
@@ -12541,7 +12541,7 @@
         <v>9</v>
       </c>
       <c r="E458">
-        <v>0.28</v>
+        <v>0.15</v>
       </c>
       <c r="F458" t="s">
         <v>60</v>
@@ -12561,7 +12561,7 @@
         <v>9</v>
       </c>
       <c r="E459">
-        <v>0.19</v>
+        <v>0.16</v>
       </c>
       <c r="F459" t="s">
         <v>60</v>
@@ -12581,7 +12581,7 @@
         <v>9</v>
       </c>
       <c r="E460">
-        <v>0.39</v>
+        <v>0.3</v>
       </c>
       <c r="F460" t="s">
         <v>60</v>
@@ -12601,7 +12601,7 @@
         <v>9</v>
       </c>
       <c r="E461">
-        <v>0.29</v>
+        <v>0.11</v>
       </c>
       <c r="F461" t="s">
         <v>60</v>
@@ -12621,7 +12621,7 @@
         <v>9</v>
       </c>
       <c r="E462">
-        <v>0.39</v>
+        <v>0.4</v>
       </c>
       <c r="F462" t="s">
         <v>60</v>
@@ -12641,7 +12641,7 @@
         <v>9</v>
       </c>
       <c r="E463">
-        <v>0.14</v>
+        <v>0.3</v>
       </c>
       <c r="F463" t="s">
         <v>60</v>
@@ -12661,7 +12661,7 @@
         <v>9</v>
       </c>
       <c r="E464">
-        <v>0.18</v>
+        <v>0.31</v>
       </c>
       <c r="F464" t="s">
         <v>60</v>
@@ -12681,7 +12681,7 @@
         <v>9</v>
       </c>
       <c r="E465">
-        <v>0.39</v>
+        <v>0.34</v>
       </c>
       <c r="F465" t="s">
         <v>60</v>
@@ -12701,7 +12701,7 @@
         <v>9</v>
       </c>
       <c r="E466">
-        <v>0.1</v>
+        <v>0.27</v>
       </c>
       <c r="F466" t="s">
         <v>60</v>
@@ -12721,7 +12721,7 @@
         <v>9</v>
       </c>
       <c r="E467">
-        <v>0.26</v>
+        <v>0.24</v>
       </c>
       <c r="F467" t="s">
         <v>60</v>
@@ -12741,7 +12741,7 @@
         <v>9</v>
       </c>
       <c r="E468">
-        <v>0.33</v>
+        <v>0.39</v>
       </c>
       <c r="F468" t="s">
         <v>60</v>
@@ -12761,7 +12761,7 @@
         <v>9</v>
       </c>
       <c r="E469">
-        <v>0.27</v>
+        <v>0.13</v>
       </c>
       <c r="F469" t="s">
         <v>60</v>
@@ -12781,7 +12781,7 @@
         <v>9</v>
       </c>
       <c r="E470">
-        <v>0.37</v>
+        <v>0.1</v>
       </c>
       <c r="F470" t="s">
         <v>60</v>
@@ -12801,7 +12801,7 @@
         <v>9</v>
       </c>
       <c r="E471">
-        <v>0.21</v>
+        <v>0.16</v>
       </c>
       <c r="F471" t="s">
         <v>60</v>

</xml_diff>